<commit_message>
fix(procurement): replace Converge references with Comclark/TelTech across all bidder clarifications and bulletin
</commit_message>
<xml_diff>
--- a/RFP_Tender_Package/09_RFP_5G_FWA_Official_Clarifications_Responses_Master.xlsx
+++ b/RFP_Tender_Package/09_RFP_5G_FWA_Official_Clarifications_Responses_Master.xlsx
@@ -501,7 +501,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CONVERGE ICT SOLUTIONS / TELTECH 5G FWA NATIONWIDE TURNKEY TENDER</t>
+          <t>COMCLARK NETWORK &amp; TECHNOLOGY CORP. / TELTECH 5G FWA NATIONWIDE TURNKEY TENDER</t>
         </is>
       </c>
     </row>
@@ -512,6 +512,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -540,7 +541,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Converge Official Response</t>
+          <t>Comclark / TelTech Official Response</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -650,7 +651,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>To support the above planning activities, vendor kindly requests Converge to share the following information for the nearest tower(s): location (longitude / latitude) and tower height.</t>
+          <t>To support the above planning activities, vendor kindly requests Comclark/TelTech to share the following information for the nearest tower(s): location (longitude / latitude) and tower height.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -685,14 +686,14 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Vendor proposes that Converge may clarify the defination of "fiber segments" and the "optical nodes"</t>
+          <t>Vendor proposes that Comclark/TelTech clarify the defination of "fiber segments" and the "optical nodes"</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
           <t>CLARIFICATION OF DEFINITIONS:
-- 'Optical Node': An audited, active Converge point-of-interconnect—specifically an Optical Distribution Frame (ODF), Fiber Distribution Terminal (FDT), or Primary Fiber Hub equipped with available optical splice/splitter capacity to serve as the backhaul transmission handover point.
-- 'Fiber Segment': An audited physical fiber optic cable route (feeder, distribution, or lateral FOC) spanning between the optical node/central office and the customer/tower drop point, as verified in Converge's audited GIS distribution plant.</t>
+- 'Optical Node': An audited, active Comclark/TelTech point-of-interconnect—specifically an Optical Distribution Frame (ODF), Fiber Distribution Terminal (FDT), or Primary Fiber Hub equipped with available optical splice/splitter capacity to serve as the backhaul transmission handover point.
+- 'Fiber Segment': An audited physical fiber optic cable route (feeder, distribution, or lateral FOC) spanning between the optical node/central office and the customer/tower drop point, as verified in Comclark/TelTech's audited GIS distribution plant.</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
@@ -722,13 +723,13 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Vendor proposes that Converge may clarify the defination of " C: Line-tap splice closure &lt;= 0.5 km"</t>
+          <t>Vendor proposes that Comclark/TelTech clarify the defination of " C: Line-tap splice closure &lt;= 0.5 km"</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
           <t>CLARIFICATION OF DEFINITION:
-'Class C: Line-tap splice closure &lt;= 0.5 km' designates a candidate macro tower location where an existing aerial or underground Converge trunk/distribution fiber optic cable passes within 500 meters of the site compound, and interconnection will be achieved by cutting into the cable at an existing or newly inserted inline splice closure (FOSC / Dome Enclosure) rather than routing back to a centralized ODF/node.</t>
+'Class C: Line-tap splice closure &lt;= 0.5 km' designates a candidate macro tower location where an existing aerial or underground Comclark/TelTech trunk/distribution fiber optic cable passes within 500 meters of the site compound, and interconnection will be achieved by cutting into the cable at an existing or newly inserted inline splice closure (FOSC / Dome Enclosure) rather than routing back to a centralized ODF/node.</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -759,13 +760,13 @@
       <c r="E10" s="8" t="inlineStr">
         <is>
           <t>Does the "distance to the nearest node" refer to the distance to the 5G base station ?
- Vendor proposes that Converge may clarify the defination of " distance to line-tap closure"</t>
+ Vendor proposes that Comclark/TelTech clarify the defination of " distance to line-tap closure"</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
           <t>CLARIFICATION OF DEFINITIONS:
-- 'Distance to Nearest Node': Refers to the estimated terrestrial linear cable route distance from the proposed 5G Macro Tower compound to the nearest confirmed Converge Optical Node (Class A &lt;= 0.5 km; Class B &lt;= 1.0 km).
+- 'Distance to Nearest Node': Refers to the estimated terrestrial linear cable route distance from the proposed 5G Macro Tower compound to the nearest confirmed Comclark/TelTech Optical Node (Class A &lt;= 0.5 km; Class B &lt;= 1.0 km).
 - 'Distance to Line-Tap Closure': Refers to the linear cable distance from the 5G Base Station to the designated trunk cable splice closure (Class C &lt;= 0.5 km).</t>
         </is>
       </c>
@@ -796,13 +797,13 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Vendor respectfully proposes that Converge confirm whether the Microwave solution for Class D is to be considered within the Vendor's scope of supply, or whether it will be provided by Converge directly.</t>
+          <t>Vendor respectfully proposes that Comclark/TelTech confirm whether the Microwave solution for Class D is to be considered within the Vendor's scope of supply, or whether it will be provided by Comclark/TelTech directly.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
           <t>CONFIRMED: VENDOR SCOPE OF SUPPLY / PRICING.
-Class D sites (~1.7% of Phase 1 sites, plus microwave backup links for island sites) require a turnkey high-capacity microwave backhaul link (11 GHz / 18 GHz / 23 GHz or E-Band 80 GHz, minimum 1.0 Gbps full-duplex throughput). Bidders must quote the microwave split-mount hardware (IDU, ODU, antenna, IF cabling) and installation services in Appendix B (Commercial BoQ) under Lot 1 / Lot 3 options. Converge reserves the right to provide direct fiber drops prior to NTP where feasible.</t>
+Class D sites (~1.7% of Phase 1 sites, plus microwave backup links for island sites) require a turnkey high-capacity microwave backhaul link (11 GHz / 18 GHz / 23 GHz or E-Band 80 GHz, minimum 1.0 Gbps full-duplex throughput). Bidders must quote the microwave split-mount hardware (IDU, ODU, antenna, IF cabling) and installation services in Appendix B (Commercial BoQ) under Lot 1 / Lot 3 options. Comclark/TelTech reserves the right to provide direct fiber drops prior to NTP where feasible.</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -917,7 +918,7 @@
       <c r="F14" s="8" t="inlineStr">
         <is>
           <t>DIVISION OF RESPONSIBILITY:
-- Converge / TelTech Scope: Core IP/MPLS network, backbone transport, optical node infrastructure, upstream bandwidth, fiber drop cable provisioning up to the tower demarcation/ODF, and Starlink satellite terminals.
+- Comclark / TelTech Scope: Core IP/MPLS network, backbone transport, optical node infrastructure, upstream bandwidth, fiber drop cable provisioning up to the tower demarcation/ODF, and Starlink satellite terminals.
 - Vendor Scope: Turnkey supply of optical transceivers (10G/25G SFP28 eCPRI and 10G/25G SFP+ backhaul optics), armored optical patchcords, terminal fiber interconnect from tower demarcation box to Baseband Unit (BBU), and end-to-end backhaul circuit acceptance testing during SSV.</t>
         </is>
       </c>
@@ -1067,7 +1068,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CONVERGE ICT SOLUTIONS / TELTECH 5G FWA NATIONWIDE TURNKEY TENDER</t>
+          <t>COMCLARK NETWORK &amp; TECHNOLOGY CORP. / TELTECH 5G FWA NATIONWIDE TURNKEY TENDER</t>
         </is>
       </c>
     </row>
@@ -1078,6 +1079,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1106,7 +1108,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Converge Official Response</t>
+          <t>Comclark / TelTech Official Response</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -1177,7 +1179,7 @@
       <c r="F6" s="8" t="inlineStr">
         <is>
           <t>CLARIFICATION OF BILLING SCOPE:
-In Phase 1, real-time Convergent Charging (CCS/CHF via 3GPP Nchf/Diameter Ro) for prepaid FWA balance management, session cutoff, and quota tracking is the mandatory turnkey scope. Complex postpaid cyclic invoice generation and accounts receivable (A/R) are handled by Converge's enterprise billing system via standard CDR/API export, or may be proposed as an optional modular add-on.</t>
+In Phase 1, real-time Convergent Charging (CCS/CHF via 3GPP Nchf/Diameter Ro) for prepaid FWA balance management, session cutoff, and quota tracking is the mandatory turnkey scope. Complex postpaid cyclic invoice generation and accounts receivable (A/R) are handled by Comclark/TelTech's enterprise billing system via standard CDR/API export, or may be proposed as an optional modular add-on.</t>
         </is>
       </c>
       <c r="G6" s="9" t="inlineStr">
@@ -1376,7 +1378,7 @@
       <c r="F11" s="5" t="inlineStr">
         <is>
           <t>PAYMENT MODE ARCHITECTURE:
-The primary business model for Phase 1 is 100% Prepaid with 30-day recurring subscription validity. Postpaid hybrid invoicing is handled via integration with Converge's enterprise billing platform; vendors are only required to provide the real-time prepaid CHF/CCS engine and payment gateway connectors.</t>
+The primary business model for Phase 1 is 100% Prepaid with 30-day recurring subscription validity. Postpaid hybrid invoicing is handled via integration with Comclark/TelTech's enterprise billing platform; vendors are only required to provide the real-time prepaid CHF/CCS engine and payment gateway connectors.</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -1412,7 +1414,7 @@
       <c r="F12" s="8" t="inlineStr">
         <is>
           <t>ENTERPRISE INTEGRATIONS:
-The BSS must support standard daily accounting journal export (GL feed) to Converge's SAP ERP and daily CDR/event extraction to the enterprise Data Warehouse (DWH). Real-time Kafka-based event streaming is preferred for operational analytics.</t>
+The BSS must support standard daily accounting journal export (GL feed) to Comclark/TelTech's SAP ERP and daily CDR/event extraction to the enterprise Data Warehouse (DWH). Real-time Kafka-based event streaming is preferred for operational analytics.</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
@@ -1778,9 +1780,9 @@
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>1. For the TowerCo site, Is it Converge Scope to rent and negotiate with TowerCo?
-Suggest: For towerco site, should be converge's responsibility for site renting and negoitate with towerco.
-2. If the site hunting fail, whats the next step? (Converge to provide another site for hunting to swap the fail site? or cancel the site).
+          <t>1. For the TowerCo site, Is it Comclark/TelTech scope to rent and negotiate with TowerCo?
+Suggest: For towerco site, should be Comclark/TelTech's responsibility for site renting and negotiating with TowerCo.
+2. If the site hunting fail, whats the next step? (Comclark/TelTech to provide another site for hunting to swap the failed site? or cancel the site).
 Suggest: Vendor will hunt each site with 5 options, if site still failed, suggest customer change the site or provide VO for new option hunting.</t>
         </is>
       </c>
@@ -1854,13 +1856,13 @@
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Is it Converge scope for Fiber or the vendor is required to execute?</t>
+          <t>Is it Comclark/TelTech scope for Fiber or the vendor is required to execute?</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
           <t>FIBER BACKHAUL RESPONSIBILITY:
-Converge provides the core optical distribution network, terrestrial fiber drop cable up to the site boundary/ODF, and Starlink satellite terminals. The vendor is responsible for optical transceivers, patchcords, and joint I&amp;C testing from the demarcation box to the BBU.</t>
+Comclark/TelTech provides the core optical distribution network, terrestrial fiber drop cable up to the site boundary/ODF, and Starlink satellite terminals. The vendor is responsible for optical transceivers, patchcords, and joint I&amp;C testing from the demarcation box to the BBU.</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">
@@ -1999,7 +2001,7 @@
       <c r="E28" s="8" t="inlineStr">
         <is>
           <t>1. Please provide the verified per-site fiber node/segment list (optical node ID, connection class A-D, committed bandwidth) after on-ground verification — the site list shows all Starlink-fed sites have dist-to-node &gt; 20 km.
-2. Please confirm that backhaul resources (Converge fiber SLA, Starlink links) are Operator/third-party provided, and the Operator is responsible for their availability, bandwidth and latency.
+2. Please confirm that backhaul resources (Comclark/TelTech fiber SLA, Starlink links) are Operator/third-party provided, and the Operator is responsible for their availability, bandwidth and latency.
 3. Do you accept media-tiered RTT KPIs: fiber-fed sites bound by &lt;= 30ms, while satellite-fed sites follow their link physics (e.g. &lt;= 100ms)?
 4. Please confirm backhaul outage time is excluded from KPI assessment (RAN availability, end-to-end availability, packet loss).
 Expected: written confirmation + per-site backhaul list.</t>
@@ -2009,7 +2011,7 @@
         <is>
           <t>BACKHAUL RESOURCES &amp; SLA EXCLUSIONS:
 1. Candidate site list in Document 07 provides audited fiber distance classes (Class A &lt;= 0.5km to Class D).
-2. Confirmed: Backhaul transport facilities (Converge terrestrial FOC and Starlink links) are Operator-provided.
+2. Confirmed: Backhaul transport facilities (Comclark/TelTech terrestrial FOC and Starlink links) are Operator-provided.
 3. Media-tiered RTT KPIs are formally confirmed: Fiber sites &lt;= 30 ms maximum; Satellite sites &lt;= 80 ms maximum.
 4. Confirmed: Downtime caused by upstream third-party transmission outages or fiber cuts outside the site compound is excluded from vendor RAN availability penalty assessments.</t>
         </is>
@@ -2203,7 +2205,7 @@
       <c r="E33" s="5" t="inlineStr">
         <is>
           <t>1. According to ITU-R M.2159-0, the 1518–1525 MHz frequency band is used for maritime communications satellites. If the frequency range of the RRU includes 1512–1517 MHz, it cannot ensure a -30 dB suppression within the 1518–1523 MHz band. Therefore, please confirm whether the NTC allows the use of the 1512–1517 MHz spectrum.
-2. We understand that the 1427–1457 MHz frequency band will be allocated by the NTC as spectrum for enterprises. Please consider whether Converge intends to use the 1457–1467 MHz band. It is recommended to refer to the NTC's spectrum usage regulations to determine whether a guard band is required. Therefore, please confirm whether the NTC allows the use of the 1457–1467 MHz spectrum.</t>
+2. We understand that the 1427–1457 MHz frequency band will be allocated by the NTC as spectrum for enterprises. Please consider whether Comclark/TelTech intends to use the 1457–1467 MHz band. It is recommended to refer to the NTC's spectrum usage regulations to determine whether a guard band is required. Therefore, please confirm whether the NTC allows the use of the 1457–1467 MHz spectrum.</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
@@ -2529,7 +2531,7 @@
       <c r="F42" s="8" t="inlineStr">
         <is>
           <t>OSS INTEGRATION:
-Vendor must deliver EMS/NMS for domain element management, equipped with open northbound interfaces (REST APIs, SNMPv3, Kafka) for integration into Converge's enterprise monitoring umbrella (AUTIN).</t>
+Vendor must deliver EMS/NMS for domain element management, equipped with open northbound interfaces (REST APIs, SNMPv3, Kafka) for integration into Comclark/TelTech's enterprise monitoring umbrella (AUTIN).</t>
         </is>
       </c>
       <c r="G42" s="9" t="inlineStr">

</xml_diff>

<commit_message>
feat(portal): add return to portal button on bulletin, hide raw clarification matrix from public view, enforce Bidder/Supplier terminology
</commit_message>
<xml_diff>
--- a/RFP_Tender_Package/09_RFP_5G_FWA_Official_Clarifications_Responses_Master.xlsx
+++ b/RFP_Tender_Package/09_RFP_5G_FWA_Official_Clarifications_Responses_Master.xlsx
@@ -612,7 +612,7 @@
       <c r="E6" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Further clarification is required regarding the bandwidth that needs to be supported. Are there any special customization requirements for the filter's out-of-band rejection and emissions?
-Point 1: If the 1437–1457 MHz band is occupied by another operator, are there any specific spurious emission requirements that vendor's equipment must comply with for the low end and high end(1457M and 1517M)?
+Point 1: If the 1437–1457 MHz band is occupied by another operator, are there any specific spurious emission requirements that supplier's equipment must comply with for the low end and high end(1457M and 1517M)?
 Point 2: If the 1437–1457 MHz band is available for use outside the NCR areas, does the NTC impose any spurious emission requirements for the low and high end(1437M and 1517M)?
 </t>
         </is>
@@ -620,7 +620,7 @@
       <c r="F6" s="8" t="inlineStr">
         <is>
           <t>CONFIRMED &amp; DETAILED:
-Point 1 (NCR Carrier: 1457–1517 MHz): Vendor equipment must comply with 3GPP TS 38.104 Category B Operating Band Unwanted Emissions (OBUE) and standard NTC Type Approval spurious emission masks. At the low end (1457 MHz), the RRU digital filtering and DPD must ensure sharp attenuation to protect adjacent users below 1457 MHz. At the high end (1517 MHz), equipment must implement appropriate filtering to protect the adjacent Maritime Mobile Satellite Service (MSS, 1518–1525 MHz per ITU-R M.2159-0), with unwanted emissions not exceeding -30 dBm/MHz.
+Point 1 (NCR Carrier: 1457–1517 MHz): Supplier equipment must comply with 3GPP TS 38.104 Category B Operating Band Unwanted Emissions (OBUE) and standard NTC Type Approval spurious emission masks. At the low end (1457 MHz), the RRU digital filtering and DPD must ensure sharp attenuation to protect adjacent users below 1457 MHz. At the high end (1517 MHz), equipment must implement appropriate filtering to protect the adjacent Maritime Mobile Satellite Service (MSS, 1518–1525 MHz per ITU-R M.2159-0), with unwanted emissions not exceeding -30 dBm/MHz.
 Point 2 (Outside NCR: 1437–1517 MHz): Standard 3GPP Band n50 TS 38.104 Category B emission masks apply at the 1437 MHz lower edge and 1517 MHz upper edge. No non-standard or proprietary hardware filtering customization is required beyond compliant 3GPP Release 16/17 Band n50 radio hardware.</t>
         </is>
       </c>
@@ -651,7 +651,7 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t>To support the above planning activities, vendor kindly requests Comclark/TelTech to share the following information for the nearest tower(s): location (longitude / latitude) and tower height.</t>
+          <t>To support the above planning activities, bidder kindly requests Comclark/TelTech to share the following information for the nearest tower(s): location (longitude / latitude) and tower height.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
@@ -686,7 +686,7 @@
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>Vendor proposes that Comclark/TelTech clarify the defination of "fiber segments" and the "optical nodes"</t>
+          <t>Bidder proposes that Comclark/TelTech clarify the defination of "fiber segments" and the "optical nodes"</t>
         </is>
       </c>
       <c r="F8" s="8" t="inlineStr">
@@ -723,7 +723,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t>Vendor proposes that Comclark/TelTech clarify the defination of " C: Line-tap splice closure &lt;= 0.5 km"</t>
+          <t>Bidder proposes that Comclark/TelTech clarify the defination of " C: Line-tap splice closure &lt;= 0.5 km"</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
@@ -760,7 +760,7 @@
       <c r="E10" s="8" t="inlineStr">
         <is>
           <t>Does the "distance to the nearest node" refer to the distance to the 5G base station ?
- Vendor proposes that Comclark/TelTech clarify the defination of " distance to line-tap closure"</t>
+ Bidder proposes that Comclark/TelTech clarify the defination of " distance to line-tap closure"</t>
         </is>
       </c>
       <c r="F10" s="8" t="inlineStr">
@@ -797,12 +797,12 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>Vendor respectfully proposes that Comclark/TelTech confirm whether the Microwave solution for Class D is to be considered within the Vendor's scope of supply, or whether it will be provided by Comclark/TelTech directly.</t>
+          <t>Bidder respectfully proposes that Comclark/TelTech confirm whether the Microwave solution for Class D is to be considered within the Supplier's scope of supply, or whether it will be provided by Comclark/TelTech directly.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>CONFIRMED: VENDOR SCOPE OF SUPPLY / PRICING.
+          <t>CONFIRMED: SUPPLIER SCOPE OF SUPPLY / PRICING.
 Class D sites (~1.7% of Phase 1 sites, plus microwave backup links for island sites) require a turnkey high-capacity microwave backhaul link (11 GHz / 18 GHz / 23 GHz or E-Band 80 GHz, minimum 1.0 Gbps full-duplex throughput). Bidders must quote the microwave split-mount hardware (IDU, ODU, antenna, IF cabling) and installation services in Appendix B (Commercial BoQ) under Lot 1 / Lot 3 options. Comclark/TelTech reserves the right to provide direct fiber drops prior to NTP where feasible.</t>
         </is>
       </c>
@@ -835,7 +835,7 @@
         <is>
           <t>Kindly confirm whether the 12 kW rating refers to the total installed rectifier capacity (4 × 3 kW modules, including one N+1 redundant module) rather than the output that must be maintained after a single module failure.
 For reference, a typical load — 3 kW BTS with a 400 Ah battery charged at 0.2C — requires a total DC demand of 7.28 kW (4.28 kW charging + 3 kW BTS load). This demand is fully served by three 3 kW modules, with a fourth module providing N+1 redundancy (12 kW installed; 9 kW available under N+1).
-Vendor appreciates your confirmation that this load-based N+1 sizing methodology is acceptable, including functionally equivalent configurations.</t>
+Supplier appreciates your confirmation that this load-based N+1 sizing methodology is acceptable, including functionally equivalent configurations.</t>
         </is>
       </c>
       <c r="F12" s="8" t="inlineStr">
@@ -844,7 +844,7 @@
 The required sizing methodology is confirmed as follows:
 - Total Installed Rectifier Capacity: &gt;= 12.0 kW composed of 4 × 3.0 kW (or 4 × 4.0 kW) modular hot-swappable switchmode rectifier modules in an N+1 architecture.
 - Active Operational Capacity under N+1: With a single module failure (3 operational modules), the system provides 9.0 kW continuous DC output, which comfortably exceeds the peak site DC demand of 7.28 kW (3.0 kW BTS RAN load + 4.28 kW fast battery recharging at 0.2C for 400 Ah / 20 kWh lithium bank).
-Vendor's proposed load-based N+1 configuration is fully compliant.</t>
+Supplier's proposed load-based N+1 configuration is fully compliant.</t>
         </is>
       </c>
       <c r="G12" s="9" t="inlineStr">
@@ -919,7 +919,7 @@
         <is>
           <t>DIVISION OF RESPONSIBILITY:
 - Comclark / TelTech Scope: Core IP/MPLS network, backbone transport, optical node infrastructure, upstream bandwidth, fiber drop cable provisioning up to the tower demarcation/ODF, and Starlink satellite terminals.
-- Vendor Scope: Turnkey supply of optical transceivers (10G/25G SFP28 eCPRI and 10G/25G SFP+ backhaul optics), armored optical patchcords, terminal fiber interconnect from tower demarcation box to Baseband Unit (BBU), and end-to-end backhaul circuit acceptance testing during SSV.</t>
+- Supplier Scope: Turnkey supply of optical transceivers (10G/25G SFP28 eCPRI and 10G/25G SFP+ backhaul optics), armored optical patchcords, terminal fiber interconnect from tower demarcation box to Baseband Unit (BBU), and end-to-end backhaul circuit acceptance testing during SSV.</t>
         </is>
       </c>
       <c r="G14" s="9" t="inlineStr">
@@ -949,7 +949,7 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t>There are no engineering services items about Rectifier, Battery, Tap-Off Box &amp; Submeter, Getset, pls confirm engineering services isn't vendor's scope.</t>
+          <t>There are no engineering services items about Rectifier, Battery, Tap-Off Box &amp; Submeter, Getset, pls confirm engineering services isn't supplier's scope.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
@@ -1022,14 +1022,14 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t>There are no engineering services items about Commercial Power Access, pls confirm engineering services isn't vendor's scope.</t>
+          <t>There are no engineering services items about Commercial Power Access, pls confirm engineering services isn't supplier's scope.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
           <t>COORDINATED SCOPE:
 - TelTech / Operator Scope: Payment of official electric cooperative (EC / Meralco / DU) application fees, transformer capital contributions, security deposits, and power supply contracts.
-- Vendor Scope: Turnkey on-site civil and electrical works from the property line / service drop demarcation pole to the equipment pad—including service entrance conduit/riser, utility revenue class kWh meter base/enclosure, main service disconnect switch, AC panel (ACPDB), and surge protective device (Type 1+2 SPD).</t>
+- Supplier Scope: Turnkey on-site civil and electrical works from the property line / service drop demarcation pole to the equipment pad—including service entrance conduit/riser, utility revenue class kWh meter base/enclosure, main service disconnect switch, AC panel (ACPDB), and surge protective device (Type 1+2 SPD).</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
@@ -1372,13 +1372,13 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>What's the payment mode shall be supported by the BSS? Prepaid, Postpaid, Hybrid? If need postpaid, and hybrid, does it meant the vendor need to provide the billing, invoice relevant components?</t>
+          <t>What's the payment mode shall be supported by the BSS? Prepaid, Postpaid, Hybrid? If need postpaid, and hybrid, does it meant the supplier need to provide the billing, invoice relevant components?</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
           <t>PAYMENT MODE ARCHITECTURE:
-The primary business model for Phase 1 is 100% Prepaid with 30-day recurring subscription validity. Postpaid hybrid invoicing is handled via integration with Comclark/TelTech's enterprise billing platform; vendors are only required to provide the real-time prepaid CHF/CCS engine and payment gateway connectors.</t>
+The primary business model for Phase 1 is 100% Prepaid with 30-day recurring subscription validity. Postpaid hybrid invoicing is handled via integration with Comclark/TelTech's enterprise billing platform; bidders / suppliers are only required to provide the real-time prepaid CHF/CCS engine and payment gateway connectors.</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
@@ -1444,13 +1444,13 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t>Beside the self-care channels, shall the vendor provide the retail portal which can be used by the in-shop agent or call center agent?</t>
+          <t>Beside the self-care channels, shall the supplier provide the retail portal which can be used by the in-shop agent or call center agent?</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
           <t>RETAIL &amp; AGENT PORTAL SCOPE:
-CONFIRMED. Vendor must provide a secure, web-based Customer Service Representative (CSR) and Authorized Dealer Portal for retail store agents, partner distribution dealers, and call center hotlines to perform customer onboarding, balance lookups, and troubleshooting.</t>
+CONFIRMED. Supplier must provide a secure, web-based Customer Service Representative (CSR) and Authorized Dealer Portal for retail store agents, partner distribution dealers, and call center hotlines to perform customer onboarding, balance lookups, and troubleshooting.</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -1522,7 +1522,7 @@
       <c r="F15" s="5" t="inlineStr">
         <is>
           <t>POLICY CONTROL (PCF) INTEGRATION:
-Under Lot 3 (5G Core Network), the vendor is delivering the turnkey 5G SA Core, which includes the Policy Control Function (PCF). The BSS will integrate directly with the vendor's supplied PCF via standard 3GPP N7 / N28 interfaces.</t>
+Under Lot 3 (5G Core Network), the supplier is delivering the turnkey 5G SA Core, which includes the Policy Control Function (PCF). The BSS will integrate directly with the supplier's supplied PCF via standard 3GPP N7 / N28 interfaces.</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -1634,7 +1634,7 @@
       <c r="F18" s="8" t="inlineStr">
         <is>
           <t>STRUCTURAL LOADING RESPONSIBILITY:
-1. For the 897 TowerCo co-location sites, Tower Structural Loading Verification is the responsibility of the Operator and the TowerCo under the executed Master Lease Agreement (MLA). The vendor provides equipment weights, dimensions, wind load surface area, and cable routing details.
+1. For the 897 TowerCo co-location sites, Tower Structural Loading Verification is the responsibility of the Operator and the TowerCo under the executed Master Lease Agreement (MLA). The supplier provides equipment weights, dimensions, wind load surface area, and cable routing details.
 2. If loading verification fails, the TowerCo is obligated under the MLA to perform structural retrofitting, or the Operator will reassign an alternative candidate tower from the pre-approved pool.</t>
         </is>
       </c>
@@ -1662,13 +1662,13 @@
       <c r="E19" s="5" t="inlineStr">
         <is>
           <t>Whats the acceptance standard and procedure for Tower, Civil and Power part?
-Suggest: Vendor can propose if needed.</t>
+Suggest: Supplier can propose if needed.</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
           <t>ACCEPTANCE STANDARDS:
-Acceptance standards and checklists for Civil, Tower, and Power are detailed in Document 05 ('05_Appendix_D_Site_Survey_RF_Planning_Civil_Power_Guidelines.pdf') and Document 04 (Appendix C). Vendor's standard QA/QC procedure and handover templates are acceptable subject to Joint Technical Committee approval.</t>
+Acceptance standards and checklists for Civil, Tower, and Power are detailed in Document 05 ('05_Appendix_D_Site_Survey_RF_Planning_Civil_Power_Guidelines.pdf') and Document 04 (Appendix C). Supplier's standard QA/QC procedure and handover templates are acceptable subject to Joint Technical Committee approval.</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -1701,7 +1701,7 @@
       <c r="E20" s="8" t="inlineStr">
         <is>
           <t>For New Site, the BOQ not include the commerical power application and installation (From COOP to Site). Do we need to quote this part? 
-If the commerical power not ready, does the vendor need to provide the temporary power to turn on the site?
+If the commerical power not ready, does the supplier need to provide the temporary power to turn on the site?
 Suggest: Commerical power shall included and temporary power can consider as VO when needed.</t>
         </is>
       </c>
@@ -1709,7 +1709,7 @@
         <is>
           <t>COMMERCIAL POWER &amp; TEMPORARY POWER:
 1. Official electric cooperative (EC/DU) application fees and power connection contracts are Operator scope.
-2. Turnkey on-site civil and electrical installation (service entrance, meter base, disconnect, ACPDB) is Vendor scope.
+2. Turnkey on-site civil and electrical installation (service entrance, meter base, disconnect, ACPDB) is Supplier scope.
 3. If commercial utility power is delayed by the power utility, the site will be provisionally accepted using temporary generator power where expedited on-air is mutually agreed, with generator runtime costs handled via established Variation Order (VO).</t>
         </is>
       </c>
@@ -1742,8 +1742,8 @@
       <c r="E21" s="5" t="inlineStr">
         <is>
           <t>1. Do you have Type approved brand for Tower, Genset, Aviation light, ACPDB and other power or civil material?
-2. Can you provide Typical Design drawing for Tower, Fence and foundation? Or turnkey contractor to propose the solution.
-Suggest: Vendor can propose if needed.</t>
+2. Can you provide Typical Design drawing for Tower, Fence and foundation? Or bidder / supplier to propose the solution.
+Suggest: Supplier can propose if needed.</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
@@ -1783,14 +1783,14 @@
           <t>1. For the TowerCo site, Is it Comclark/TelTech scope to rent and negotiate with TowerCo?
 Suggest: For towerco site, should be Comclark/TelTech's responsibility for site renting and negotiating with TowerCo.
 2. If the site hunting fail, whats the next step? (Comclark/TelTech to provide another site for hunting to swap the failed site? or cancel the site).
-Suggest: Vendor will hunt each site with 5 options, if site still failed, suggest customer change the site or provide VO for new option hunting.</t>
+Suggest: Supplier will hunt each site with 5 options, if site still failed, suggest customer change the site or provide VO for new option hunting.</t>
         </is>
       </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
           <t>SITE ACQUISITION &amp; TOWERCO LEASE NEGOTIATION:
 1. For the 897 Co-location sites, lease agreements, space reservation, and commercial negotiations with TowerCos (PhilTower, EdgePoint, EDOTCO, Unity) are strictly the Operator's responsibility under Master Lease Agreements (MLA).
-2. For the 103 Greenfield sites, the vendor performs primary site hunting with up to 3 candidate parcels. If site hunting fails due to zoning, legal, or title defects, the Operator will provide a replacement candidate site without vendor penalty.</t>
+2. For the 103 Greenfield sites, the supplier performs primary site hunting with up to 3 candidate parcels. If site hunting fails due to zoning, legal, or title defects, the Operator will provide a replacement candidate site without bidder penalty.</t>
         </is>
       </c>
       <c r="G22" s="9" t="inlineStr">
@@ -1856,13 +1856,13 @@
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>Is it Comclark/TelTech scope for Fiber or the vendor is required to execute?</t>
+          <t>Is it Comclark/TelTech scope for Fiber or the supplier is required to execute?</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
           <t>FIBER BACKHAUL RESPONSIBILITY:
-Comclark/TelTech provides the core optical distribution network, terrestrial fiber drop cable up to the site boundary/ODF, and Starlink satellite terminals. The vendor is responsible for optical transceivers, patchcords, and joint I&amp;C testing from the demarcation box to the BBU.</t>
+Comclark/TelTech provides the core optical distribution network, terrestrial fiber drop cable up to the site boundary/ODF, and Starlink satellite terminals. The supplier is responsible for optical transceivers, patchcords, and joint I&amp;C testing from the demarcation box to the BBU.</t>
         </is>
       </c>
       <c r="G24" s="9" t="inlineStr">
@@ -1892,7 +1892,7 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">For the non-standard and special construction reuqirment, such as manul hauling, retaining wall and others, Can the turnkey contractor claim separately as VO? </t>
+          <t xml:space="preserve">For the non-standard and special construction reuqirment, such as manul hauling, retaining wall and others, Can the bidder / supplier claim separately as VO? </t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
@@ -1928,13 +1928,13 @@
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>For TowerCo Power part, Usually Towerco will provide AC and DC, Please suggest if the turnkey contractor needs to provide the meter and releated power material to tap to existing power system.</t>
+          <t>For TowerCo Power part, Usually Towerco will provide AC and DC, Please suggest if the bidder / supplier needs to provide the meter and releated power material to tap to existing power system.</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
         <is>
           <t>TOWERCO POWER EQUIPMENT:
-Where TowerCo supplies regulated -48V DC power directly, vendor needs only connect to the designated DC distribution breaker. Where TowerCo provides raw AC utility power, vendor supplies the submeter, ACPDB, and surge suppression.</t>
+Where TowerCo supplies regulated -48V DC power directly, supplier needs only connect to the designated DC distribution breaker. Where TowerCo provides raw AC utility power, supplier supplies the submeter, ACPDB, and surge suppression.</t>
         </is>
       </c>
       <c r="G26" s="9" t="inlineStr">
@@ -2013,7 +2013,7 @@
 1. Candidate site list in Document 07 provides audited fiber distance classes (Class A &lt;= 0.5km to Class D).
 2. Confirmed: Backhaul transport facilities (Comclark/TelTech terrestrial FOC and Starlink links) are Operator-provided.
 3. Media-tiered RTT KPIs are formally confirmed: Fiber sites &lt;= 30 ms maximum; Satellite sites &lt;= 80 ms maximum.
-4. Confirmed: Downtime caused by upstream third-party transmission outages or fiber cuts outside the site compound is excluded from vendor RAN availability penalty assessments.</t>
+4. Confirmed: Downtime caused by upstream third-party transmission outages or fiber cuts outside the site compound is excluded from supplier RAN availability penalty assessments.</t>
         </is>
       </c>
       <c r="G28" s="9" t="inlineStr">
@@ -2248,7 +2248,7 @@
       <c r="F34" s="8" t="inlineStr">
         <is>
           <t>FREQUENCY CLEARANCE TEST:
-CONFIRMED &amp; AGREED. Vendor and Operator RF teams will conduct joint baseline spectrum clearance sweeps prior to site commercial on-air to identify and resolve any legacy co-channel or adjacent interference.</t>
+CONFIRMED &amp; AGREED. Supplier and Operator RF teams will conduct joint baseline spectrum clearance sweeps prior to site commercial on-air to identify and resolve any legacy co-channel or adjacent interference.</t>
         </is>
       </c>
       <c r="G34" s="9" t="inlineStr">
@@ -2531,7 +2531,7 @@
       <c r="F42" s="8" t="inlineStr">
         <is>
           <t>OSS INTEGRATION:
-Vendor must deliver EMS/NMS for domain element management, equipped with open northbound interfaces (REST APIs, SNMPv3, Kafka) for integration into Comclark/TelTech's enterprise monitoring umbrella (AUTIN).</t>
+Supplier must deliver EMS/NMS for domain element management, equipped with open northbound interfaces (REST APIs, SNMPv3, Kafka) for integration into Comclark/TelTech's enterprise monitoring umbrella (AUTIN).</t>
         </is>
       </c>
       <c r="G42" s="9" t="inlineStr">

</xml_diff>

<commit_message>
feat(clarifications): populate Document 09 Part 3 with 57 vendor-neutral Bid Bulletin 02 items including NTC MC 006-11-2025
</commit_message>
<xml_diff>
--- a/RFP_Tender_Package/09_RFP_5G_FWA_Official_Clarifications_Responses_Master.xlsx
+++ b/RFP_Tender_Package/09_RFP_5G_FWA_Official_Clarifications_Responses_Master.xlsx
@@ -1,14 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Part 1 - RAN &amp; Spectrum" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Part 2 - Civil, Power &amp; BSS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Part 1 - RAN &amp; Spectrum" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Part 2 - Civil, Power &amp; BSS" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Part 3 - Bid Bulletin No. 2" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -49,8 +50,14 @@
       <color rgb="001E293B"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000A192F"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +74,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00F8FAFC"/>
         <bgColor rgb="00F8FAFC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
   </fills>
@@ -96,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -120,6 +133,15 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -512,7 +534,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -1079,7 +1100,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -2828,4 +2848,2104 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="68" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>COMCLARK NETWORK &amp; TECHNOLOGY CORP. / TELTECH 5G FWA NATIONWIDE TURNKEY TENDER</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>BID BULLETIN NO. 2 — OFFICIAL CLARIFICATION RESPONSES (PART 3: 5GC, RAN, CIVIL, OSS/BSS &amp; COMMERCIAL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="12" customHeight="1"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="10" t="inlineStr">
+        <is>
+          <t>Item No.</t>
+        </is>
+      </c>
+      <c r="B4" s="10" t="inlineStr">
+        <is>
+          <t>Domain Classification</t>
+        </is>
+      </c>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Document Reference</t>
+        </is>
+      </c>
+      <c r="D4" s="10" t="inlineStr">
+        <is>
+          <t>Section / Chapter Reference</t>
+        </is>
+      </c>
+      <c r="E4" s="10" t="inlineStr">
+        <is>
+          <t>Prospective Bidder Inquiry</t>
+        </is>
+      </c>
+      <c r="F4" s="10" t="inlineStr">
+        <is>
+          <t>Comclark / TelTech Official Response</t>
+        </is>
+      </c>
+      <c r="G4" s="10" t="inlineStr">
+        <is>
+          <t>Procurement Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="128" customHeight="1">
+      <c r="A5" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>5G Core &amp; IT Infrastructure (Lot 3)</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>01_RFP_5G_FWA_Master_Tender_Document.pdf</t>
+        </is>
+      </c>
+      <c r="D5" s="11" t="inlineStr">
+        <is>
+          <t>1.2
+ProgramLOT 3: CLOUD-NATIVE 5G CORE (5GC SA) &amp; DATACENTER INFRASTRUCTURE</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>Please specify how much throughput is required for 1 million users in the first phase, and how much total throughput will be needed for 3 million users in the future.</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>For Phase 1 (1,000,000 registered subscribers / initial 300,000 active broadband households), the cloud-native 5G SA Core User Plane Function (UPF) must be dimensioned for an aggregated throughput of 300 Gbps to 500 Gbps, based on an average busy-hour throughput (ABHT) of 1.5–2.0 Mbps per active subscriber with a 15–20% peak concurrency factor. For the future 3,000,000 subscriber expansion, the 5G Core architecture must support horizontal auto-scaling of containerized UPF instances up to a total aggregated throughput of 1.5 Tbps without control plane redesign.</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="112" customHeight="1">
+      <c r="A6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="11" t="inlineStr">
+        <is>
+          <t>RAN Equipment &amp; Access Hardware (Lot 1)</t>
+        </is>
+      </c>
+      <c r="C6" s="11" t="inlineStr">
+        <is>
+          <t>07_RFP_5G_FWA_Candidate_Site_List_and_Rollout_Schedule.xlsx</t>
+        </is>
+      </c>
+      <c r="D6" s="11" t="inlineStr">
+        <is>
+          <t>Phase 1 (First 1,000 Sites)</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>We have obtained the latest document and found that column T in the table only contains tower IDs without specific latitude and longitude coordinates. Could you provide these tower's latitude and longitude coordinates to support simulation and construction evaluation?</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. High-precision WGS84 geographic coordinates (6 decimal places) for all nearest towers have been populated in Document 07 (07_RFP_5G_FWA_Candidate_Site_List_and_Rollout_Schedule.xlsx) across Tab 'All 5,000 Sites' and Batch 1 through Batch 5. As noted, these tower coordinates constitute confidential operator assets provided strictly under the RFP Non-Disclosure Agreement (NDA) solely for RF propagation modeling, link simulation, and construction feasibility assessment.</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="350" customHeight="1">
+      <c r="A7" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>RAN Equipment &amp; Access Hardware (Lot 1)</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>01_RFP_5G_FWA_Master_Tender_Document.pdf</t>
+        </is>
+      </c>
+      <c r="D7" s="11" t="inlineStr">
+        <is>
+          <t>2.1 Spectrum Physics: Band n50 Advantage</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>The current capability does not support the frequency range of 1512~1517 MHz. Kindly provide more detailed RF specifications to conduct an evaluation. It is recommended to forward the NTC's demonstration spectrum requirements to the Prospective Bidder, including the following information: the suppression level requirements for RF signals in the 1432~1457 MHz range and the suppression level requirements for RF signals above 1517 MHz.</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>CONFIRMED &amp; CLARIFIED. Under National Telecommunications Commission (NTC) Memorandum Circular No. 006-11-2025 (https://ntc.gov.ph/wp-content/uploads/2025/MEMORANDUM_CIRCULAR/006-11-2025.pdf), International Mobile Telecommunications (IMT) spectrum in the 1427.0–1518.0 MHz range is officially allocated as follows:
+1. Non-Public Networks (NPN) Allocation: 1427.0–1457.0 MHz (30 MHz) is designated for dedicated private wireless / enterprise networks.
+2. Public Networks (PN) Allocation: 1457.0–1518.0 MHz (61 MHz) is designated for Public Networks, formally establishing the regulatory statutory foundation for TelTech's authorized 1457.0–1517.0 MHz (60 MHz continuous TDD) active operational carrier.
+3. Guardband &amp; Maritime Satellite Protection: A 1.0 MHz guardband (1517.0–1518.0 MHz) is established adjacent to the upper band edge. Out-of-band emissions (OOBE) into the maritime satellite service band (1518.0–1525.0 MHz) must not exceed -30 dBm/MHz at the antenna connector, strictly compliant with ITU-R M.2159-0 / WRC-15 Resolution 223.
+4. Out-of-Band Emission Limits: Unwanted radiated and conducted emissions in the adjacent 1432.0–1457.0 MHz lower block must strictly meet 3GPP TS 38.104 Category B standards with an Adjacent Channel Leakage Ratio (ACLR &gt;= 45 dB).
+5. NTC Consultations on Spectrum Expansion: TelTech is actively conducting regulatory and technical consultations with the NTC to clarify mechanisms for expanding operational spectrum bandwidth beyond the baseline 60 MHz (up to 80 MHz channel operation). Specifically, TelTech is clarifying whether supplemental operational access or secondary co-channel/adjacent-channel usage may be authorized, particularly across suburban, provincial, and rural clusters where: (a) No Non-Public Networks (NPN) are licensed or physically operating within 1427.0–1457.0 MHz; and/or (b) Incumbent mobile network operators (Globe Telecom, Smart Communications) are not actively utilizing the L-Band / Band n75 as Supplemental Downlink (SDL).
+6. Mandatory Equipment Capability: All proposed 5G NR Baseband Units (BBU), Remote Radio Units (RRU) / Active Antenna Units (AAU), and Customer Premises Equipment (CPE) RF front-ends must natively support the full 3GPP Band n50 tuning range (1432.0–1517.0 MHz, 85 MHz Instantaneous Bandwidth / IBW) in hardware. Systems must support remote software/firmware reconfiguration (e.g., expanding from 60 MHz to 80 MHz channel bandwidth or activating carrier aggregation) without requiring physical antenna swaps, hardware replacements, or tower truck rolls.</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="96" customHeight="1">
+      <c r="A8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="11" t="inlineStr">
+        <is>
+          <t>Customer Premises Equipment (Lot 7)</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>SECTION 7: 5G CUSTOMER PREMISES EQUIPMENT (CPE - LOT 7)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>There is no ODU N50 product yet, and will take a long while for development. will we consider to launch the indoor N50 first</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. TelTech authorizes a phased CPE rollout: Bidders are permitted to offer high-performance 5G Indoor Units (IDU) with high-gain internal antennas (minimum 8–10 dBi equivalent) and external antenna port capability for initial Phase 1 deployments. Bidders must concurrently commit to a roadmap delivery for high-gain Outdoor Units (ODU, &gt;= 12 dBi gain, IP67 weather-proofed) within 6 to 9 months of contract award.</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="96" customHeight="1">
+      <c r="A9" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Digital OSS/BSS &amp; Automation (Lot 4)</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="D9" s="11" t="inlineStr">
+        <is>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>Is there an existing BI/reporting system? If yes, please confirm if BSS doesn't need to provide basic report anymore.</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. The BSS/OSS platform must include native, automated BI reporting dashboards capable of generating scheduled reports (daily, weekly, monthly) in CSV, XLSX, and PDF formats for all operational, revenue, provisioning, and SLA metrics. Additionally, the platform must provide open REST APIs / secure database views to enable automated data pipeline ingestion into TelTech's enterprise analytics repository.</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="96" customHeight="1">
+      <c r="A10" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="11" t="inlineStr">
+        <is>
+          <t>Digital OSS/BSS &amp; Automation (Lot 4)</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>Is there an existing contact center? Is there a need for a separate customer ticketing system?</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. TelTech is deploying a cloud-based Contact Center as a Service (CCaaS) platform. The Bidder's BSS/CRM solution must provide standard RESTful open APIs (supporting TM Forum Open APIs including TMF621 Customer Management, TMF622 Product Ordering, and TMF632 Party Management) to integrate seamlessly with TelTech's contact center for single-pane customer service, automated CTI screen-pops, and unified trouble ticketing.</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="96" customHeight="1">
+      <c r="A11" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Digital OSS/BSS &amp; Automation (Lot 4)</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="D11" s="11" t="inlineStr">
+        <is>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>How about VAS system? Does BSS need to integrate with existing SMS?</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>The BSS platform must include standard out-of-the-box integration capabilities (via standard SMPP v3.4 and RESTful SMS API) to interface with SMSC / SMS gateways for automated transactional messaging (one-time passwords [OTP], billing alerts, provisioning status, payment reminders, and outage notifications). Third-party SMS gateway connectivity and termination aggregators will be provided by TelTech.</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="256" customHeight="1">
+      <c r="A12" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Civil Works &amp; Site Siting (Lot 5)</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>01_RFP_5G_FWA_Master_Tender_Document</t>
+        </is>
+      </c>
+      <c r="D12" s="11" t="inlineStr">
+        <is>
+          <t>LOT 5: RF PLANNING, SITE SURVEY &amp; CLUSTER OPTIMIZATION</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>We note your confirmation that the drone survey waiver is accepted. To align execution, please confirm the following:
+(a) TSSR photographic evidence shall be obtained  360° panoramic photography only via target installation height from towerco. Drone survey is not required for TSSR.
+(b) The acceptance criterion for site photographs is that they clearly depict the 360° surrounding environment (including neighbouring structures, potential obstructions, and general terrain) at a level sufficient for line-of-sight assessment. No specific camera resolution, focal length, or equipment type is required; standard photographic equipment available to the site survey team is acceptable.</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. For sites with existing towers (Class T1–T3), drone surveys shall be conducted to capture 360° panoramic photographic sweeps at antenna mounting height (and 20m, 30m, 40m AGL) to assess line-of-sight and structural clearances. Where local aviation restrictions (CAAP no-fly zones, military airspace, or adverse local weather) prohibit drone flights, manual panoramic photography taken by qualified tower riggers from the tower mounting platform is acceptable.</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="144" customHeight="1">
+      <c r="A13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Civil Works &amp; Site Siting (Lot 5)</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>05_Appendix_D_Site_Survey_RF_Planning_Civil_Power_Guidelines.pdf</t>
+        </is>
+      </c>
+      <c r="D13" s="11" t="inlineStr">
+        <is>
+          <t>4. CIVIL WORKS &amp; STRUCTURAL ENGINEERING (CLASS T4 GREENFIELD SITES)</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>For 103 sites, Do we need to consider elevated foundation in the commercial directly? If Yes, please confirm the required height. If No, Is it will be consider as VO.</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Clarified. Equipment pad foundation design for the 103 Class T4 Greenfield Monopole sites shall be determined by the site-specific hydrological survey and historical flood levels: (1) Standard Non-Flood Zone: Standard reinforced concrete equipment plinth with elevation of 300 mm (0.30 m) above finished grade level. (2) Flood-Prone Areas (50-year flood zone history): Elevated equipment platform raised 1.0 m to 1.5 m above finished grade. Civil construction works exceeding standard 300 mm plinth height necessitated by extreme local flood conditions shall be priced per the Master Rate Card (Appendix E) as an approved scope adjustment.</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="96" customHeight="1">
+      <c r="A14" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="11" t="inlineStr">
+        <is>
+          <t>Civil Works &amp; Site Siting (Lot 5)</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
+        <is>
+          <t>03_Appendix_B_Commercial_Proposal_BoQ_Templates</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>TABLE 3: LOT 2 — POWER SYSTEMS &amp; PASSIVE INFRASTRUCTURE</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>1. Please suggest the refuel of fuel tank scope is under the Contractor scope or not before we handover the site to the Operator (Finish acceptance). 
+2. If Yes, When we handover the site to the Operator, do we need to refuel the fuel tank to full.</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. Bidders are not required to provide a fully filled diesel fuel tank upon final site handover. The contractor is only responsible for supplying commissioning fuel necessary to perform the mandatory on-site load bank and generator acceptance testing (minimum 4-hour full-load burn-in). Following Provisional Acceptance Certificate (PAC), routine fuel replenishment transitions to TelTech's managed operations.</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="96" customHeight="1">
+      <c r="A15" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Civil Works &amp; Site Siting (Lot 5)</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>05_Appendix_D_Site_Survey_RF_Planning_Civil_Power_Guidelines.pdf</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>2.4 Backhaul Transmission Path Survey</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>Do we need to provide a seperate mouting Pole for the Starlink? If yes, please speficy the size or diemension for the pole.</t>
+        </is>
+      </c>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. Where Starlink LEO satellite backhaul is designated for hybrid resilience, bidders shall provide a dedicated hot-dip galvanized mounting pipe (minimum 60 mm / 2.375 inch outer diameter, 2.5 mm wall thickness) with unobstructed sky visibility. For ground-based Greenfield sites, an integrated standoff arm on the equipment gantry or perimeter fence post is acceptable; for tower sites, a tower-leg standoff clamp shall be utilized.</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="112" customHeight="1">
+      <c r="A16" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Civil Works &amp; Site Siting (Lot 5)</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>05_Appendix_D_Site_Survey_RF_Planning_Civil_Power_Guidelines.pdf</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>4. CIVIL WORKS &amp; STRUCTURAL ENGINEERING (CLASS T4 GREENFIELD SITES)</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>Please suggest how many RRU and MW need to be consider in the monopole design. and please also provide the dimension and weight for the Antenna、RRU、MW which need to be consider in the design.</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. The Class T4 Greenfield Monopole structural design shall be calculated per NSCP 2015 (EIA/TIA-222-G) for 270 km/h wind gusts, accommodating a minimum design payload of: 6x 5G Remote Radio Units (RRUs), 1x Active Antenna Unit (AAU) or 3x directional sector antennas (approx. 2.0 m length each), up to 1.2 m² total projected windward surface area for microwave transmission antennas (equivalent to 1x 1.2m or 2x 0.6m parabolic dishes), and associated feeder cables, mounting brackets, and lightning protection rod.</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="128" customHeight="1">
+      <c r="A17" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Civil Works &amp; Site Siting (Lot 5)</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>05_Appendix_D_Site_Survey_RF_Planning_Civil_Power_Guidelines
+03_Appendix_B_Commercial_Proposal_BoQ_Templates</t>
+        </is>
+      </c>
+      <c r="D17" s="11" t="inlineStr">
+        <is>
+          <t>2.3 Power Infrastructure &amp; Utility Audit
+TABLE 3: LOT 2 — POWER SYSTEMS &amp; PASSIVE INFRASTRUCTURE</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>For the New monopole sites, please suggest the AC capacity we need to apply from Coop.</t>
+        </is>
+      </c>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. The electrical service entrance shall be dimensioned for a 100A, 230V single-phase (or 3-phase where commercially available) service drop. The contractor's scope of work includes installation of the weatherhead, service mast, utility-grade meter base, manual transfer switch (MTS), main AC distribution panel with Class I+II surge protective devices (SPD), and grounding grid. Final electric cooperative (EC/Meralco) utility energization and monthly power billing accounts shall be arranged and paid directly by TelTech.</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="144" customHeight="1">
+      <c r="A18" s="4" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Digital OSS/BSS &amp; Automation (Lot 4)</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="D18" s="11" t="inlineStr">
+        <is>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>Regarding the CPE recovery rate (&gt;= 70%), the Bidder's / Contractor's 2-year warranty period allows for free replacement if any issues arise. Is such a service acceptable? The CPE recovery rate cannot be controlled.</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Accepted and clarified. The &gt;= 70% CPE Recovery Rate defined in the RFP applies strictly to churned subscriber recovery and reverse logistics (i.e. retrieving TelTech-owned CPE hardware from canceled or disconnected subscriber premises by field force teams), not OEM factory warranty returns. For defective CPE units under the 24-month Defect Liability Period (DLP), OEM free replacement applies for hardware failures due to manufacturing defects. Hardware damage resulting from proven subscriber misuse, vandalism, or force majeure shall be handled via spare parts replacement at the contracted master rate card.</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="144" customHeight="1">
+      <c r="A19" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>SLAs, KPIs &amp; Acceptance Standards (App C)</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>04_Appendix_C_SLAs_KPIs_Liquidated_Damages.pdf</t>
+        </is>
+      </c>
+      <c r="D19" s="11" t="inlineStr">
+        <is>
+          <t>3. RADIO ACCESS NETWORK (RAN) OPERATIONAL KPIS &amp; SERVICE CREDITS</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>Regarding the MTTR、NAV、SPMS SLA,
+Due to the lack of live network conditions and other inputs, it is impossible to assess the achievability of KPIs:
+SLA is recommended to be finalized based on the actual values observed during the 6 months following acceptance and commissioning.</t>
+        </is>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. The SLA targets defined in Appendix C represent standard telecommunications industry benchmarks for enterprise 5G fixed wireless networks. For Phase 1, TelTech grants a 90-day post-PAC stabilization period for each rollout cluster, during which service credits / SLA penalties for network availability (NAV) and MTTR are waived while operational baselines and spares logistics are stabilized.</t>
+        </is>
+      </c>
+      <c r="G19" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="96" customHeight="1">
+      <c r="A20" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Commercial Proposal &amp; BoQ (Doc 06)</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
+        <is>
+          <t>06_RFP_Commercial_Price_Book_and_BoQ_Template</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>The portal "3. Commercial BoQ &amp; Financing Lots 1-7" contents is different with the tender documents "06_RFP_Commercial_Price_Book_and_BoQ_Template"
+Kindly clarify which version to follow and filled?</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. The online portal Commercial BoQ tables and Excel Document 06 (06_RFP_Commercial_Price_Book_and_BoQ_Template.xlsx) have been fully harmonized. In case of any technical discrepancy, the official Excel Document 06 workbook shall serve as the governing commercial baseline.</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="208" customHeight="1">
+      <c r="A21" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Commercial Proposal &amp; BoQ (Doc 06)</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Portal "3. Commercial BoQ &amp; Financing Lots 1-7"</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>Regarding the vendor submissions in the portal under "3. Commercial BoQ &amp; Financing Lots 1-7":
+Since the current BOQ only reflects Phase 1 of the project, please clarify the pricing mechanism for the subsequent years:
+CAPEX: Assuming the Phase 1 price is fixed, will this exact pricing be applicable directly to Years 2 through 5?
+OPEX: Since vendors are only providing the OPEX for Phase 1, how should we calculate the following phases? For Phase 2, do we multiply the Phase 1 cost by 2? Does this same logic apply to the subsequent years up to Year 5?</t>
+        </is>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. Commercial proposals must quote firm, fixed unit rates and total pricing based on the complete 5,000 candidate site scope (Lot 1 through Lot 7). The project execution schedule follows the multi-batch rollout roadmap (Phase 1: 1,000 sites; Batches 2–5: 1,000 sites each).</t>
+        </is>
+      </c>
+      <c r="G21" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="96" customHeight="1">
+      <c r="A22" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="11" t="inlineStr">
+        <is>
+          <t>Commercial Proposal &amp; BoQ (Doc 06)</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
+        <is>
+          <t>Portal "3. Commercial BoQ &amp; Financing Lots 1-7"</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>As the USD to PHP exchange rate is fluctuating significantly right now, locking in a fixed rate poses a financial risk. We propose issuing all commercial documents (BoQ, PO, and Invoices) strictly in USD. If you prefer to pay in PHP, we will use the actual exchange rate on the date the payment is remitted.</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. Commercial unit rates in foreign currency (USD) and local currency (PHP) shall be evaluated using the benchmark exchange rate of USD 1.00 = PHP 55.00 as stipulated in Document 06. For imported telecom equipment (Lots 1, 2, 3, 7), contract billing and letters of credit (LC) may be settled in USD, eliminating currency conversion risk for offshore OEM suppliers.</t>
+        </is>
+      </c>
+      <c r="G22" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="96" customHeight="1">
+      <c r="A23" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
+          <t>Commercial Proposal &amp; BoQ (Doc 06)</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
+        <is>
+          <t>Portal "3. Commercial BoQ &amp; Financing Lots 1-7"</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>Kindly clarify for Commercial BoQ &amp; Financing which need to be filled online:
+1. If we are unable to provide a certain line item, should the bidder leave the unit price blank?
+2. Where is the best place to add our pricing assumptions?</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. 1. Bidders are permitted to submit proposals on an individual Lot or combination of Lots (e.g. RAN only, Core only, Civil only). Bidders not bidding on specific lots shall leave those lot pricing sheets unpriced or mark 'NO BID'. 2. Custom or proprietary value-add components may be added using the custom line-item entry rows in Document 06.</t>
+        </is>
+      </c>
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="192" customHeight="1">
+      <c r="A24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="11" t="inlineStr">
+        <is>
+          <t>Service Level Indicators &amp; Field Metrics</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>01_RFP_5G_FWA_Master_Tender_Document</t>
+        </is>
+      </c>
+      <c r="D24" s="11" t="inlineStr">
+        <is>
+          <t>LOT</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>What is installation? In which scenarios is installation required? Is the Prospective Bidder responsible for the installation? How to calculate the New Installation Dispatch Lead Time?</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Clarified. 1. Installation Scope: Installation refers to Customer Premises Equipment (CPE) installation and commissioning at subscriber premises, encompassing RF site survey, optimal wall/pole/roof mounting, outdoor Cat6 cabling up to 30m, PoE injector, Wi-Fi router setup, zero-touch provisioning via Field Force App, and speed test sign-off. When Lot 5 (Turnkey Managed Services) is awarded, the bidder is responsible for installation; otherwise, TelTech's accredited installation contractors execute the work. 2. First-Time-Right (FTR) Installation Rate Calculation: FTR Rate = [(Total Completed Installations - Repeat Truck Rolls within 14 Days) / Total Completed Installations] x 100%. Any physical revisit required within 14 calendar days due to faulty installation, cabling defect, antenna misalignment, or provisioning failure counts against FTR.</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="192" customHeight="1">
+      <c r="A25" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>Service Level Indicators &amp; Field Metrics</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>01_RFP_5G_FWA_Master_Tender_Document</t>
+        </is>
+      </c>
+      <c r="D25" s="11" t="inlineStr">
+        <is>
+          <t>LOT</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>How is the First-Time-Right (FTR) Installation Rate calculated?</t>
+        </is>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Clarified. 1. Installation Scope: Installation refers to Customer Premises Equipment (CPE) installation and commissioning at subscriber premises, encompassing RF site survey, optimal wall/pole/roof mounting, outdoor Cat6 cabling up to 30m, PoE injector, Wi-Fi router setup, zero-touch provisioning via Field Force App, and speed test sign-off. When Lot 5 (Turnkey Managed Services) is awarded, the bidder is responsible for installation; otherwise, TelTech's accredited installation contractors execute the work. 2. First-Time-Right (FTR) Installation Rate Calculation: FTR Rate = [(Total Completed Installations - Repeat Truck Rolls within 14 Days) / Total Completed Installations] x 100%. Any physical revisit required within 14 calendar days due to faulty installation, cabling defect, antenna misalignment, or provisioning failure counts against FTR.</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="96" customHeight="1">
+      <c r="A26" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
+        <is>
+          <t>Digital OSS/BSS &amp; Automation (Lot 4)</t>
+        </is>
+      </c>
+      <c r="C26" s="11" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="D26" s="11" t="inlineStr">
+        <is>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Since it is a managed service, why do we need to accept the OSS tools of the managed service?
+How to handle the tools after MS ends?</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Clarified. Bidders delivering Managed Services (MS) are required to provide all specialized tool licenses, diagnostic suites, and automation software necessary to fulfill their contracted scope and meet SLA obligations during the 5-year MS term. Following expiration of the MS term, TelTech reserves the option to transition tool operation in-house under standard commercial software maintenance terms.</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="80" customHeight="1">
+      <c r="A27" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>SLAs, KPIs &amp; Acceptance Standards (App C)</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>04_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
+        </is>
+      </c>
+      <c r="D27" s="11" t="inlineStr">
+        <is>
+          <t>3.1 Core Radio KPIs
+(Calculated 24/7/365 Nationwide)</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>Service  creadit penalty (&lt; threshold)-- does this threshold mean Minimum threshold or target standard?</t>
+        </is>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Service Credit penalties are assessed when monthly performance drops below the Minimum Threshold (not the Target Standard). Performance between the Target Standard and Minimum Threshold triggers mandatory corrective action and root-cause analysis without financial liquidated damages. Service Credits apply only when monthly performance breaches the Minimum Threshold floor.</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="96" customHeight="1">
+      <c r="A28" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>SLAs, KPIs &amp; Acceptance Standards (App C)</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>05_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
+        </is>
+      </c>
+      <c r="D28" s="11" t="inlineStr">
+        <is>
+          <t>3.1 Core Radio KPIs
+(Calculated 24/7/366 Nationwide)</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>kindly provide formula , or is it " initial RRC connection rate X erab assignment success rate"</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Per 3GPP TS 38.331 and ETSI standards, Call/Session Setup Success Rate (CSSR) is defined as: CSSR = [RRC Connection Setup Success Rate] x [QoS Flow / NG-C Setup Success Rate] x 100%. Where RRC Setup Success Rate = (Successful RRC Setup Completions / RRC Setup Requests excluding rejections) and QoS Flow Setup Success Rate = (Successful 5G QoS Flow Establishments / QoS Flow Establishment Requests).</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="64" customHeight="1">
+      <c r="A29" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>SLAs, KPIs &amp; Acceptance Standards (App C)</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>06_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
+        </is>
+      </c>
+      <c r="D29" s="11" t="inlineStr">
+        <is>
+          <t>3.1 Core Radio KPIs
+(Calculated 24/7/367 Nationwide)</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>busy hour means auto busy hour or fixed busy hour such as 19:00- 20:00?</t>
+        </is>
+      </c>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. Busy Hour is defined as Time-Consistent Busy Hour (TCBH) per 3GPP/ITU-T recommendations, determined on a per-cell basis as the continuous 60-minute interval exhibiting the highest combined uplink and downlink traffic volume over a 30-day rolling observation window.</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="96" customHeight="1">
+      <c r="A30" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>SLAs, KPIs &amp; Acceptance Standards (App C)</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>07_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>3.1 Core Radio KPIs
+(Calculated 24/7/368 Nationwide)</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>1. because there is " cell edge DL&amp;UL user speed", is this drive test KPI ? user throughput means  CPE throughput? 
+2. how to define cell edge here?</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. Cell-edge user speed is evaluated at the outer boundary of the designed coverage footprint (nominally RSRP between -95 dBm and -105 dBm). During acceptance, it is verified via stationary drive/walk tests and CPE performance logs. For operational KPI reporting, cell-edge performance is tracked via 5-percentile user throughput metrics extracted from gNodeB OSS performance counters.</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="96" customHeight="1">
+      <c r="A31" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>SLAs, KPIs &amp; Acceptance Standards (App C)</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr"/>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>5.7 Radio Frequency (RF) Cluster Optimization</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>the target of  cluster optimization is only for coverage outdoor target , any target for other KPIs such as throughput ?</t>
+        </is>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. Cluster optimization acceptance requires meeting both coverage and quality criteria: (1) Coverage: RSRP &gt;= -95 dBm over &gt;= 90% of the designated target populated settlement area; (2) Quality: SINR &gt;= 3 dB over &gt;= 90% of the cluster footprint; (3) Throughput: SSV speed targets verified at near, mid, and edge testing points; (4) Accessibility/Retainability: Cluster-wide CSSR &gt;= 97% and Call Drop Rate (CDR) &lt;= 1.5%.</t>
+        </is>
+      </c>
+      <c r="G31" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="64" customHeight="1">
+      <c r="A32" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>SLAs, KPIs &amp; Acceptance Standards (App C)</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>05_Appendix_D_Site_Survey_RF_Planning_Civil_Power_Guidelines.pdf</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>5.. SINGLE SITE VERIFICATION (SSV) &amp; CLUSTER ACCEPTANCE CRITERIA</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>for Near , mid and far location, suggest to based on simulation of typcial site ( antenna height, tilt, power ), and give proper distance of near , mid and far. or use RSRP level at -90, -100, -105</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. The classification of Near (&lt;500m), Mid (1.0–1.5 km), and Far (&gt;=2.0 km) zones is established based on baseline RF propagation modeling for 30m nominal antenna height, adjusted during physical cluster drive testing and SSV based on local terrain, clutter, and morphology.</t>
+        </is>
+      </c>
+      <c r="G32" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="112" customHeight="1">
+      <c r="A33" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>RAN Equipment &amp; Access Hardware (Lot 1)</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>01_RFP_5G_FWA_Master_Tender_Document.pdf</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>2.1 Spectrum Physics: Band n50 Advantage</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>From our general understanding, the rules for spectrum allocation are usually uniform nationwide. We would like to know whether the Operator has obtained authorization from the NTC to use 80 MHz of spectrum in areas outside the NCR.</t>
+        </is>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. The operational frequency authorization is governed by the National Telecommunications Commission (NTC) framework covering dedicated broadband wireless/private enterprise allocations within 1457.0 – 1518.0 MHz nationwide across the 5,000 candidate barangays. TelTech is finalizing formal commercial coordination with NTC; bidders shall design their RAN solutions for a standard 60 MHz TDD carrier (1457–1517 MHz) with 30 kHz Subcarrier Spacing (SCS).</t>
+        </is>
+      </c>
+      <c r="G33" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="144" customHeight="1">
+      <c r="A34" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>RAN Equipment &amp; Access Hardware (Lot 1)</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>SECTION 1: RADIO ACCESS NETWORK (RAN) TECHNICAL SPECIFICATIONS</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Antennas are generally installed at relatively high positions on towers. Towers have requirements for the antenna's windward area and wind load capacity. Does the Operator have requirements for the antenna's windward area and wind load capacity? Based on the Bidder's / Contractor's experience in delivering macro base stations, it is recommended that the windward area does not exceed 0.8 square meters.</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. For Class T1–T3 co-location sites, allowable antenna projected windward surface area, EPA (Effective Projected Area), and mounting centerline elevations are governed by each TowerCo's structural design limits and master lease agreements (MLA). Bidders shall submit equipment dimensions and weight specifications. For Class T4 Greenfield Monopoles, the tower structure must be designed to withstand NSCP 2015 wind speeds of up to 270 km/h (Category V typhoon resistance) accommodating 6 RRUs, 1 integrated active antenna (or 3 passive antennas), and up to 1.2 m² total microwave dish surface area.</t>
+        </is>
+      </c>
+      <c r="G34" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="128" customHeight="1">
+      <c r="A35" s="4" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>CPE Warranty &amp; Reverse Logistics</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
+          <t>01_RFP_5G_FWA_Master_Tender_Document.pdf</t>
+        </is>
+      </c>
+      <c r="D35" s="11" t="inlineStr"/>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>Please confirm that the mandatory base Defect Liability Period (DLP / Hardware Warranty) for network equipment remains 24 months (2 years) from the date of PAC issuance per site/phase. Furthermore, please clarify whether the Extended Warranty and Spare Parts Management Service (SPMS) for Years 3–5 (as well as Years 6–10 for TCO calculation) should be quoted as separate, optional line items per Phase in the Appendix B Commercial BoQ.</t>
+        </is>
+      </c>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. The mandatory base Defect Liability Period (DLP / Hardware Warranty) for all active network equipment (Lots 1, 2, 3, 6) is confirmed as twenty-four (24) months (2 years) commencing from the issuance of the Provisional Acceptance Certificate (PAC).</t>
+        </is>
+      </c>
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="128" customHeight="1">
+      <c r="A36" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>OEM Technical Training &amp; Enablement</t>
+        </is>
+      </c>
+      <c r="C36" s="11" t="inlineStr">
+        <is>
+          <t>01_RFP_5G_FWA_Master_Tender_Document.pdf</t>
+        </is>
+      </c>
+      <c r="D36" s="11" t="inlineStr"/>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Please clarify whether formal OEM technical training and certification programs (covering 5G SA Core, Band n50 RAN, BSS/OSS, and FMS) are required for TelTech’s engineering and O&amp;M personnel. If required, kindly provide the estimated number of trainees, preferred training location (e.g., local classroom in Manila/Clark vs. OEM headquarters), and confirm if this should be quoted as a dedicated line item in the Commercial BoQ.</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. Formal OEM technical training and certification programs covering 5G SA Core administration, Band n50 RAN RF optimization, OSS/BSS operations, and field maintenance are mandatory deliverables under Lot 5 / Services, dimensioned for at least 20 TelTech engineering personnel.</t>
+        </is>
+      </c>
+      <c r="G36" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="80" customHeight="1">
+      <c r="A37" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>Commercial Proposal &amp; BoQ (Doc 06)</t>
+        </is>
+      </c>
+      <c r="C37" s="11" t="inlineStr">
+        <is>
+          <t>Portal "3. Commercial BoQ &amp; Financing Lots 1-7"</t>
+        </is>
+      </c>
+      <c r="D37" s="11" t="inlineStr"/>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>For the Years 6–10 Cumulative OPEX (Managed Services and Extended Maintenance) in the 10-Year TCO evaluation, please confirm if bidders are permitted to include an annual Consumer Price Index (CPI) inflation indexation and FX adjustment clause to account for long-term macroeconomic fluctuations.</t>
+        </is>
+      </c>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. Bidders are permitted to quote Years 6–10 Managed Services and extended software maintenance as an optional annual escalation or fixed rate in the 10-Year Total Cost of Ownership (TCO) financial model.</t>
+        </is>
+      </c>
+      <c r="G37" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="64" customHeight="1">
+      <c r="A38" s="4" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="11" t="inlineStr">
+        <is>
+          <t>Commercial Proposal &amp; BoQ (Doc 06)</t>
+        </is>
+      </c>
+      <c r="C38" s="11" t="inlineStr">
+        <is>
+          <t>Portal "3. Commercial BoQ &amp; Financing Lots 1-7"</t>
+        </is>
+      </c>
+      <c r="D38" s="11" t="inlineStr"/>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Are all unit prices in Commercial BOQ to be quoted in VAT Ex (Value Added Tax Exclusive)?</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. All unit rates and total prices in the Commercial BoQ must be quoted exclusive of 12% Philippine Value Added Tax (VAT-Exclusive). VAT will be added as a separate line item on billing invoices in accordance with Bureau of Internal Revenue (BIR) regulations.</t>
+        </is>
+      </c>
+      <c r="G38" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="144" customHeight="1">
+      <c r="A39" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="11" t="inlineStr">
+        <is>
+          <t>Power Systems &amp; Facilities (Lot 2)</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="D39" s="11" t="inlineStr">
+        <is>
+          <t>SECTION 2: POWER SYSTEMS &amp; PASSIVE SITE INFRASTRUCTURE</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>1. Does it requires 2 Rectifier System per site or 2N Configuration? For ex: 1000 sites will be 2000 rectifier?
+2. Do they need monitoring software to cover all sites??
+3. Please confirm weather the rectifier will be installed indoor or outdoor?
+4. If outdoor installation, does all the 5000 sites is same set up?</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. (1) Each site requires one (1) high-efficiency outdoor-rated rectifier system with N+1 modular rectifier redundancy (e.g. 3x 50A modules providing 100A N+1 output). For ground-based Greenfield sites, an outdoor cabinet-housed rectifier is utilized; for tower co-location sites with limited footprint, blade/pole-mounted outdoor rectifiers are preferred. (2) Remote power monitoring software/controller with SNMPv3 / Modbus-TCP telemetry reporting into the centralized OSS is mandatory.</t>
+        </is>
+      </c>
+      <c r="G39" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="64" customHeight="1">
+      <c r="A40" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="11" t="inlineStr">
+        <is>
+          <t>Digital OSS/BSS &amp; Automation (Lot 4)</t>
+        </is>
+      </c>
+      <c r="C40" s="11" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="D40" s="11" t="inlineStr">
+        <is>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>In the FM app, is it acceptable that the navigation function redirects to an external app, such as Google Maps?</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. In the Field Force Management (FMS) mobile application, deep-linking or redirecting to external standard navigation applications (e.g., Google Maps, Waze) for route guidance to site/subscriber coordinates is fully acceptable.</t>
+        </is>
+      </c>
+      <c r="G40" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="64" customHeight="1">
+      <c r="A41" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="11" t="inlineStr">
+        <is>
+          <t>Digital OSS/BSS &amp; Automation (Lot 4)</t>
+        </is>
+      </c>
+      <c r="C41" s="11" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="D41" s="11" t="inlineStr">
+        <is>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>In the FM app, is the e-sign used only to collect users' handwritten signatures? If the electronic signature is used for strong authentication, a third-party SDK needs to be integrated. Currently, this is not supported.</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. Capturing the subscriber's handwritten signature on the mobile touchscreen interface at completion of installation/service is acceptable for job acceptance. Third-party digital signature authority (CA/PKI) integration is not mandatory for standard residential installation sign-offs.</t>
+        </is>
+      </c>
+      <c r="G41" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="80" customHeight="1">
+      <c r="A42" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="11" t="inlineStr">
+        <is>
+          <t>Digital OSS/BSS &amp; Automation (Lot 4)</t>
+        </is>
+      </c>
+      <c r="C42" s="11" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="D42" s="11" t="inlineStr">
+        <is>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>For RF signal verification, it is recommended to use professional software such as Cellular-Z to obtain more accurate and professional policy data.</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. Any industry-standard, calibrated RF measurement application or handheld scanner (e.g., Cellular-Z, G-NetTrack Pro, Nemo Handy, or OEM-native diagnostic tool) is acceptable for post-installation RF verification, provided it logs accurate RSRP, RSRQ, SINR, and Cell ID parameters into the installation completion report.</t>
+        </is>
+      </c>
+      <c r="G42" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="80" customHeight="1">
+      <c r="A43" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>Digital OSS/BSS &amp; Automation (Lot 4)</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="D43" s="11" t="inlineStr">
+        <is>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>Does the installation order involve service provisioning?</t>
+        </is>
+      </c>
+      <c r="F43" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. Installation work orders executed by field technicians must trigger automated service provisioning in the BSS/OSS upon successful on-site RF validation and customer digital sign-off, regardless of whether installation is performed by OEM managed service teams or outsourced subcontractors.</t>
+        </is>
+      </c>
+      <c r="G43" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="80" customHeight="1">
+      <c r="A44" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="11" t="inlineStr">
+        <is>
+          <t>RAN Equipment &amp; Access Hardware (Lot 1)</t>
+        </is>
+      </c>
+      <c r="C44" s="11" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="D44" s="11" t="inlineStr">
+        <is>
+          <t>SECTION 5: RF PLANNING, SITE SURVEY &amp; CLUSTER OPTIMIZATION</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>The areas covered by the issued tender documents are mostly suburban or rural regions, which do not have the capability to use 5-meter HD maps. Should we switch to using 2D maps entirely for simulation planning?</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. For rural and remote Class T4 candidate barangays where 5-meter HD clutter maps are commercially unavailable, bidders are permitted to utilize standard 20m/25m digital elevation and land-use clutter datasets supplemented by satellite imagery and digital surface models (DSM) for macro-cellular nominal RF planning and cluster simulation.</t>
+        </is>
+      </c>
+      <c r="G44" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="80" customHeight="1">
+      <c r="A45" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="11" t="inlineStr">
+        <is>
+          <t>RAN Equipment &amp; Access Hardware (Lot 1)</t>
+        </is>
+      </c>
+      <c r="C45" s="11" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="D45" s="11" t="inlineStr">
+        <is>
+          <t>SECTION 1: RADIO ACCESS NETWORK (RAN) TECHNICAL SPECIFICATIONS</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>According to the current site capability planning, the maximum average traffic of a single site does not exceed 1 Gbit/s. Therefore, the site does not need to support 2 x 10GE + 2 x 25GE interfaces. It is recommended that only the maximum capability be reserved, that is, 2 x 25GE interfaces.</t>
+        </is>
+      </c>
+      <c r="F45" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. An initial backhaul transport capacity of 1 Gbit/s per gNodeB site is acceptable for Day 1 traffic dimensioning. However, backhaul transmission interfaces (both optical transceivers and microwave links) must support hardware upgradeability to 10 Gbit/s via standard SFP+ interfaces to accommodate future multi-carrier expansion and subscriber growth.</t>
+        </is>
+      </c>
+      <c r="G45" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="96" customHeight="1">
+      <c r="A46" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="B46" s="11" t="inlineStr">
+        <is>
+          <t>RAN Equipment &amp; Access Hardware (Lot 1)</t>
+        </is>
+      </c>
+      <c r="C46" s="11" t="inlineStr">
+        <is>
+          <t>07_RFP_5G_FWA_Candidate_Site_List_and_Rollout_Schedule.xlsx</t>
+        </is>
+      </c>
+      <c r="D46" s="11" t="inlineStr">
+        <is>
+          <t>Phase 1 (First 1,000 Sites)</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Considering there are 897 co-sited base stations, is it advisable to use cabinet BBUs instead of blade BBUs?</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. Blade BBUs (outdoor zero-footprint pole/wall-mounted baseband units) are strongly preferred across all 897 co-location sites to eliminate ground footprint leasing penalties, reduce shelter space requirements, and facilitate rapid deployment. Compact outdoor cabinet BBUs are acceptable only where indoor/shelter space is pre-contracted or where blade mounting is structurally restricted by the TowerCo.</t>
+        </is>
+      </c>
+      <c r="G46" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="112" customHeight="1">
+      <c r="A47" s="4" t="n">
+        <v>43</v>
+      </c>
+      <c r="B47" s="11" t="inlineStr">
+        <is>
+          <t>Digital OSS/BSS &amp; Automation (Lot 4)</t>
+        </is>
+      </c>
+      <c r="C47" s="11" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="D47" s="11" t="inlineStr">
+        <is>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>Regarding the CPE recovery rate (&gt;= 70%), the Bidder's / Contractor's 2-year warranty period allows for free replacement if any issues arise. Is such a service acceptable? The CPE recovery rate cannot be controlled.</t>
+        </is>
+      </c>
+      <c r="F47" s="5" t="inlineStr">
+        <is>
+          <t>Accepted and clarified. The &gt;= 70% CPE Recovery Rate defined in the RFP applies strictly to churned subscriber recovery and reverse logistics (retrieving TelTech-owned CPE hardware from canceled subscriber premises), not OEM warranty returns. For defective CPE units under the 24-month DLP, OEM free replacement applies for manufacturing defects. Hardware damage resulting from proven subscriber misuse, vandalism, or force majeure shall be handled via spare parts replacement at the contracted master rate card.</t>
+        </is>
+      </c>
+      <c r="G47" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="144" customHeight="1">
+      <c r="A48" s="4" t="n">
+        <v>44</v>
+      </c>
+      <c r="B48" s="11" t="inlineStr">
+        <is>
+          <t>SLAs, KPIs &amp; Acceptance Standards (App C)</t>
+        </is>
+      </c>
+      <c r="C48" s="11" t="inlineStr">
+        <is>
+          <t>04_Appendix_C_SLAs_KPIs_Liquidated_Damages.pdf</t>
+        </is>
+      </c>
+      <c r="D48" s="11" t="inlineStr">
+        <is>
+          <t>3. RADIO ACCESS NETWORK (RAN) OPERATIONAL KPIS &amp; SERVICE CREDITS</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Regarding the MTTR、NAV、SPMS SLA,
+Due to the lack of live network conditions and other inputs, it is impossible to assess the achievability of KPIs:
+SLA is recommended to be finalized based on the actual values observed during the 6 months following acceptance and commissioning.</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. The SLA targets defined in Appendix C represent standard telecommunications industry benchmarks for enterprise 5G fixed wireless networks. For Phase 1, TelTech grants a 90-day post-PAC stabilization period for each rollout cluster, during which service credits / SLA penalties for network availability (NAV) and MTTR are waived while operational baselines and spares logistics are stabilized.</t>
+        </is>
+      </c>
+      <c r="G48" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="112" customHeight="1">
+      <c r="A49" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="B49" s="11" t="inlineStr">
+        <is>
+          <t>Service Level Indicators &amp; Field Metrics</t>
+        </is>
+      </c>
+      <c r="C49" s="11" t="inlineStr">
+        <is>
+          <t>01_RFP_5G_FWA_Master_Tender_Document</t>
+        </is>
+      </c>
+      <c r="D49" s="11" t="inlineStr">
+        <is>
+          <t>LOT</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>What is installation? In which scenarios is installation required? Is the Prospective Bidder responsible for the installation? How to calculate the New Installation Dispatch Lead Time?</t>
+        </is>
+      </c>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>Installation refers to Customer Premises Equipment (CPE) installation and commissioning at subscriber premises, encompassing RF site survey, optimal wall/pole/roof mounting, outdoor Cat6 cabling up to 30m, PoE injector, Wi-Fi router setup, zero-touch provisioning via Field Force App, and speed test sign-off. When Lot 5 (Turnkey Managed Services) is awarded, the bidder is responsible for installation; otherwise, TelTech's accredited installation contractors execute the work.</t>
+        </is>
+      </c>
+      <c r="G49" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="96" customHeight="1">
+      <c r="A50" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="B50" s="11" t="inlineStr">
+        <is>
+          <t>Service Level Indicators &amp; Field Metrics</t>
+        </is>
+      </c>
+      <c r="C50" s="11" t="inlineStr">
+        <is>
+          <t>01_RFP_5G_FWA_Master_Tender_Document</t>
+        </is>
+      </c>
+      <c r="D50" s="11" t="inlineStr">
+        <is>
+          <t>LOT</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>How is the First-Time-Right (FTR) Installation Rate calculated?</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr">
+        <is>
+          <t>The First-Time-Right (FTR) Installation Rate is calculated on a monthly rolling basis using the standard formula: FTR Rate = [(Total Completed Installations - Repeat Truck Rolls within 14 Days) / Total Completed Installations] x 100%. Any physical revisit required within 14 calendar days due to hardware failure, cabling defect, antenna misalignment, or provisioning failure counts against FTR.</t>
+        </is>
+      </c>
+      <c r="G50" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="192" customHeight="1">
+      <c r="A51" s="4" t="n">
+        <v>47</v>
+      </c>
+      <c r="B51" s="11" t="inlineStr">
+        <is>
+          <t>Service Level Indicators &amp; Field Metrics</t>
+        </is>
+      </c>
+      <c r="C51" s="11" t="inlineStr">
+        <is>
+          <t>01_RFP_5G_FWA_Master_Tender_Document</t>
+        </is>
+      </c>
+      <c r="D51" s="11" t="inlineStr">
+        <is>
+          <t>LOT</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>Please provide the procedures for CPE distribution, recovery, and maintenance.</t>
+        </is>
+      </c>
+      <c r="F51" s="5" t="inlineStr">
+        <is>
+          <t>TelTech's standard CPE lifecycle procedure operates as follows: (1) Distribution/Provisioning: Bulk CPE shipments arrive at TelTech's central staging warehouse, undergo barcode/IMEI ingestion into BSS/OSS asset tracking, and are dispatched to regional forward staging hubs. Installers scan serial numbers on-site and initiate automated zero-touch provisioning (TR-069 / USP via ACS). (2) Maintenance/RMA: Faulty units identified during subscriber trouble tickets are swapped by field technicians with buffer units from regional staging stock. Defective units are returned for RMA batching under the 24-month DLP warranty. (3) Recovery/Reverse Logistics: Upon subscriber service termination, BSS triggers a CPE Retrieval Work Order in the Field Force App. Recovered units undergo factory reset, testing, refurbishment, repackaging, and re-entry into active inventory.</t>
+        </is>
+      </c>
+      <c r="G51" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="80" customHeight="1">
+      <c r="A52" s="4" t="n">
+        <v>48</v>
+      </c>
+      <c r="B52" s="11" t="inlineStr">
+        <is>
+          <t>SLAs, KPIs &amp; Acceptance Standards (App C)</t>
+        </is>
+      </c>
+      <c r="C52" s="11" t="inlineStr">
+        <is>
+          <t>04_Appendix_C_SLAs_KPIs_Liquidated_Damages.pdf</t>
+        </is>
+      </c>
+      <c r="D52" s="11" t="inlineStr">
+        <is>
+          <t>3. RADIO ACCESS NETWORK (RAN) OPERATIONAL KPIS &amp; SERVICE CREDITS</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Does NBD in SPMS mean sending to the Bidder's / Contractor's regional spare parts warehouse?</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr">
+        <is>
+          <t>NBD (Next Business Day) replacement under the Spare Parts Management Service (SPMS) requires the replacement spare part to be delivered to the designated regional forward logistics hub / TelTech regional maintenance center within the next business day (Monday through Saturday, cut-off time 15:00) following RMA dispatch notification.</t>
+        </is>
+      </c>
+      <c r="G52" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="128" customHeight="1">
+      <c r="A53" s="4" t="n">
+        <v>49</v>
+      </c>
+      <c r="B53" s="11" t="inlineStr">
+        <is>
+          <t>Digital OSS/BSS &amp; Automation (Lot 4)</t>
+        </is>
+      </c>
+      <c r="C53" s="11" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="D53" s="11" t="inlineStr">
+        <is>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+        </is>
+      </c>
+      <c r="E53" s="5" t="inlineStr">
+        <is>
+          <t>Can the standalone OSS/BSS software scope be decoupled from  the following indicators: New Installation Dispatch Lead Time, First-Time-Right (FTR) Installation Rate, and Churned CPE Hardware Recovery Rate.</t>
+        </is>
+      </c>
+      <c r="F53" s="5" t="inlineStr">
+        <is>
+          <t>Accepted and clarified. For standalone OSS/BSS software delivery (Lot 4), SLA commitments apply to software availability, transaction processing latency, and API throughput (e.g. system uptime &gt;= 99.95%, work order dispatch generation &lt; 5 seconds). Operational field performance indicators such as New Installation Dispatch Lead Time, First-Time-Right (FTR) Installation Rate, and Churned CPE Recovery Rate apply strictly to the Managed Services &amp; Field Operations scope (Lot 5 / Appendix E) when awarded to the managed service provider.</t>
+        </is>
+      </c>
+      <c r="G53" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="112" customHeight="1">
+      <c r="A54" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>Civil Works &amp; Site Siting (Lot 5)</t>
+        </is>
+      </c>
+      <c r="C54" s="11" t="inlineStr">
+        <is>
+          <t>APPENDIX E: SERVICES STATEMENT OF WORK &amp; MASTER RATE CARD</t>
+        </is>
+      </c>
+      <c r="D54" s="11" t="inlineStr">
+        <is>
+          <t>4. MASTER SERVICES PRICING SCHEDULE &amp; COMMERCIAL RATE CARD</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>1. Please suggest on which scenario we need to do tower retrofitting works, since towerco tower is belong to towerco to do retrofitting.
+2. Tower retrofitting need to have retrofitting design first, and this scope are based on each site situation, case by case, Please suggest how to quote this item.</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. For Class T1–T3 co-location sites, tower structural strengthening is primary responsibility of the respective TowerCo under master co-location arrangements. However, to mitigate potential TowerCo lead time delays, bidders shall provide unit rate pricing in the Appendix E Master Rate Card for structural surveys, structural integrity assessments, engineering design, and structural reinforcement fabrication/installation in the event TelTech elects to self-execute retrofitting.</t>
+        </is>
+      </c>
+      <c r="G54" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="96" customHeight="1">
+      <c r="A55" s="4" t="n">
+        <v>51</v>
+      </c>
+      <c r="B55" s="11" t="inlineStr">
+        <is>
+          <t>SLAs, KPIs &amp; Acceptance Standards (App C)</t>
+        </is>
+      </c>
+      <c r="C55" s="11" t="inlineStr">
+        <is>
+          <t>05_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
+        </is>
+      </c>
+      <c r="D55" s="11" t="inlineStr">
+        <is>
+          <t>3.1 Core Radio KPIs
+(Calculated 24/7/366 Nationwide)</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>Suggest CSSR target 97%, minimum threshold 96; based on global 5G FWA network deployment benchmarks , RRC setup success rate 99% , and qos 98.5%；
+The CSSR further improvement is constrainted from terminal compatibility issues, the extent of network coverage, and transmission loss in indoor CPE.</t>
+        </is>
+      </c>
+      <c r="F55" s="5" t="inlineStr">
+        <is>
+          <t>Accepted. TelTech officially updates the nationwide Call/Session Setup Success Rate (CSSR) operational KPI as follows: Target Standard: 97.0% (revised from 99.0%); Minimum Threshold: 96.0% (revised from 97.5%). This adjustment accounts for real-world FWA CPE propagation environments while maintaining premium carrier-grade service reliability.</t>
+        </is>
+      </c>
+      <c r="G55" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="80" customHeight="1">
+      <c r="A56" s="4" t="n">
+        <v>52</v>
+      </c>
+      <c r="B56" s="11" t="inlineStr">
+        <is>
+          <t>SLAs, KPIs &amp; Acceptance Standards (App C)</t>
+        </is>
+      </c>
+      <c r="C56" s="11" t="inlineStr">
+        <is>
+          <t>05_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
+        </is>
+      </c>
+      <c r="D56" s="11" t="inlineStr">
+        <is>
+          <t>3.1 Core Radio KPIs
+(Calculated 24/7/366 Nationwide)</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Suggest target 1.5%， maximum 2%；
+The same reason that KPI CDR further improvement is constrainted from terminal compatibility issues, the extent of network coverage, and transmission loss in indoor CPE.</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr">
+        <is>
+          <t>Accepted. TelTech officially updates the nationwide Call Drop Rate (CDR) operational KPI as follows: Target Standard: &lt;= 1.5% (revised from &lt;= 0.5%); Maximum Threshold: &lt;= 2.0% (revised from &lt;= 1.0%). Service Credits apply only if monthly nationwide aggregate CDR exceeds 2.0%.</t>
+        </is>
+      </c>
+      <c r="G56" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="96" customHeight="1">
+      <c r="A57" s="4" t="n">
+        <v>53</v>
+      </c>
+      <c r="B57" s="11" t="inlineStr">
+        <is>
+          <t>SLAs, KPIs &amp; Acceptance Standards (App C)</t>
+        </is>
+      </c>
+      <c r="C57" s="11" t="inlineStr">
+        <is>
+          <t>05_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
+        </is>
+      </c>
+      <c r="D57" s="11" t="inlineStr">
+        <is>
+          <t>3.1 Core Radio KPIs
+(Calculated 24/7/366 Nationwide)</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>suggest to remove both KPIs , this is more factored by user behavior and user distribution ;also throughput already reflected in SSV KPI</t>
+        </is>
+      </c>
+      <c r="F57" s="5" t="inlineStr">
+        <is>
+          <t>Accepted in part. TelTech confirms that contractual financial liquidated damages / service credits shall not be assessed against daily instantaneous user throughput OSS counters. However, gNodeB scheduler throughput metrics (5-percentile and 50-percentile user throughput) shall remain active in OSS performance management for network traffic monitoring and capacity trigger planning.</t>
+        </is>
+      </c>
+      <c r="G57" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="80" customHeight="1">
+      <c r="A58" s="4" t="n">
+        <v>54</v>
+      </c>
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>SLAs, KPIs &amp; Acceptance Standards (App C)</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
+          <t>05_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
+        </is>
+      </c>
+      <c r="D58" s="11" t="inlineStr">
+        <is>
+          <t>3.1 Core Radio KPIs
+(Calculated 24/7/366 Nationwide)</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>There is no OSS KPI latency statistics; only drive tests are available, which have been reflected in SSV.</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr">
+        <is>
+          <t>Accepted. TelTech confirms that the round-trip latency KPI (target &lt;= 20 ms) shall be formally validated during Single Site Verification (SSV) and periodic cluster drive testing using standardized ping / TWAMP (Two-Way Active Measurement Protocol) test procedures between the test CPE and gNodeB / UPF test endpoints.</t>
+        </is>
+      </c>
+      <c r="G58" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="48" customHeight="1">
+      <c r="A59" s="4" t="n">
+        <v>55</v>
+      </c>
+      <c r="B59" s="11" t="inlineStr">
+        <is>
+          <t>SLAs, KPIs &amp; Acceptance Standards (App C)</t>
+        </is>
+      </c>
+      <c r="C59" s="11" t="inlineStr">
+        <is>
+          <t>05_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
+        </is>
+      </c>
+      <c r="D59" s="11" t="inlineStr">
+        <is>
+          <t>3.1 Core Radio KPIs
+(Calculated 24/7/366 Nationwide)</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>suggest target 0.1%，0.2% max; and PDCP layer;</t>
+        </is>
+      </c>
+      <c r="F59" s="5" t="inlineStr">
+        <is>
+          <t>Accepted. Packet loss rate shall be formally evaluated at the PDCP (Packet Data Convergence Protocol) layer per 3GPP TS 38.314 standards, with updated KPI thresholds: Target Standard: &lt;= 0.10%; Maximum Threshold: &lt;= 0.20%.</t>
+        </is>
+      </c>
+      <c r="G59" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="304" customHeight="1">
+      <c r="A60" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>RAN Equipment &amp; Access Hardware (Lot 1)</t>
+        </is>
+      </c>
+      <c r="C60" s="11" t="inlineStr">
+        <is>
+          <t>05_Appendix_D_Site_Survey_RF_Planning_Civil_Power_Guidelines.pdf</t>
+        </is>
+      </c>
+      <c r="D60" s="11" t="inlineStr">
+        <is>
+          <t>5.. SINGLE SITE VERIFICATION (SSV) &amp; CLUSTER ACCEPTANCE CRITERIA</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>from last time clarification , the Operator feedback :
+SSV SPEED TARGETS PER DISTANCE ZONE:
+- Near Zone (&lt; 500m): DL &gt;= 200 Mbps / UL &gt;= 30 Mbps.
+- Mid Zone (1.0 – 1.5 km): DL &gt;= 100 Mbps / UL &gt;= 20 Mbps.
+- Far / Cell Edge (&gt;= 2.0 km): DL &gt;= 25 Mbps / UL &gt;= 5 Mbps (minimum SLA threshold).
+Suggest to be :
+Slot configuration: DL:UL=8：2(DDDDDDDSUU) and static test,
+&gt;-80dBm: DL 200Mbps / UL 25Mbps
+[-80~-95)dBm: DL 100Mbps/UL 10Mbps
+[-95~-105)dBm: DL 35Mbps/UL 1.5Mbps</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>Accepted with clarification. TelTech approves the adoption of RSRP-correlated benchmark thresholds for static Single Site Verification (SSV) under a standard 8:2 (DDDDDDDSUU) or 7:3 TDD frame structure in a 60 MHz Band n50 channel: (1) Near Zone (RSRP &gt;= -80 dBm): DL &gt;= 200 Mbps / UL &gt;= 25 Mbps; (2) Mid Zone (-95 dBm &lt;= RSRP &lt; -80 dBm): DL &gt;= 100 Mbps / UL &gt;= 10 Mbps; (3) Cell Edge Zone (-105 dBm &lt;= RSRP &lt; -95 dBm): DL &gt;= 35 Mbps / UL &gt;= 5 Mbps (UL minimum floor of 5 Mbps is maintained to ensure reliable TCP ACK and two-way interactive video traffic). Stationary SSV measurements shall be recorded using standard outdoor/indoor CPE units matching Lot 7 technical specifications.</t>
+        </is>
+      </c>
+      <c r="G60" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="224" customHeight="1">
+      <c r="A61" s="4" t="n">
+        <v>57</v>
+      </c>
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>Backhaul &amp; Transmission Interconnect</t>
+        </is>
+      </c>
+      <c r="C61" s="11" t="inlineStr">
+        <is>
+          <t>01_RFP_5G_FWA_Master_Tender_Document</t>
+        </is>
+      </c>
+      <c r="D61" s="11" t="inlineStr">
+        <is>
+          <t>2.3 Transmission &amp; Backhaul Topology</t>
+        </is>
+      </c>
+      <c r="E61" s="5" t="inlineStr">
+        <is>
+          <t>1, The SFP of Transmission devices for Interconnections with BBU will be provided by the RAN Contractor or the Operator (TelTech)?
+2, The SFP of BBU will be 25GE/10GE Adaptive Optical Module, the SFP of transmission device will be adaptive also, or specific ones and what types they will be(need confirm the transmission port capability also)
+3, The related configurations on Transmission backhaul for BBU integration will be under the Operator or the Prospective Bidder?</t>
+        </is>
+      </c>
+      <c r="F61" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. 1. SFP Supply Boundary: The RAN bidder is responsible for supplying optical transceivers (SFPs) for all BBU/gNodeB ports. TelTech/TelTech will provide the compatible optical transceivers for the customer-facing ports on the demarcation transmission device (IP-RAN router / cell site gateway / GPON ONT). 2. Optics Specification: BBU optical modules shall be dual-rate 10GE/25GE eCPRI/CPRI/Ethernet adaptive transceivers (supporting standard 1310nm Single-Mode Fiber, LC duplex connectors, up to 10 km reach). Demarcation switch ports provided by TelTech support auto-negotiation at 10GE and 25GE. 3. Configuration Responsibilities: The RAN bidder is responsible for end-to-end BBU interface configuration (VLAN tagging, IP addressing, QoS markings per DSCP matrix, and sync synchronization IEEE 1588v2 PTP / SyncE). TelTech/TelTech transmission engineers will configure the transport network (VLAN tunneling, MPLS-VPN / SRv6 L2/L3 transport) up to the BBU handoff port.</t>
+        </is>
+      </c>
+      <c r="G61" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(bulletin-2.1): update Document 09 date to Oct 30 and codify Bid Bulletin 2.1 across portal and master register
</commit_message>
<xml_diff>
--- a/RFP_Tender_Package/09_RFP_5G_FWA_Official_Clarifications_Responses_Master.xlsx
+++ b/RFP_Tender_Package/09_RFP_5G_FWA_Official_Clarifications_Responses_Master.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Master Register (Q001 - Q100)" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Part 1 - RAN &amp; Spectrum" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Part 2 - Civil, Power &amp; BSS" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Part 3 - Bid Bulletin No. 2" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Part 3 - Bid Bulletin No. 2.1" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -509,7 +509,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H105"/>
+  <dimension ref="A1:H104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -532,7 +532,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>MASTER CLARIFICATIONS REGISTER — CONSOLIDATED INQUIRIES &amp; OFFICIAL RESPONSES (Q001 – Q100)</t>
+          <t>MASTER CLARIFICATIONS REGISTER — CONSOLIDATED INQUIRIES &amp; OFFICIAL RESPONSES (Q001 – Q100) — PROMULGATED UNDER BID BULLETIN NO. 2.1 (OCTOBER 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -615,7 +615,7 @@
       </c>
       <c r="H5" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
       </c>
       <c r="H6" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -702,7 +702,7 @@
       </c>
       <c r="H7" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="H8" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -792,7 +792,7 @@
       </c>
       <c r="H9" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="H10" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
       </c>
       <c r="H11" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -921,7 +921,7 @@
       </c>
       <c r="H12" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -962,7 +962,7 @@
       </c>
       <c r="H13" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="H14" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="H15" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1087,7 @@
       </c>
       <c r="H16" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1127,7 +1127,7 @@
       </c>
       <c r="H17" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1172,7 +1172,7 @@
       </c>
       <c r="H18" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="H19" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1257,7 +1257,7 @@
       </c>
       <c r="H20" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1302,7 +1302,7 @@
       </c>
       <c r="H21" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1347,7 @@
       </c>
       <c r="H22" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1388,7 +1388,7 @@
       </c>
       <c r="H23" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="H24" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1470,7 +1470,7 @@
       </c>
       <c r="H25" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
       </c>
       <c r="H26" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1552,7 +1552,7 @@
       </c>
       <c r="H27" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1600,7 +1600,7 @@
       </c>
       <c r="H28" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1645,7 +1645,7 @@
       </c>
       <c r="H29" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1693,7 +1693,7 @@
       </c>
       <c r="H30" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1734,7 +1734,7 @@
       </c>
       <c r="H31" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="H32" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1824,7 +1824,7 @@
       </c>
       <c r="H33" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1865,7 +1865,7 @@
       </c>
       <c r="H34" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1905,7 +1905,7 @@
       </c>
       <c r="H35" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="H36" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="H37" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="H38" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2067,7 @@
       </c>
       <c r="H39" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -2107,7 +2107,7 @@
       </c>
       <c r="H40" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -2147,7 +2147,7 @@
       </c>
       <c r="H41" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -2188,7 +2188,7 @@
       </c>
       <c r="H42" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="H43" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -2271,7 +2271,7 @@
       </c>
       <c r="H44" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2313,7 @@
       </c>
       <c r="H45" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -2349,7 +2349,7 @@
       <c r="G46" s="5" t="inlineStr"/>
       <c r="H46" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -2384,12 +2384,12 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>Clarified and incorporated into the unified baseline promulgated under Bid Bulletin No. 2.</t>
+          <t>Clarified and incorporated into the unified baseline promulgated under Bid Bulletin No. 2.1 (October 30, 2026).</t>
         </is>
       </c>
       <c r="H47" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -2424,12 +2424,12 @@
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>Clarified and incorporated into the unified baseline promulgated under Bid Bulletin No. 2.</t>
+          <t>Clarified and incorporated into the unified baseline promulgated under Bid Bulletin No. 2.1 (October 30, 2026).</t>
         </is>
       </c>
       <c r="H48" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -2470,7 +2470,7 @@
       </c>
       <c r="H49" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -2510,7 +2510,7 @@
       </c>
       <c r="H50" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -2572,7 +2572,7 @@
       </c>
       <c r="H51" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
       </c>
       <c r="H52" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -2652,7 +2652,7 @@
       </c>
       <c r="H53" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -2692,7 +2692,7 @@
       </c>
       <c r="H54" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -2732,7 +2732,7 @@
       </c>
       <c r="H55" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -2774,7 +2774,7 @@
       </c>
       <c r="H56" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -2814,7 +2814,7 @@
       </c>
       <c r="H57" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -2855,7 +2855,7 @@
       </c>
       <c r="H58" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -2895,7 +2895,7 @@
       </c>
       <c r="H59" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2935,7 @@
       </c>
       <c r="H60" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="H61" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3017,7 +3017,7 @@
       </c>
       <c r="H62" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3059,7 +3059,7 @@
       </c>
       <c r="H63" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3100,7 +3100,7 @@
       </c>
       <c r="H64" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3143,7 +3143,7 @@
       </c>
       <c r="H65" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="H66" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3225,7 +3225,7 @@
       </c>
       <c r="H67" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3255,7 +3255,8 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>What is installation? In which scenarios is installation required? Is the Contractor / Prospective Bidder responsible for the installation? How to calculate the New Installation Dispatch Lead Time?</t>
+          <t>1. Installation Scope &amp; Lead Time: What is installation? In which scenarios is installation required? Is the Contractor / Prospective Bidder responsible for the installation? How to calculate the New Installation Dispatch Lead Time?
+2. FTR Calculation: How is the First-Time-Right (FTR) Installation Rate calculated?</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr">
@@ -3265,7 +3266,7 @@
       </c>
       <c r="H68" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3275,37 +3276,38 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Q064</t>
+          <t>Q065</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>SLI</t>
+          <t>OSS &amp; BSS Integration</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>01_RFP_5G_FWA_Master_Tender_Document</t>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>How is the First-Time-Right (FTR) Installation Rate calculated?</t>
+          <t>Since it is a managed service, why do we need to accept the OSS tools of the managed service?
+How to handle the tools after MS ends?</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>Clarified. 1. Installation Scope: Installation refers to Customer Premises Equipment (CPE) installation and commissioning at subscriber premises, encompassing RF site survey, optimal wall/pole/roof mounting, outdoor Cat6 cabling up to 30m, PoE injector, Wi-Fi router setup, zero-touch provisioning via Field Force App, and speed test sign-off. When Lot 5 (Turnkey Managed Services) is awarded, the bidder is responsible for installation; otherwise, TelTech's accredited installation contractors execute the work. 2. First-Time-Right (FTR) Installation Rate Calculation: FTR Rate = [(Total Completed Installations - Repeat Truck Rolls within 14 Days) / Total Completed Installations] x 100%. Any physical revisit required within 14 calendar days due to faulty installation, cabling defect, antenna misalignment, or provisioning failure counts against FTR.</t>
+          <t>Clarified. Bidders delivering Managed Services (MS) are required to provide all specialized tool licenses, diagnostic suites, and automation software necessary to fulfill their contracted scope and meet SLA obligations during the 5-year MS term. Following expiration of the MS term, TelTech reserves the option to transition tool operation in-house under standard commercial software maintenance terms.</t>
         </is>
       </c>
       <c r="H69" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3315,38 +3317,38 @@
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Q065</t>
+          <t>Q066</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>OSS &amp; BSS Integration</t>
+          <t>SLA&amp;KPIs</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+          <t>04_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+          <t>3.1 Core Radio KPIs
+(Calculated 24/7/365 Nationwide)</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>Since it is a managed service, why do we need to accept the OSS tools of the managed service?
-How to handle the tools after MS ends?</t>
+          <t>Service  creadit penalty (&lt; threshold)-- does this threshold mean Minimum threshold or target standard?</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
-          <t>Clarified. Bidders delivering Managed Services (MS) are required to provide all specialized tool licenses, diagnostic suites, and automation software necessary to fulfill their contracted scope and meet SLA obligations during the 5-year MS term. Following expiration of the MS term, TelTech reserves the option to transition tool operation in-house under standard commercial software maintenance terms.</t>
+          <t>Service Credit penalties are assessed when monthly performance drops below the Minimum Threshold (not the Target Standard). Performance between the Target Standard and Minimum Threshold triggers mandatory corrective action and root-cause analysis without financial liquidated damages. Service Credits apply only when monthly performance breaches the Minimum Threshold floor.</t>
         </is>
       </c>
       <c r="H70" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3356,7 +3358,7 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Q066</t>
+          <t>Q067</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
@@ -3366,28 +3368,28 @@
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>04_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
+          <t>05_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
           <t>3.1 Core Radio KPIs
-(Calculated 24/7/365 Nationwide)</t>
+(Calculated 24/7/366 Nationwide)</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>Service  creadit penalty (&lt; threshold)-- does this threshold mean Minimum threshold or target standard?</t>
+          <t>kindly provide formula , or is it " initial RRC connection rate X erab assignment success rate"</t>
         </is>
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>Service Credit penalties are assessed when monthly performance drops below the Minimum Threshold (not the Target Standard). Performance between the Target Standard and Minimum Threshold triggers mandatory corrective action and root-cause analysis without financial liquidated damages. Service Credits apply only when monthly performance breaches the Minimum Threshold floor.</t>
+          <t>Per 3GPP TS 38.331 and ETSI standards, Call/Session Setup Success Rate (CSSR) is defined as: CSSR = [RRC Connection Setup Success Rate] x [QoS Flow / NG-C Setup Success Rate] x 100%. Where RRC Setup Success Rate = (Successful RRC Setup Completions / RRC Setup Requests excluding rejections) and QoS Flow Setup Success Rate = (Successful 5G QoS Flow Establishments / QoS Flow Establishment Requests).</t>
         </is>
       </c>
       <c r="H71" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3397,7 +3399,7 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Q067</t>
+          <t>Q068</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
@@ -3407,28 +3409,28 @@
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>05_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
+          <t>06_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
           <t>3.1 Core Radio KPIs
-(Calculated 24/7/366 Nationwide)</t>
+(Calculated 24/7/367 Nationwide)</t>
         </is>
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>kindly provide formula , or is it " initial RRC connection rate X erab assignment success rate"</t>
+          <t>busy hour means auto busy hour or fixed busy hour such as 19:00- 20:00?</t>
         </is>
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>Per 3GPP TS 38.331 and ETSI standards, Call/Session Setup Success Rate (CSSR) is defined as: CSSR = [RRC Connection Setup Success Rate] x [QoS Flow / NG-C Setup Success Rate] x 100%. Where RRC Setup Success Rate = (Successful RRC Setup Completions / RRC Setup Requests excluding rejections) and QoS Flow Setup Success Rate = (Successful 5G QoS Flow Establishments / QoS Flow Establishment Requests).</t>
+          <t>Confirmed. Busy Hour is defined as Time-Consistent Busy Hour (TCBH) per 3GPP/ITU-T recommendations, determined on a per-cell basis as the continuous 60-minute interval exhibiting the highest combined uplink and downlink traffic volume over a 30-day rolling observation window.</t>
         </is>
       </c>
       <c r="H72" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3438,7 +3440,7 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Q068</t>
+          <t>Q069</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
@@ -3448,28 +3450,29 @@
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>06_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
+          <t>07_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
           <t>3.1 Core Radio KPIs
-(Calculated 24/7/367 Nationwide)</t>
+(Calculated 24/7/368 Nationwide)</t>
         </is>
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>busy hour means auto busy hour or fixed busy hour such as 19:00- 20:00?</t>
+          <t>1. because there is " cell edge DL&amp;UL user speed", is this drive test KPI ? user throughput means  CPE throughput? 
+2. how to define cell edge here?</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Busy Hour is defined as Time-Consistent Busy Hour (TCBH) per 3GPP/ITU-T recommendations, determined on a per-cell basis as the continuous 60-minute interval exhibiting the highest combined uplink and downlink traffic volume over a 30-day rolling observation window.</t>
+          <t>Confirmed. Cell-edge user speed is evaluated at the outer boundary of the designed coverage footprint (nominally RSRP between -95 dBm and -105 dBm). During acceptance, it is verified via stationary drive/walk tests and CPE performance logs. For operational KPI reporting, cell-edge performance is tracked via 5-percentile user throughput metrics extracted from gNodeB OSS performance counters.</t>
         </is>
       </c>
       <c r="H73" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3482,7 @@
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Q069</t>
+          <t>Q070</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
@@ -3487,31 +3490,25 @@
           <t>SLA&amp;KPIs</t>
         </is>
       </c>
-      <c r="D74" s="5" t="inlineStr">
-        <is>
-          <t>07_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
-        </is>
-      </c>
+      <c r="D74" s="5" t="inlineStr"/>
       <c r="E74" s="5" t="inlineStr">
         <is>
-          <t>3.1 Core Radio KPIs
-(Calculated 24/7/368 Nationwide)</t>
+          <t>5.7 Radio Frequency (RF) Cluster Optimization</t>
         </is>
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>1. because there is " cell edge DL&amp;UL user speed", is this drive test KPI ? user throughput means  CPE throughput? 
-2. how to define cell edge here?</t>
+          <t>the target of  cluster optimization is only for coverage outdoor target , any target for other KPIs such as throughput ?</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Cell-edge user speed is evaluated at the outer boundary of the designed coverage footprint (nominally RSRP between -95 dBm and -105 dBm). During acceptance, it is verified via stationary drive/walk tests and CPE performance logs. For operational KPI reporting, cell-edge performance is tracked via 5-percentile user throughput metrics extracted from gNodeB OSS performance counters.</t>
+          <t>Confirmed. Cluster optimization acceptance requires meeting both coverage and quality criteria: (1) Coverage: RSRP &gt;= -95 dBm over &gt;= 90% of the designated target populated settlement area; (2) Quality: SINR &gt;= 3 dB over &gt;= 90% of the cluster footprint; (3) Throughput: SSV speed targets verified at near, mid, and edge testing points; (4) Accessibility/Retainability: Cluster-wide CSSR &gt;= 97% and Call Drop Rate (CDR) &lt;= 1.5%.</t>
         </is>
       </c>
       <c r="H74" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3521,7 +3518,7 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Q070</t>
+          <t>Q071</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
@@ -3529,25 +3526,29 @@
           <t>SLA&amp;KPIs</t>
         </is>
       </c>
-      <c r="D75" s="5" t="inlineStr"/>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>05_Appendix_D_Site_Survey_RF_Planning_Civil_Power_Guidelines.pdf</t>
+        </is>
+      </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t>5.7 Radio Frequency (RF) Cluster Optimization</t>
+          <t>5.. SINGLE SITE VERIFICATION (SSV) &amp; CLUSTER ACCEPTANCE CRITERIA</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>the target of  cluster optimization is only for coverage outdoor target , any target for other KPIs such as throughput ?</t>
+          <t>for Near , mid and far location, suggest to based on simulation of typcial site ( antenna height, tilt, power ), and give proper distance of near , mid and far. or use RSRP level at -90, -100, -105</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Cluster optimization acceptance requires meeting both coverage and quality criteria: (1) Coverage: RSRP &gt;= -95 dBm over &gt;= 90% of the designated target populated settlement area; (2) Quality: SINR &gt;= 3 dB over &gt;= 90% of the cluster footprint; (3) Throughput: SSV speed targets verified at near, mid, and edge testing points; (4) Accessibility/Retainability: Cluster-wide CSSR &gt;= 97% and Call Drop Rate (CDR) &lt;= 1.5%.</t>
+          <t>Confirmed. The classification of Near (&lt;500m), Mid (1.0–1.5 km), and Far (&gt;=2.0 km) zones is established based on baseline RF propagation modeling for 30m nominal antenna height, adjusted during physical cluster drive testing and SSV based on local terrain, clutter, and morphology.</t>
         </is>
       </c>
       <c r="H75" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3557,37 +3558,37 @@
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Q071</t>
+          <t>Q072</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>SLA&amp;KPIs</t>
+          <t>Wireless and Delivery</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>05_Appendix_D_Site_Survey_RF_Planning_Civil_Power_Guidelines.pdf</t>
+          <t>01_RFP_5G_FWA_Master_Tender_Document.pdf</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>5.. SINGLE SITE VERIFICATION (SSV) &amp; CLUSTER ACCEPTANCE CRITERIA</t>
+          <t>2.1 Spectrum Physics: Band n50 Advantage</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>for Near , mid and far location, suggest to based on simulation of typcial site ( antenna height, tilt, power ), and give proper distance of near , mid and far. or use RSRP level at -90, -100, -105</t>
+          <t>From our general understanding, the rules for spectrum allocation are usually uniform nationwide. We would like to know whether TelTech has obtained authorization from the NTC to use 80 MHz of spectrum in areas outside the NCR.</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. The classification of Near (&lt;500m), Mid (1.0–1.5 km), and Far (&gt;=2.0 km) zones is established based on baseline RF propagation modeling for 30m nominal antenna height, adjusted during physical cluster drive testing and SSV based on local terrain, clutter, and morphology.</t>
+          <t>Confirmed. The operational frequency authorization is governed by the National Telecommunications Commission (NTC) framework covering dedicated broadband wireless/private enterprise allocations within 1457.0 – 1518.0 MHz nationwide across the 5,000 candidate barangays. TelTech is finalizing formal commercial coordination with NTC; bidders shall design their RAN solutions for a standard 60 MHz TDD carrier (1457–1517 MHz) with 30 kHz Subcarrier Spacing (SCS).</t>
         </is>
       </c>
       <c r="H76" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3597,7 +3598,7 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Q072</t>
+          <t>Q073</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
@@ -3607,27 +3608,27 @@
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>01_RFP_5G_FWA_Master_Tender_Document.pdf</t>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t>2.1 Spectrum Physics: Band n50 Advantage</t>
+          <t>SECTION 1: RADIO ACCESS NETWORK (RAN) TECHNICAL SPECIFICATIONS</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>From our general understanding, the rules for spectrum allocation are usually uniform nationwide. We would like to know whether TelTech has obtained authorization from the NTC to use 80 MHz of spectrum in areas outside the NCR.</t>
+          <t>Antennas are generally installed at relatively high positions on towers. Towers have requirements for the antenna's windward area and wind load capacity. Does TelTech have requirements for the antenna's windward area and wind load capacity? Based on the Contractor / Prospective Bidder's experience in delivering macro base stations, it is recommended that the windward area does not exceed 0.8 square meters.</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. The operational frequency authorization is governed by the National Telecommunications Commission (NTC) framework covering dedicated broadband wireless/private enterprise allocations within 1457.0 – 1518.0 MHz nationwide across the 5,000 candidate barangays. TelTech is finalizing formal commercial coordination with NTC; bidders shall design their RAN solutions for a standard 60 MHz TDD carrier (1457–1517 MHz) with 30 kHz Subcarrier Spacing (SCS).</t>
+          <t>Confirmed. For Class T1–T3 co-location sites, allowable antenna projected windward surface area, EPA (Effective Projected Area), and mounting centerline elevations are governed by each TowerCo's structural design limits and master lease agreements (MLA). Bidders shall submit equipment dimensions and weight specifications. For Class T4 Greenfield Monopoles, the tower structure must be designed to withstand NSCP 2015 wind speeds of up to 270 km/h (Category V typhoon resistance) accommodating 6 RRUs, 1 integrated active antenna (or 3 passive antennas), and up to 1.2 m² total microwave dish surface area.</t>
         </is>
       </c>
       <c r="H77" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3637,37 +3638,33 @@
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Q073</t>
+          <t>Q074</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Wireless and Delivery</t>
+          <t>Warranty</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
-        </is>
-      </c>
-      <c r="E78" s="5" t="inlineStr">
-        <is>
-          <t>SECTION 1: RADIO ACCESS NETWORK (RAN) TECHNICAL SPECIFICATIONS</t>
-        </is>
-      </c>
+          <t>01_RFP_5G_FWA_Master_Tender_Document.pdf</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr"/>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>Antennas are generally installed at relatively high positions on towers. Towers have requirements for the antenna's windward area and wind load capacity. Does TelTech have requirements for the antenna's windward area and wind load capacity? Based on the Contractor / Prospective Bidder's experience in delivering macro base stations, it is recommended that the windward area does not exceed 0.8 square meters.</t>
+          <t>Please confirm that the mandatory base Defect Liability Period (DLP / Hardware Warranty) for network equipment remains 24 months (2 years) from the date of PAC issuance per site/phase. Furthermore, please clarify whether the Extended Warranty and Spare Parts Management Service (SPMS) for Years 3–5 (as well as Years 6–10 for TCO calculation) should be quoted as separate, optional line items per Phase in the Appendix B Commercial BoQ.</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. For Class T1–T3 co-location sites, allowable antenna projected windward surface area, EPA (Effective Projected Area), and mounting centerline elevations are governed by each TowerCo's structural design limits and master lease agreements (MLA). Bidders shall submit equipment dimensions and weight specifications. For Class T4 Greenfield Monopoles, the tower structure must be designed to withstand NSCP 2015 wind speeds of up to 270 km/h (Category V typhoon resistance) accommodating 6 RRUs, 1 integrated active antenna (or 3 passive antennas), and up to 1.2 m² total microwave dish surface area.</t>
+          <t>Confirmed. The mandatory base Defect Liability Period (DLP / Hardware Warranty) for all active network equipment (Lots 1, 2, 3, 6) is confirmed as twenty-four (24) months (2 years) commencing from the issuance of the Provisional Acceptance Certificate (PAC).</t>
         </is>
       </c>
       <c r="H78" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3677,12 +3674,12 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Q074</t>
+          <t>Q075</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Warranty</t>
+          <t>Training</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
@@ -3693,17 +3690,17 @@
       <c r="E79" s="5" t="inlineStr"/>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>Please confirm that the mandatory base Defect Liability Period (DLP / Hardware Warranty) for network equipment remains 24 months (2 years) from the date of PAC issuance per site/phase. Furthermore, please clarify whether the Extended Warranty and Spare Parts Management Service (SPMS) for Years 3–5 (as well as Years 6–10 for TCO calculation) should be quoted as separate, optional line items per Phase in the Appendix B Commercial BoQ.</t>
+          <t>Please clarify whether formal OEM technical training and certification programs (covering 5G SA Core, Band n50 RAN, BSS/OSS, and FMS) are required for TelTech’s engineering and O&amp;M personnel. If required, kindly provide the estimated number of trainees, preferred training location (e.g., local classroom in Manila/Clark vs. OEM headquarters), and confirm if this should be quoted as a dedicated line item in the Commercial BoQ.</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. The mandatory base Defect Liability Period (DLP / Hardware Warranty) for all active network equipment (Lots 1, 2, 3, 6) is confirmed as twenty-four (24) months (2 years) commencing from the issuance of the Provisional Acceptance Certificate (PAC).</t>
+          <t>Confirmed. Formal OEM technical training and certification programs covering 5G SA Core administration, Band n50 RAN RF optimization, OSS/BSS operations, and field maintenance are mandatory deliverables under Lot 5 / Services, dimensioned for at least 20 TelTech engineering personnel.</t>
         </is>
       </c>
       <c r="H79" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3713,33 +3710,33 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Q075</t>
+          <t>Q076</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Commercial Template</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>01_RFP_5G_FWA_Master_Tender_Document.pdf</t>
+          <t>Portal "3. Commercial BoQ &amp; Financing Lots 1-7"</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr"/>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>Please clarify whether formal OEM technical training and certification programs (covering 5G SA Core, Band n50 RAN, BSS/OSS, and FMS) are required for TelTech’s engineering and O&amp;M personnel. If required, kindly provide the estimated number of trainees, preferred training location (e.g., local classroom in Manila/Clark vs. OEM headquarters), and confirm if this should be quoted as a dedicated line item in the Commercial BoQ.</t>
+          <t>For the Years 6–10 Cumulative OPEX (Managed Services and Extended Maintenance) in the 10-Year TCO evaluation, please confirm if bidders are permitted to include an annual Consumer Price Index (CPI) inflation indexation and FX adjustment clause to account for long-term macroeconomic fluctuations.</t>
         </is>
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Formal OEM technical training and certification programs covering 5G SA Core administration, Band n50 RAN RF optimization, OSS/BSS operations, and field maintenance are mandatory deliverables under Lot 5 / Services, dimensioned for at least 20 TelTech engineering personnel.</t>
+          <t>Confirmed. Bidders are permitted to quote Years 6–10 Managed Services and extended software maintenance as an optional annual escalation or fixed rate in the 10-Year Total Cost of Ownership (TCO) financial model.</t>
         </is>
       </c>
       <c r="H80" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3749,7 +3746,7 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Q076</t>
+          <t>Q077</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
@@ -3765,17 +3762,17 @@
       <c r="E81" s="5" t="inlineStr"/>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>For the Years 6–10 Cumulative OPEX (Managed Services and Extended Maintenance) in the 10-Year TCO evaluation, please confirm if bidders are permitted to include an annual Consumer Price Index (CPI) inflation indexation and FX adjustment clause to account for long-term macroeconomic fluctuations.</t>
+          <t>Are all unit prices in Commercial BOQ to be quoted in VAT Ex (Value Added Tax Exclusive)?</t>
         </is>
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Bidders are permitted to quote Years 6–10 Managed Services and extended software maintenance as an optional annual escalation or fixed rate in the 10-Year Total Cost of Ownership (TCO) financial model.</t>
+          <t>Confirmed. All unit rates and total prices in the Commercial BoQ must be quoted exclusive of 12% Philippine Value Added Tax (VAT-Exclusive). VAT will be added as a separate line item on billing invoices in accordance with Bureau of Internal Revenue (BIR) regulations.</t>
         </is>
       </c>
       <c r="H81" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3785,61 +3782,25 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Q077</t>
+          <t>Q078</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Commercial Template</t>
+          <t>Power system and delivery</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>Portal "3. Commercial BoQ &amp; Financing Lots 1-7"</t>
-        </is>
-      </c>
-      <c r="E82" s="5" t="inlineStr"/>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>SECTION 2: POWER SYSTEMS &amp; PASSIVE SITE INFRASTRUCTURE</t>
+        </is>
+      </c>
       <c r="F82" s="5" t="inlineStr">
-        <is>
-          <t>Are all unit prices in Commercial BOQ to be quoted in VAT Ex (Value Added Tax Exclusive)?</t>
-        </is>
-      </c>
-      <c r="G82" s="5" t="inlineStr">
-        <is>
-          <t>Confirmed. All unit rates and total prices in the Commercial BoQ must be quoted exclusive of 12% Philippine Value Added Tax (VAT-Exclusive). VAT will be added as a separate line item on billing invoices in accordance with Bureau of Internal Revenue (BIR) regulations.</t>
-        </is>
-      </c>
-      <c r="H82" s="12" t="inlineStr">
-        <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="4" t="n">
-        <v>79</v>
-      </c>
-      <c r="B83" s="4" t="inlineStr">
-        <is>
-          <t>Q078</t>
-        </is>
-      </c>
-      <c r="C83" s="5" t="inlineStr">
-        <is>
-          <t>Power system and delivery</t>
-        </is>
-      </c>
-      <c r="D83" s="5" t="inlineStr">
-        <is>
-          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
-        </is>
-      </c>
-      <c r="E83" s="5" t="inlineStr">
-        <is>
-          <t>SECTION 2: POWER SYSTEMS &amp; PASSIVE SITE INFRASTRUCTURE</t>
-        </is>
-      </c>
-      <c r="F83" s="5" t="inlineStr">
         <is>
           <t>1. Does it requires 2 Rectifier System per site or 2N Configuration? For ex: 1000 sites will be 2000 rectifier?
 2. Do they need monitoring software to cover all sites??
@@ -3847,14 +3808,54 @@
 4. If outdoor installation, does all the 5000 sites is same set up?</t>
         </is>
       </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. (1) Each site requires one (1) high-efficiency outdoor-rated rectifier system with N+1 modular rectifier redundancy (e.g. 3x 50A modules providing 100A N+1 output). For ground-based Greenfield sites, an outdoor cabinet-housed rectifier is utilized; for tower co-location sites with limited footprint, blade/pole-mounted outdoor rectifiers are preferred. (2) Remote power monitoring software/controller with SNMPv3 / Modbus-TCP telemetry reporting into the centralized OSS is mandatory.</t>
+        </is>
+      </c>
+      <c r="H82" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Q079</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>OSS &amp; BSS Integration</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>In the FM app, is it acceptable that the navigation function redirects to an external app, such as Google Maps?</t>
+        </is>
+      </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. (1) Each site requires one (1) high-efficiency outdoor-rated rectifier system with N+1 modular rectifier redundancy (e.g. 3x 50A modules providing 100A N+1 output). For ground-based Greenfield sites, an outdoor cabinet-housed rectifier is utilized; for tower co-location sites with limited footprint, blade/pole-mounted outdoor rectifiers are preferred. (2) Remote power monitoring software/controller with SNMPv3 / Modbus-TCP telemetry reporting into the centralized OSS is mandatory.</t>
+          <t>Confirmed. In the Field Force Management (FMS) mobile application, deep-linking or redirecting to external standard navigation applications (e.g., Google Maps, Waze) for route guidance to site/subscriber coordinates is fully acceptable.</t>
         </is>
       </c>
       <c r="H83" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3864,7 +3865,7 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Q079</t>
+          <t>Q080</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
@@ -3884,17 +3885,17 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>In the FM app, is it acceptable that the navigation function redirects to an external app, such as Google Maps?</t>
+          <t>In the FM app, is the e-sign used only to collect users' handwritten signatures? If the electronic signature is used for strong authentication, a third-party SDK needs to be integrated. Currently, this is not supported.</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. In the Field Force Management (FMS) mobile application, deep-linking or redirecting to external standard navigation applications (e.g., Google Maps, Waze) for route guidance to site/subscriber coordinates is fully acceptable.</t>
+          <t>Confirmed. Capturing the subscriber's handwritten signature on the mobile touchscreen interface at completion of installation/service is acceptable for job acceptance. Third-party digital signature authority (CA/PKI) integration is not mandatory for standard residential installation sign-offs.</t>
         </is>
       </c>
       <c r="H84" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3904,7 +3905,7 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Q080</t>
+          <t>Q081</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
@@ -3924,17 +3925,17 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>In the FM app, is the e-sign used only to collect users' handwritten signatures? If the electronic signature is used for strong authentication, a third-party SDK needs to be integrated. Currently, this is not supported.</t>
+          <t>For RF signal verification, it is recommended to use professional software such as Cellular-Z to obtain more accurate and professional policy data.</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Capturing the subscriber's handwritten signature on the mobile touchscreen interface at completion of installation/service is acceptable for job acceptance. Third-party digital signature authority (CA/PKI) integration is not mandatory for standard residential installation sign-offs.</t>
+          <t>Confirmed. Any industry-standard, calibrated RF measurement application or handheld scanner (e.g., Cellular-Z, G-NetTrack Pro, Nemo Handy, or OEM-native diagnostic tool) is acceptable for post-installation RF verification, provided it logs accurate RSRP, RSRQ, SINR, and Cell ID parameters into the installation completion report.</t>
         </is>
       </c>
       <c r="H85" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3944,7 +3945,7 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Q081</t>
+          <t>Q082</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
@@ -3964,17 +3965,17 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>For RF signal verification, it is recommended to use professional software such as Cellular-Z to obtain more accurate and professional policy data.</t>
+          <t>Does the installation order involve service provisioning?</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Any industry-standard, calibrated RF measurement application or handheld scanner (e.g., Cellular-Z, G-NetTrack Pro, Nemo Handy, or OEM-native diagnostic tool) is acceptable for post-installation RF verification, provided it logs accurate RSRP, RSRQ, SINR, and Cell ID parameters into the installation completion report.</t>
+          <t>Confirmed. Installation work orders executed by field technicians must trigger automated service provisioning in the BSS/OSS upon successful on-site RF validation and customer digital sign-off, regardless of whether installation is performed by OEM managed service teams or outsourced subcontractors.</t>
         </is>
       </c>
       <c r="H86" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -3984,12 +3985,12 @@
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Q082</t>
+          <t>Q083</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>OSS &amp; BSS Integration</t>
+          <t>Wireless and Delivery</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
@@ -3999,22 +4000,22 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+          <t>SECTION 5: RF PLANNING, SITE SURVEY &amp; CLUSTER OPTIMIZATION</t>
         </is>
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>Does the installation order involve service provisioning?</t>
+          <t>The areas covered by the issued tender documents are mostly suburban or rural regions, which do not have the capability to use 5-meter HD maps. Should we switch to using 2D maps entirely for simulation planning?</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Installation work orders executed by field technicians must trigger automated service provisioning in the BSS/OSS upon successful on-site RF validation and customer digital sign-off, regardless of whether installation is performed by OEM managed service teams or outsourced subcontractors.</t>
+          <t>Confirmed. For rural and remote Class T4 candidate barangays where 5-meter HD clutter maps are commercially unavailable, bidders are permitted to utilize standard 20m/25m digital elevation and land-use clutter datasets supplemented by satellite imagery and digital surface models (DSM) for macro-cellular nominal RF planning and cluster simulation.</t>
         </is>
       </c>
       <c r="H87" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -4024,7 +4025,7 @@
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Q083</t>
+          <t>Q084</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
@@ -4039,22 +4040,22 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t>SECTION 5: RF PLANNING, SITE SURVEY &amp; CLUSTER OPTIMIZATION</t>
+          <t>SECTION 1: RADIO ACCESS NETWORK (RAN) TECHNICAL SPECIFICATIONS</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>The areas covered by the issued tender documents are mostly suburban or rural regions, which do not have the capability to use 5-meter HD maps. Should we switch to using 2D maps entirely for simulation planning?</t>
+          <t>According to the current site capability planning, the maximum average traffic of a single site does not exceed 1 Gbit/s. Therefore, the site does not need to support 2 x 10GE + 2 x 25GE interfaces. It is recommended that only the maximum capability be reserved, that is, 2 x 25GE interfaces.</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. For rural and remote Class T4 candidate barangays where 5-meter HD clutter maps are commercially unavailable, bidders are permitted to utilize standard 20m/25m digital elevation and land-use clutter datasets supplemented by satellite imagery and digital surface models (DSM) for macro-cellular nominal RF planning and cluster simulation.</t>
+          <t>Confirmed. An initial backhaul transport capacity of 1 Gbit/s per gNodeB site is acceptable for Day 1 traffic dimensioning. However, backhaul transmission interfaces (both optical transceivers and microwave links) must support hardware upgradeability to 10 Gbit/s via standard SFP+ interfaces to accommodate future multi-carrier expansion and subscriber growth.</t>
         </is>
       </c>
       <c r="H88" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -4064,7 +4065,7 @@
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Q084</t>
+          <t>Q085</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
@@ -4074,27 +4075,27 @@
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+          <t>07_RFP_5G_FWA_Candidate_Site_List_and_Rollout_Schedule.xlsx</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
         <is>
-          <t>SECTION 1: RADIO ACCESS NETWORK (RAN) TECHNICAL SPECIFICATIONS</t>
+          <t>Phase 1 (First 1,000 Sites)</t>
         </is>
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>According to the current site capability planning, the maximum average traffic of a single site does not exceed 1 Gbit/s. Therefore, the site does not need to support 2 x 10GE + 2 x 25GE interfaces. It is recommended that only the maximum capability be reserved, that is, 2 x 25GE interfaces.</t>
+          <t>Considering there are 897 co-sited base stations, is it advisable to use cabinet BBUs instead of blade BBUs?</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. An initial backhaul transport capacity of 1 Gbit/s per gNodeB site is acceptable for Day 1 traffic dimensioning. However, backhaul transmission interfaces (both optical transceivers and microwave links) must support hardware upgradeability to 10 Gbit/s via standard SFP+ interfaces to accommodate future multi-carrier expansion and subscriber growth.</t>
+          <t>Confirmed. Blade BBUs (outdoor zero-footprint pole/wall-mounted baseband units) are strongly preferred across all 897 co-location sites to eliminate ground footprint leasing penalties, reduce shelter space requirements, and facilitate rapid deployment. Compact outdoor cabinet BBUs are acceptable only where indoor/shelter space is pre-contracted or where blade mounting is structurally restricted by the TowerCo.</t>
         </is>
       </c>
       <c r="H89" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -4104,37 +4105,37 @@
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Q085</t>
+          <t>Q086</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Wireless and Delivery</t>
+          <t>OSS &amp; BSS Integration</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>07_RFP_5G_FWA_Candidate_Site_List_and_Rollout_Schedule.xlsx</t>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 (First 1,000 Sites)</t>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
         </is>
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>Considering there are 897 co-sited base stations, is it advisable to use cabinet BBUs instead of blade BBUs?</t>
+          <t>Regarding the CPE recovery rate (&gt;= 70%), the Contractor / Prospective Bidder's 2-year warranty period allows for free replacement if any issues arise. Is such a service acceptable? The CPE recovery rate cannot be controlled.</t>
         </is>
       </c>
       <c r="G90" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Blade BBUs (outdoor zero-footprint pole/wall-mounted baseband units) are strongly preferred across all 897 co-location sites to eliminate ground footprint leasing penalties, reduce shelter space requirements, and facilitate rapid deployment. Compact outdoor cabinet BBUs are acceptable only where indoor/shelter space is pre-contracted or where blade mounting is structurally restricted by the TowerCo.</t>
+          <t>Accepted and clarified. The &gt;= 70% CPE Recovery Rate defined in the RFP applies strictly to churned subscriber recovery and reverse logistics (retrieving TelTech-owned CPE hardware from canceled subscriber premises), not OEM warranty returns. For defective CPE units under the 24-month DLP, OEM free replacement applies for manufacturing defects. Hardware damage resulting from proven subscriber misuse, vandalism, or force majeure shall be handled via spare parts replacement at the contracted master rate card.</t>
         </is>
       </c>
       <c r="H90" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -4144,37 +4145,39 @@
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Q086</t>
+          <t>Q087</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>OSS &amp; BSS Integration</t>
+          <t>SLA&amp;KPIs</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+          <t>04_Appendix_C_SLAs_KPIs_Liquidated_Damages.pdf</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+          <t>3. RADIO ACCESS NETWORK (RAN) OPERATIONAL KPIS &amp; SERVICE CREDITS</t>
         </is>
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>Regarding the CPE recovery rate (&gt;= 70%), the Contractor / Prospective Bidder's 2-year warranty period allows for free replacement if any issues arise. Is such a service acceptable? The CPE recovery rate cannot be controlled.</t>
+          <t>Regarding the MTTR、NAV、SPMS SLA,
+Due to the lack of live network conditions and other inputs, it is impossible to assess the achievability of KPIs:
+SLA is recommended to be finalized based on the actual values observed during the 6 months following acceptance and commissioning.</t>
         </is>
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>Accepted and clarified. The &gt;= 70% CPE Recovery Rate defined in the RFP applies strictly to churned subscriber recovery and reverse logistics (retrieving TelTech-owned CPE hardware from canceled subscriber premises), not OEM warranty returns. For defective CPE units under the 24-month DLP, OEM free replacement applies for manufacturing defects. Hardware damage resulting from proven subscriber misuse, vandalism, or force majeure shall be handled via spare parts replacement at the contracted master rate card.</t>
+          <t>Confirmed. The SLA targets defined in Appendix C represent standard telecommunications industry benchmarks for enterprise 5G fixed wireless networks. For Phase 1, TelTech grants a 90-day post-PAC stabilization period for each rollout cluster, during which service credits / SLA penalties for network availability (NAV) and MTTR are waived while operational baselines and spares logistics are stabilized.</t>
         </is>
       </c>
       <c r="H91" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -4184,39 +4187,37 @@
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Q087</t>
+          <t>Q088</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>SLA&amp;KPIs</t>
+          <t>SLI</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>04_Appendix_C_SLAs_KPIs_Liquidated_Damages.pdf</t>
+          <t>01_RFP_5G_FWA_Master_Tender_Document</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
-          <t>3. RADIO ACCESS NETWORK (RAN) OPERATIONAL KPIS &amp; SERVICE CREDITS</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>Regarding the MTTR、NAV、SPMS SLA,
-Due to the lack of live network conditions and other inputs, it is impossible to assess the achievability of KPIs:
-SLA is recommended to be finalized based on the actual values observed during the 6 months following acceptance and commissioning.</t>
+          <t>What is installation? In which scenarios is installation required? Is the Contractor / Prospective Bidder responsible for the installation? How to calculate the New Installation Dispatch Lead Time?</t>
         </is>
       </c>
       <c r="G92" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. The SLA targets defined in Appendix C represent standard telecommunications industry benchmarks for enterprise 5G fixed wireless networks. For Phase 1, TelTech grants a 90-day post-PAC stabilization period for each rollout cluster, during which service credits / SLA penalties for network availability (NAV) and MTTR are waived while operational baselines and spares logistics are stabilized.</t>
+          <t>Installation refers to Customer Premises Equipment (CPE) installation and commissioning at subscriber premises, encompassing RF site survey, optimal wall/pole/roof mounting, outdoor Cat6 cabling up to 30m, PoE injector, Wi-Fi router setup, zero-touch provisioning via Field Force App, and speed test sign-off. When Lot 5 (Turnkey Managed Services) is awarded, the bidder is responsible for installation; otherwise, TelTech's accredited installation contractors execute the work.</t>
         </is>
       </c>
       <c r="H92" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4227,7 @@
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Q088</t>
+          <t>Q089</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
@@ -4246,17 +4247,17 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>What is installation? In which scenarios is installation required? Is the Contractor / Prospective Bidder responsible for the installation? How to calculate the New Installation Dispatch Lead Time?</t>
+          <t>How is the First-Time-Right (FTR) Installation Rate calculated?</t>
         </is>
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>Installation refers to Customer Premises Equipment (CPE) installation and commissioning at subscriber premises, encompassing RF site survey, optimal wall/pole/roof mounting, outdoor Cat6 cabling up to 30m, PoE injector, Wi-Fi router setup, zero-touch provisioning via Field Force App, and speed test sign-off. When Lot 5 (Turnkey Managed Services) is awarded, the bidder is responsible for installation; otherwise, TelTech's accredited installation contractors execute the work.</t>
+          <t>The First-Time-Right (FTR) Installation Rate is calculated on a monthly rolling basis using the standard formula: FTR Rate = [(Total Completed Installations - Repeat Truck Rolls within 14 Days) / Total Completed Installations] x 100%. Any physical revisit required within 14 calendar days due to hardware failure, cabling defect, antenna misalignment, or provisioning failure counts against FTR.</t>
         </is>
       </c>
       <c r="H93" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -4266,7 +4267,7 @@
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>Q089</t>
+          <t>Q090</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
@@ -4286,17 +4287,17 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>How is the First-Time-Right (FTR) Installation Rate calculated?</t>
+          <t>Please provide the procedures for CPE distribution, recovery, and maintenance.</t>
         </is>
       </c>
       <c r="G94" s="5" t="inlineStr">
         <is>
-          <t>The First-Time-Right (FTR) Installation Rate is calculated on a monthly rolling basis using the standard formula: FTR Rate = [(Total Completed Installations - Repeat Truck Rolls within 14 Days) / Total Completed Installations] x 100%. Any physical revisit required within 14 calendar days due to hardware failure, cabling defect, antenna misalignment, or provisioning failure counts against FTR.</t>
+          <t>TelTech's standard CPE lifecycle procedure operates as follows: (1) Distribution/Provisioning: Bulk CPE shipments arrive at TelTech's central staging warehouse, undergo barcode/IMEI ingestion into BSS/OSS asset tracking, and are dispatched to regional forward staging hubs. Installers scan serial numbers on-site and initiate automated zero-touch provisioning (TR-069 / USP via ACS). (2) Maintenance/RMA: Faulty units identified during subscriber trouble tickets are swapped by field technicians with buffer units from regional staging stock. Defective units are returned for RMA batching under the 24-month DLP warranty. (3) Recovery/Reverse Logistics: Upon subscriber service termination, BSS triggers a CPE Retrieval Work Order in the Field Force App. Recovered units undergo factory reset, testing, refurbishment, repackaging, and re-entry into active inventory.</t>
         </is>
       </c>
       <c r="H94" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -4306,37 +4307,37 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Q090</t>
+          <t>Q091</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>SLI</t>
+          <t>SLA&amp;KPIs</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>01_RFP_5G_FWA_Master_Tender_Document</t>
+          <t>04_Appendix_C_SLAs_KPIs_Liquidated_Damages.pdf</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>3. RADIO ACCESS NETWORK (RAN) OPERATIONAL KPIS &amp; SERVICE CREDITS</t>
         </is>
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>Please provide the procedures for CPE distribution, recovery, and maintenance.</t>
+          <t>Does NBD in SPMS mean sending to the Contractor / Prospective Bidder's regional spare parts warehouse?</t>
         </is>
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>TelTech's standard CPE lifecycle procedure operates as follows: (1) Distribution/Provisioning: Bulk CPE shipments arrive at TelTech's central staging warehouse, undergo barcode/IMEI ingestion into BSS/OSS asset tracking, and are dispatched to regional forward staging hubs. Installers scan serial numbers on-site and initiate automated zero-touch provisioning (TR-069 / USP via ACS). (2) Maintenance/RMA: Faulty units identified during subscriber trouble tickets are swapped by field technicians with buffer units from regional staging stock. Defective units are returned for RMA batching under the 24-month DLP warranty. (3) Recovery/Reverse Logistics: Upon subscriber service termination, BSS triggers a CPE Retrieval Work Order in the Field Force App. Recovered units undergo factory reset, testing, refurbishment, repackaging, and re-entry into active inventory.</t>
+          <t>NBD (Next Business Day) replacement under the Spare Parts Management Service (SPMS) requires the replacement spare part to be delivered to the designated regional forward logistics hub / TelTech regional maintenance center within the next business day (Monday through Saturday, cut-off time 15:00) following RMA dispatch notification.</t>
         </is>
       </c>
       <c r="H95" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -4346,37 +4347,37 @@
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Q091</t>
+          <t>Q092</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>SLA&amp;KPIs</t>
+          <t>OSS &amp; BSS Integration</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>04_Appendix_C_SLAs_KPIs_Liquidated_Damages.pdf</t>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t>3. RADIO ACCESS NETWORK (RAN) OPERATIONAL KPIS &amp; SERVICE CREDITS</t>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
         </is>
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>Does NBD in SPMS mean sending to the Contractor / Prospective Bidder's regional spare parts warehouse?</t>
+          <t>Can the standalone OSS/BSS software scope be decoupled from  the following indicators: New Installation Dispatch Lead Time, First-Time-Right (FTR) Installation Rate, and Churned CPE Hardware Recovery Rate.</t>
         </is>
       </c>
       <c r="G96" s="5" t="inlineStr">
         <is>
-          <t>NBD (Next Business Day) replacement under the Spare Parts Management Service (SPMS) requires the replacement spare part to be delivered to the designated regional forward logistics hub / TelTech regional maintenance center within the next business day (Monday through Saturday, cut-off time 15:00) following RMA dispatch notification.</t>
+          <t>Accepted and clarified. For standalone OSS/BSS software delivery (Lot 4), SLA commitments apply to software availability, transaction processing latency, and API throughput (e.g. system uptime &gt;= 99.95%, work order dispatch generation &lt; 5 seconds). Operational field performance indicators such as New Installation Dispatch Lead Time, First-Time-Right (FTR) Installation Rate, and Churned CPE Recovery Rate apply strictly to the Managed Services &amp; Field Operations scope (Lot 5 / Appendix E) when awarded to the managed service provider.</t>
         </is>
       </c>
       <c r="H96" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -4386,37 +4387,38 @@
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Q092</t>
+          <t>Q093</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>OSS &amp; BSS Integration</t>
+          <t>Site, civil work, and managed services</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+          <t>APPENDIX E: SERVICES STATEMENT OF WORK &amp; MASTER RATE CARD</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+          <t>4. MASTER SERVICES PRICING SCHEDULE &amp; COMMERCIAL RATE CARD</t>
         </is>
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>Can the standalone OSS/BSS software scope be decoupled from  the following indicators: New Installation Dispatch Lead Time, First-Time-Right (FTR) Installation Rate, and Churned CPE Hardware Recovery Rate.</t>
+          <t>1. Please suggest on which scenario we need to do tower retrofitting works, since towerco tower is belong to towerco to do retrofitting.
+2. Tower retrofitting need to have retrofitting design first, and this scope are based on each site situation, case by case, Please suggest how to quote this item.</t>
         </is>
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>Accepted and clarified. For standalone OSS/BSS software delivery (Lot 4), SLA commitments apply to software availability, transaction processing latency, and API throughput (e.g. system uptime &gt;= 99.95%, work order dispatch generation &lt; 5 seconds). Operational field performance indicators such as New Installation Dispatch Lead Time, First-Time-Right (FTR) Installation Rate, and Churned CPE Recovery Rate apply strictly to the Managed Services &amp; Field Operations scope (Lot 5 / Appendix E) when awarded to the managed service provider.</t>
+          <t>Confirmed. For Class T1–T3 co-location sites, tower structural strengthening is primary responsibility of the respective TowerCo under master co-location arrangements. However, to mitigate potential TowerCo lead time delays, bidders shall provide unit rate pricing in the Appendix E Master Rate Card for structural surveys, structural integrity assessments, engineering design, and structural reinforcement fabrication/installation in the event TelTech elects to self-execute retrofitting.</t>
         </is>
       </c>
       <c r="H97" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -4426,38 +4428,39 @@
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Q093</t>
+          <t>Q094</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>Site, civil work, and managed services</t>
+          <t>SLA&amp;KPIs</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>APPENDIX E: SERVICES STATEMENT OF WORK &amp; MASTER RATE CARD</t>
+          <t>05_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t>4. MASTER SERVICES PRICING SCHEDULE &amp; COMMERCIAL RATE CARD</t>
+          <t>3.1 Core Radio KPIs
+(Calculated 24/7/366 Nationwide)</t>
         </is>
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>1. Please suggest on which scenario we need to do tower retrofitting works, since towerco tower is belong to towerco to do retrofitting.
-2. Tower retrofitting need to have retrofitting design first, and this scope are based on each site situation, case by case, Please suggest how to quote this item.</t>
+          <t>Suggest CSSR target 97%, minimum threshold 96; based on huawei global FWA network experience , RRC setup success rate 99% , and qos 98.5%；
+The CSSR further improvement is constrainted from terminal compatibility issues, the extent of network coverage, and transmission loss in indoor CPE.</t>
         </is>
       </c>
       <c r="G98" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. For Class T1–T3 co-location sites, tower structural strengthening is primary responsibility of the respective TowerCo under master co-location arrangements. However, to mitigate potential TowerCo lead time delays, bidders shall provide unit rate pricing in the Appendix E Master Rate Card for structural surveys, structural integrity assessments, engineering design, and structural reinforcement fabrication/installation in the event TelTech elects to self-execute retrofitting.</t>
+          <t>Accepted. TelTech officially updates the nationwide Call/Session Setup Success Rate (CSSR) operational KPI as follows: Target Standard: 97.0% (revised from 99.0%); Minimum Threshold: 96.0% (revised from 97.5%). This adjustment accounts for real-world FWA CPE propagation environments while maintaining premium carrier-grade service reliability.</t>
         </is>
       </c>
       <c r="H98" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -4467,7 +4470,7 @@
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Q094</t>
+          <t>Q095</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
@@ -4488,18 +4491,18 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>Suggest CSSR target 97%, minimum threshold 96; based on huawei global FWA network experience , RRC setup success rate 99% , and qos 98.5%；
-The CSSR further improvement is constrainted from terminal compatibility issues, the extent of network coverage, and transmission loss in indoor CPE.</t>
+          <t>Suggest target 1.5%， maximum 2%；
+The same reason that KPI CDR further improvement is constrainted from terminal compatibility issues, the extent of network coverage, and transmission loss in indoor CPE.</t>
         </is>
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>Accepted. TelTech officially updates the nationwide Call/Session Setup Success Rate (CSSR) operational KPI as follows: Target Standard: 97.0% (revised from 99.0%); Minimum Threshold: 96.0% (revised from 97.5%). This adjustment accounts for real-world FWA CPE propagation environments while maintaining premium carrier-grade service reliability.</t>
+          <t>Accepted. TelTech officially updates the nationwide Call Drop Rate (CDR) operational KPI as follows: Target Standard: &lt;= 1.5% (revised from &lt;= 0.5%); Maximum Threshold: &lt;= 2.0% (revised from &lt;= 1.0%). Service Credits apply only if monthly nationwide aggregate CDR exceeds 2.0%.</t>
         </is>
       </c>
       <c r="H99" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -4509,7 +4512,7 @@
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Q095</t>
+          <t>Q096</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
@@ -4530,18 +4533,17 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>Suggest target 1.5%， maximum 2%；
-The same reason that KPI CDR further improvement is constrainted from terminal compatibility issues, the extent of network coverage, and transmission loss in indoor CPE.</t>
+          <t>suggest to remove both KPIs , this is more factored by user behavior and user distribution ;also throughput already reflected in SSV KPI</t>
         </is>
       </c>
       <c r="G100" s="5" t="inlineStr">
         <is>
-          <t>Accepted. TelTech officially updates the nationwide Call Drop Rate (CDR) operational KPI as follows: Target Standard: &lt;= 1.5% (revised from &lt;= 0.5%); Maximum Threshold: &lt;= 2.0% (revised from &lt;= 1.0%). Service Credits apply only if monthly nationwide aggregate CDR exceeds 2.0%.</t>
+          <t>Accepted in part. TelTech confirms that contractual financial liquidated damages / service credits shall not be assessed against daily instantaneous user throughput OSS counters. However, gNodeB scheduler throughput metrics (5-percentile and 50-percentile user throughput) shall remain active in OSS performance management for network traffic monitoring and capacity trigger planning.</t>
         </is>
       </c>
       <c r="H100" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4553,7 @@
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Q096</t>
+          <t>Q097</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
@@ -4572,17 +4574,17 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>suggest to remove both KPIs , this is more factored by user behavior and user distribution ;also throughput already reflected in SSV KPI</t>
+          <t>There is no OSS KPI latency statistics; only drive tests are available, which have been reflected in SSV.</t>
         </is>
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>Accepted in part. TelTech confirms that contractual financial liquidated damages / service credits shall not be assessed against daily instantaneous user throughput OSS counters. However, gNodeB scheduler throughput metrics (5-percentile and 50-percentile user throughput) shall remain active in OSS performance management for network traffic monitoring and capacity trigger planning.</t>
+          <t>Accepted. TelTech confirms that the round-trip latency KPI (target &lt;= 20 ms) shall be formally validated during Single Site Verification (SSV) and periodic cluster drive testing using standardized ping / TWAMP (Two-Way Active Measurement Protocol) test procedures between the test CPE and gNodeB / UPF test endpoints.</t>
         </is>
       </c>
       <c r="H101" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -4592,7 +4594,7 @@
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Q097</t>
+          <t>Q098</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
@@ -4613,17 +4615,17 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>There is no OSS KPI latency statistics; only drive tests are available, which have been reflected in SSV.</t>
+          <t>suggest target 0.1%，0.2% max; and PDCP layer;</t>
         </is>
       </c>
       <c r="G102" s="5" t="inlineStr">
         <is>
-          <t>Accepted. TelTech confirms that the round-trip latency KPI (target &lt;= 20 ms) shall be formally validated during Single Site Verification (SSV) and periodic cluster drive testing using standardized ping / TWAMP (Two-Way Active Measurement Protocol) test procedures between the test CPE and gNodeB / UPF test endpoints.</t>
+          <t>Accepted. Packet loss rate shall be formally evaluated at the PDCP (Packet Data Convergence Protocol) layer per 3GPP TS 38.314 standards, with updated KPI thresholds: Target Standard: &lt;= 0.10%; Maximum Threshold: &lt;= 0.20%.</t>
         </is>
       </c>
       <c r="H102" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -4633,66 +4635,25 @@
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Q098</t>
+          <t>Q099</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>SLA&amp;KPIs</t>
+          <t>Wireless and Delivery</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>05_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
+          <t>05_Appendix_D_Site_Survey_RF_Planning_Civil_Power_Guidelines.pdf</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t>3.1 Core Radio KPIs
-(Calculated 24/7/366 Nationwide)</t>
+          <t>5.. SINGLE SITE VERIFICATION (SSV) &amp; CLUSTER ACCEPTANCE CRITERIA</t>
         </is>
       </c>
       <c r="F103" s="5" t="inlineStr">
-        <is>
-          <t>suggest target 0.1%，0.2% max; and PDCP layer;</t>
-        </is>
-      </c>
-      <c r="G103" s="5" t="inlineStr">
-        <is>
-          <t>Accepted. Packet loss rate shall be formally evaluated at the PDCP (Packet Data Convergence Protocol) layer per 3GPP TS 38.314 standards, with updated KPI thresholds: Target Standard: &lt;= 0.10%; Maximum Threshold: &lt;= 0.20%.</t>
-        </is>
-      </c>
-      <c r="H103" s="12" t="inlineStr">
-        <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="B104" s="4" t="inlineStr">
-        <is>
-          <t>Q099</t>
-        </is>
-      </c>
-      <c r="C104" s="5" t="inlineStr">
-        <is>
-          <t>Wireless and Delivery</t>
-        </is>
-      </c>
-      <c r="D104" s="5" t="inlineStr">
-        <is>
-          <t>05_Appendix_D_Site_Survey_RF_Planning_Civil_Power_Guidelines.pdf</t>
-        </is>
-      </c>
-      <c r="E104" s="5" t="inlineStr">
-        <is>
-          <t>5.. SINGLE SITE VERIFICATION (SSV) &amp; CLUSTER ACCEPTANCE CRITERIA</t>
-        </is>
-      </c>
-      <c r="F104" s="5" t="inlineStr">
         <is>
           <t>from last time clarification , converage feedback :
 SSV SPEED TARGETS PER DISTANCE ZONE:
@@ -4706,56 +4667,56 @@
 [-95~-105)dBm: DL 35Mbps/UL 1.5Mbps</t>
         </is>
       </c>
-      <c r="G104" s="5" t="inlineStr">
+      <c r="G103" s="5" t="inlineStr">
         <is>
           <t>Accepted with clarification. TelTech approves the adoption of RSRP-correlated benchmark thresholds for static Single Site Verification (SSV) under a standard 8:2 (DDDDDDDSUU) or 7:3 TDD frame structure in a 60 MHz Band n50 channel: (1) Near Zone (RSRP &gt;= -80 dBm): DL &gt;= 200 Mbps / UL &gt;= 25 Mbps; (2) Mid Zone (-95 dBm &lt;= RSRP &lt; -80 dBm): DL &gt;= 100 Mbps / UL &gt;= 10 Mbps; (3) Cell Edge Zone (-105 dBm &lt;= RSRP &lt; -95 dBm): DL &gt;= 35 Mbps / UL &gt;= 5 Mbps (UL minimum floor of 5 Mbps is maintained to ensure reliable TCP ACK and two-way interactive video traffic). Stationary SSV measurements shall be recorded using standard outdoor/indoor CPE units matching Lot 7 technical specifications.</t>
         </is>
       </c>
-      <c r="H104" s="12" t="inlineStr">
-        <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="4" t="n">
-        <v>101</v>
-      </c>
-      <c r="B105" s="4" t="inlineStr">
+      <c r="H103" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
         <is>
           <t>Q100</t>
         </is>
       </c>
-      <c r="C105" s="5" t="inlineStr">
+      <c r="C104" s="5" t="inlineStr">
         <is>
           <t>Transmission</t>
         </is>
       </c>
-      <c r="D105" s="5" t="inlineStr">
+      <c r="D104" s="5" t="inlineStr">
         <is>
           <t>01_RFP_5G_FWA_Master_Tender_Document</t>
         </is>
       </c>
-      <c r="E105" s="5" t="inlineStr">
+      <c r="E104" s="5" t="inlineStr">
         <is>
           <t>2.3 Transmission &amp; Backhaul Topology</t>
         </is>
       </c>
-      <c r="F105" s="5" t="inlineStr">
+      <c r="F104" s="5" t="inlineStr">
         <is>
           <t>1, The SFP of Transmission devices for Interconnections with BBU will be provided by the Contractor / Prospective Bidder or TelTech/TelTech?
 2, The SFP of BBU will be 25GE/10GE Adaptive Optical Module, the SFP of transmission device will be adaptive also, or specific ones and what types they will be(need confirm the transmission port capability also)
 3, The related configurations on Transmission backhaul for BBU integration will be under TelTech or the Contractor / Prospective Bidder?</t>
         </is>
       </c>
-      <c r="G105" s="5" t="inlineStr">
+      <c r="G104" s="5" t="inlineStr">
         <is>
           <t>Confirmed. 1. SFP Supply Boundary: The RAN bidder is responsible for supplying optical transceivers (SFPs) for all BBU/gNodeB ports. TelTech/TelTech will provide the compatible optical transceivers for the customer-facing ports on the demarcation transmission device (IP-RAN router / cell site gateway / GPON ONT). 2. Optics Specification: BBU optical modules shall be dual-rate 10GE/25GE eCPRI/CPRI/Ethernet adaptive transceivers (supporting standard 1310nm Single-Mode Fiber, LC duplex connectors, up to 10 km reach). Demarcation switch ports provided by TelTech support auto-negotiation at 10GE and 25GE. 3. Configuration Responsibilities: The RAN bidder is responsible for end-to-end BBU interface configuration (VLAN tagging, IP addressing, QoS markings per DSCP matrix, and sync synchronization IEEE 1588v2 PTP / SyncE). TelTech/TelTech transmission engineers will configure the transport network (VLAN tunneling, MPLS-VPN / SRv6 L2/L3 transport) up to the BBU handoff port.</t>
         </is>
       </c>
-      <c r="H105" s="12" t="inlineStr">
-        <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+      <c r="H104" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -7118,7 +7079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H105"/>
+  <dimension ref="A1:H104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -7141,7 +7102,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>BID BULLETIN NO. 2.1 — CONSOLIDATED MASTER CLARIFICATIONS (QUESTIONS 1 TO 100)</t>
+          <t>BID BULLETIN NO. 2.1 — CONSOLIDATED MASTER CLARIFICATIONS (QUESTIONS 1 TO 100) — PROMULGATED OCTOBER 30, 2026</t>
         </is>
       </c>
     </row>
@@ -7224,7 +7185,7 @@
       </c>
       <c r="H5" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7265,7 +7226,7 @@
       </c>
       <c r="H6" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7311,7 +7272,7 @@
       </c>
       <c r="H7" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7355,7 +7316,7 @@
       </c>
       <c r="H8" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7401,7 +7362,7 @@
       </c>
       <c r="H9" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7448,7 +7409,7 @@
       </c>
       <c r="H10" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7489,7 +7450,7 @@
       </c>
       <c r="H11" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7530,7 +7491,7 @@
       </c>
       <c r="H12" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7571,7 +7532,7 @@
       </c>
       <c r="H13" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7612,7 +7573,7 @@
       </c>
       <c r="H14" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7653,7 +7614,7 @@
       </c>
       <c r="H15" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7696,7 +7657,7 @@
       </c>
       <c r="H16" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7736,7 +7697,7 @@
       </c>
       <c r="H17" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7781,7 +7742,7 @@
       </c>
       <c r="H18" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7819,7 +7780,7 @@
       </c>
       <c r="H19" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7866,7 +7827,7 @@
       </c>
       <c r="H20" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7911,7 +7872,7 @@
       </c>
       <c r="H21" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7956,7 +7917,7 @@
       </c>
       <c r="H22" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -7997,7 +7958,7 @@
       </c>
       <c r="H23" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8038,7 +7999,7 @@
       </c>
       <c r="H24" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8079,7 +8040,7 @@
       </c>
       <c r="H25" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8120,7 +8081,7 @@
       </c>
       <c r="H26" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8161,7 +8122,7 @@
       </c>
       <c r="H27" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8209,7 +8170,7 @@
       </c>
       <c r="H28" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8254,7 +8215,7 @@
       </c>
       <c r="H29" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8302,7 +8263,7 @@
       </c>
       <c r="H30" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8343,7 +8304,7 @@
       </c>
       <c r="H31" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8390,7 +8351,7 @@
       </c>
       <c r="H32" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8433,7 +8394,7 @@
       </c>
       <c r="H33" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8474,7 +8435,7 @@
       </c>
       <c r="H34" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8514,7 +8475,7 @@
       </c>
       <c r="H35" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8554,7 +8515,7 @@
       </c>
       <c r="H36" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8594,7 +8555,7 @@
       </c>
       <c r="H37" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8636,7 +8597,7 @@
       </c>
       <c r="H38" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8676,7 +8637,7 @@
       </c>
       <c r="H39" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8716,7 +8677,7 @@
       </c>
       <c r="H40" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8756,7 +8717,7 @@
       </c>
       <c r="H41" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8797,7 +8758,7 @@
       </c>
       <c r="H42" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8837,7 +8798,7 @@
       </c>
       <c r="H43" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8880,7 +8841,7 @@
       </c>
       <c r="H44" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8922,7 +8883,7 @@
       </c>
       <c r="H45" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8958,7 +8919,7 @@
       <c r="G46" s="5" t="n"/>
       <c r="H46" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 1)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -8993,12 +8954,12 @@
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>Clarified and incorporated into the unified baseline promulgated under Bid Bulletin No. 2.</t>
+          <t>Clarified and incorporated into the unified baseline promulgated under Bid Bulletin No. 2.1 (October 30, 2026).</t>
         </is>
       </c>
       <c r="H47" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -9033,12 +8994,12 @@
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>Clarified and incorporated into the unified baseline promulgated under Bid Bulletin No. 2.</t>
+          <t>Clarified and incorporated into the unified baseline promulgated under Bid Bulletin No. 2.1 (October 30, 2026).</t>
         </is>
       </c>
       <c r="H48" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 1 - Oct 21, 2026)</t>
         </is>
       </c>
     </row>
@@ -9079,7 +9040,7 @@
       </c>
       <c r="H49" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9119,7 +9080,7 @@
       </c>
       <c r="H50" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9181,7 +9142,7 @@
       </c>
       <c r="H51" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9221,7 +9182,7 @@
       </c>
       <c r="H52" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9261,7 +9222,7 @@
       </c>
       <c r="H53" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9301,7 +9262,7 @@
       </c>
       <c r="H54" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9341,7 +9302,7 @@
       </c>
       <c r="H55" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9383,7 +9344,7 @@
       </c>
       <c r="H56" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9423,7 +9384,7 @@
       </c>
       <c r="H57" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9464,7 +9425,7 @@
       </c>
       <c r="H58" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9504,7 +9465,7 @@
       </c>
       <c r="H59" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9544,7 +9505,7 @@
       </c>
       <c r="H60" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9586,7 +9547,7 @@
       </c>
       <c r="H61" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9626,7 +9587,7 @@
       </c>
       <c r="H62" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9668,7 +9629,7 @@
       </c>
       <c r="H63" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9709,7 +9670,7 @@
       </c>
       <c r="H64" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9752,7 +9713,7 @@
       </c>
       <c r="H65" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9792,7 +9753,7 @@
       </c>
       <c r="H66" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9834,7 +9795,7 @@
       </c>
       <c r="H67" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9864,7 +9825,8 @@
       </c>
       <c r="F68" s="5" t="inlineStr">
         <is>
-          <t>What is installation? In which scenarios is installation required? Is the Contractor / Prospective Bidder responsible for the installation? How to calculate the New Installation Dispatch Lead Time?</t>
+          <t>1. Installation Scope &amp; Lead Time: What is installation? In which scenarios is installation required? Is the Contractor / Prospective Bidder responsible for the installation? How to calculate the New Installation Dispatch Lead Time?
+2. FTR Calculation: How is the First-Time-Right (FTR) Installation Rate calculated?</t>
         </is>
       </c>
       <c r="G68" s="5" t="inlineStr">
@@ -9874,7 +9836,7 @@
       </c>
       <c r="H68" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9884,37 +9846,38 @@
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Q064</t>
+          <t>Q065</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>SLI</t>
+          <t>OSS &amp; BSS Integration</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>01_RFP_5G_FWA_Master_Tender_Document</t>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
         </is>
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>How is the First-Time-Right (FTR) Installation Rate calculated?</t>
+          <t>Since it is a managed service, why do we need to accept the OSS tools of the managed service?
+How to handle the tools after MS ends?</t>
         </is>
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>Clarified. 1. Installation Scope: Installation refers to Customer Premises Equipment (CPE) installation and commissioning at subscriber premises, encompassing RF site survey, optimal wall/pole/roof mounting, outdoor Cat6 cabling up to 30m, PoE injector, Wi-Fi router setup, zero-touch provisioning via Field Force App, and speed test sign-off. When Lot 5 (Turnkey Managed Services) is awarded, the bidder is responsible for installation; otherwise, TelTech's accredited installation contractors execute the work. 2. First-Time-Right (FTR) Installation Rate Calculation: FTR Rate = [(Total Completed Installations - Repeat Truck Rolls within 14 Days) / Total Completed Installations] x 100%. Any physical revisit required within 14 calendar days due to faulty installation, cabling defect, antenna misalignment, or provisioning failure counts against FTR.</t>
+          <t>Clarified. Bidders delivering Managed Services (MS) are required to provide all specialized tool licenses, diagnostic suites, and automation software necessary to fulfill their contracted scope and meet SLA obligations during the 5-year MS term. Following expiration of the MS term, TelTech reserves the option to transition tool operation in-house under standard commercial software maintenance terms.</t>
         </is>
       </c>
       <c r="H69" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9924,38 +9887,38 @@
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>Q065</t>
+          <t>Q066</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>OSS &amp; BSS Integration</t>
+          <t>SLA&amp;KPIs</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+          <t>04_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
         <is>
-          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+          <t>3.1 Core Radio KPIs
+(Calculated 24/7/365 Nationwide)</t>
         </is>
       </c>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>Since it is a managed service, why do we need to accept the OSS tools of the managed service?
-How to handle the tools after MS ends?</t>
+          <t>Service  creadit penalty (&lt; threshold)-- does this threshold mean Minimum threshold or target standard?</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
-          <t>Clarified. Bidders delivering Managed Services (MS) are required to provide all specialized tool licenses, diagnostic suites, and automation software necessary to fulfill their contracted scope and meet SLA obligations during the 5-year MS term. Following expiration of the MS term, TelTech reserves the option to transition tool operation in-house under standard commercial software maintenance terms.</t>
+          <t>Service Credit penalties are assessed when monthly performance drops below the Minimum Threshold (not the Target Standard). Performance between the Target Standard and Minimum Threshold triggers mandatory corrective action and root-cause analysis without financial liquidated damages. Service Credits apply only when monthly performance breaches the Minimum Threshold floor.</t>
         </is>
       </c>
       <c r="H70" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -9965,7 +9928,7 @@
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>Q066</t>
+          <t>Q067</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
@@ -9975,28 +9938,28 @@
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>04_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
+          <t>05_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
         <is>
           <t>3.1 Core Radio KPIs
-(Calculated 24/7/365 Nationwide)</t>
+(Calculated 24/7/366 Nationwide)</t>
         </is>
       </c>
       <c r="F71" s="5" t="inlineStr">
         <is>
-          <t>Service  creadit penalty (&lt; threshold)-- does this threshold mean Minimum threshold or target standard?</t>
+          <t>kindly provide formula , or is it " initial RRC connection rate X erab assignment success rate"</t>
         </is>
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>Service Credit penalties are assessed when monthly performance drops below the Minimum Threshold (not the Target Standard). Performance between the Target Standard and Minimum Threshold triggers mandatory corrective action and root-cause analysis without financial liquidated damages. Service Credits apply only when monthly performance breaches the Minimum Threshold floor.</t>
+          <t>Per 3GPP TS 38.331 and ETSI standards, Call/Session Setup Success Rate (CSSR) is defined as: CSSR = [RRC Connection Setup Success Rate] x [QoS Flow / NG-C Setup Success Rate] x 100%. Where RRC Setup Success Rate = (Successful RRC Setup Completions / RRC Setup Requests excluding rejections) and QoS Flow Setup Success Rate = (Successful 5G QoS Flow Establishments / QoS Flow Establishment Requests).</t>
         </is>
       </c>
       <c r="H71" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10006,7 +9969,7 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>Q067</t>
+          <t>Q068</t>
         </is>
       </c>
       <c r="C72" s="5" t="inlineStr">
@@ -10016,28 +9979,28 @@
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>05_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
+          <t>06_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
         <is>
           <t>3.1 Core Radio KPIs
-(Calculated 24/7/366 Nationwide)</t>
+(Calculated 24/7/367 Nationwide)</t>
         </is>
       </c>
       <c r="F72" s="5" t="inlineStr">
         <is>
-          <t>kindly provide formula , or is it " initial RRC connection rate X erab assignment success rate"</t>
+          <t>busy hour means auto busy hour or fixed busy hour such as 19:00- 20:00?</t>
         </is>
       </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
-          <t>Per 3GPP TS 38.331 and ETSI standards, Call/Session Setup Success Rate (CSSR) is defined as: CSSR = [RRC Connection Setup Success Rate] x [QoS Flow / NG-C Setup Success Rate] x 100%. Where RRC Setup Success Rate = (Successful RRC Setup Completions / RRC Setup Requests excluding rejections) and QoS Flow Setup Success Rate = (Successful 5G QoS Flow Establishments / QoS Flow Establishment Requests).</t>
+          <t>Confirmed. Busy Hour is defined as Time-Consistent Busy Hour (TCBH) per 3GPP/ITU-T recommendations, determined on a per-cell basis as the continuous 60-minute interval exhibiting the highest combined uplink and downlink traffic volume over a 30-day rolling observation window.</t>
         </is>
       </c>
       <c r="H72" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10047,7 +10010,7 @@
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>Q068</t>
+          <t>Q069</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
@@ -10057,28 +10020,29 @@
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>06_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
+          <t>07_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
         <is>
           <t>3.1 Core Radio KPIs
-(Calculated 24/7/367 Nationwide)</t>
+(Calculated 24/7/368 Nationwide)</t>
         </is>
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>busy hour means auto busy hour or fixed busy hour such as 19:00- 20:00?</t>
+          <t>1. because there is " cell edge DL&amp;UL user speed", is this drive test KPI ? user throughput means  CPE throughput? 
+2. how to define cell edge here?</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Busy Hour is defined as Time-Consistent Busy Hour (TCBH) per 3GPP/ITU-T recommendations, determined on a per-cell basis as the continuous 60-minute interval exhibiting the highest combined uplink and downlink traffic volume over a 30-day rolling observation window.</t>
+          <t>Confirmed. Cell-edge user speed is evaluated at the outer boundary of the designed coverage footprint (nominally RSRP between -95 dBm and -105 dBm). During acceptance, it is verified via stationary drive/walk tests and CPE performance logs. For operational KPI reporting, cell-edge performance is tracked via 5-percentile user throughput metrics extracted from gNodeB OSS performance counters.</t>
         </is>
       </c>
       <c r="H73" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10088,7 +10052,7 @@
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Q069</t>
+          <t>Q070</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
@@ -10096,31 +10060,25 @@
           <t>SLA&amp;KPIs</t>
         </is>
       </c>
-      <c r="D74" s="5" t="inlineStr">
-        <is>
-          <t>07_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
-        </is>
-      </c>
+      <c r="D74" s="5" t="n"/>
       <c r="E74" s="5" t="inlineStr">
         <is>
-          <t>3.1 Core Radio KPIs
-(Calculated 24/7/368 Nationwide)</t>
+          <t>5.7 Radio Frequency (RF) Cluster Optimization</t>
         </is>
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>1. because there is " cell edge DL&amp;UL user speed", is this drive test KPI ? user throughput means  CPE throughput? 
-2. how to define cell edge here?</t>
+          <t>the target of  cluster optimization is only for coverage outdoor target , any target for other KPIs such as throughput ?</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Cell-edge user speed is evaluated at the outer boundary of the designed coverage footprint (nominally RSRP between -95 dBm and -105 dBm). During acceptance, it is verified via stationary drive/walk tests and CPE performance logs. For operational KPI reporting, cell-edge performance is tracked via 5-percentile user throughput metrics extracted from gNodeB OSS performance counters.</t>
+          <t>Confirmed. Cluster optimization acceptance requires meeting both coverage and quality criteria: (1) Coverage: RSRP &gt;= -95 dBm over &gt;= 90% of the designated target populated settlement area; (2) Quality: SINR &gt;= 3 dB over &gt;= 90% of the cluster footprint; (3) Throughput: SSV speed targets verified at near, mid, and edge testing points; (4) Accessibility/Retainability: Cluster-wide CSSR &gt;= 97% and Call Drop Rate (CDR) &lt;= 1.5%.</t>
         </is>
       </c>
       <c r="H74" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10130,7 +10088,7 @@
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>Q070</t>
+          <t>Q071</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
@@ -10138,25 +10096,29 @@
           <t>SLA&amp;KPIs</t>
         </is>
       </c>
-      <c r="D75" s="5" t="n"/>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>05_Appendix_D_Site_Survey_RF_Planning_Civil_Power_Guidelines.pdf</t>
+        </is>
+      </c>
       <c r="E75" s="5" t="inlineStr">
         <is>
-          <t>5.7 Radio Frequency (RF) Cluster Optimization</t>
+          <t>5.. SINGLE SITE VERIFICATION (SSV) &amp; CLUSTER ACCEPTANCE CRITERIA</t>
         </is>
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>the target of  cluster optimization is only for coverage outdoor target , any target for other KPIs such as throughput ?</t>
+          <t>for Near , mid and far location, suggest to based on simulation of typcial site ( antenna height, tilt, power ), and give proper distance of near , mid and far. or use RSRP level at -90, -100, -105</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Cluster optimization acceptance requires meeting both coverage and quality criteria: (1) Coverage: RSRP &gt;= -95 dBm over &gt;= 90% of the designated target populated settlement area; (2) Quality: SINR &gt;= 3 dB over &gt;= 90% of the cluster footprint; (3) Throughput: SSV speed targets verified at near, mid, and edge testing points; (4) Accessibility/Retainability: Cluster-wide CSSR &gt;= 97% and Call Drop Rate (CDR) &lt;= 1.5%.</t>
+          <t>Confirmed. The classification of Near (&lt;500m), Mid (1.0–1.5 km), and Far (&gt;=2.0 km) zones is established based on baseline RF propagation modeling for 30m nominal antenna height, adjusted during physical cluster drive testing and SSV based on local terrain, clutter, and morphology.</t>
         </is>
       </c>
       <c r="H75" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10166,37 +10128,37 @@
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>Q071</t>
+          <t>Q072</t>
         </is>
       </c>
       <c r="C76" s="5" t="inlineStr">
         <is>
-          <t>SLA&amp;KPIs</t>
+          <t>Wireless and Delivery</t>
         </is>
       </c>
       <c r="D76" s="5" t="inlineStr">
         <is>
-          <t>05_Appendix_D_Site_Survey_RF_Planning_Civil_Power_Guidelines.pdf</t>
+          <t>01_RFP_5G_FWA_Master_Tender_Document.pdf</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
         <is>
-          <t>5.. SINGLE SITE VERIFICATION (SSV) &amp; CLUSTER ACCEPTANCE CRITERIA</t>
+          <t>2.1 Spectrum Physics: Band n50 Advantage</t>
         </is>
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>for Near , mid and far location, suggest to based on simulation of typcial site ( antenna height, tilt, power ), and give proper distance of near , mid and far. or use RSRP level at -90, -100, -105</t>
+          <t>From our general understanding, the rules for spectrum allocation are usually uniform nationwide. We would like to know whether TelTech has obtained authorization from the NTC to use 80 MHz of spectrum in areas outside the NCR.</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. The classification of Near (&lt;500m), Mid (1.0–1.5 km), and Far (&gt;=2.0 km) zones is established based on baseline RF propagation modeling for 30m nominal antenna height, adjusted during physical cluster drive testing and SSV based on local terrain, clutter, and morphology.</t>
+          <t>Confirmed. The operational frequency authorization is governed by the National Telecommunications Commission (NTC) framework covering dedicated broadband wireless/private enterprise allocations within 1457.0 – 1518.0 MHz nationwide across the 5,000 candidate barangays. TelTech is finalizing formal commercial coordination with NTC; bidders shall design their RAN solutions for a standard 60 MHz TDD carrier (1457–1517 MHz) with 30 kHz Subcarrier Spacing (SCS).</t>
         </is>
       </c>
       <c r="H76" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10206,7 +10168,7 @@
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Q072</t>
+          <t>Q073</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
@@ -10216,27 +10178,27 @@
       </c>
       <c r="D77" s="5" t="inlineStr">
         <is>
-          <t>01_RFP_5G_FWA_Master_Tender_Document.pdf</t>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
         <is>
-          <t>2.1 Spectrum Physics: Band n50 Advantage</t>
+          <t>SECTION 1: RADIO ACCESS NETWORK (RAN) TECHNICAL SPECIFICATIONS</t>
         </is>
       </c>
       <c r="F77" s="5" t="inlineStr">
         <is>
-          <t>From our general understanding, the rules for spectrum allocation are usually uniform nationwide. We would like to know whether TelTech has obtained authorization from the NTC to use 80 MHz of spectrum in areas outside the NCR.</t>
+          <t>Antennas are generally installed at relatively high positions on towers. Towers have requirements for the antenna's windward area and wind load capacity. Does TelTech have requirements for the antenna's windward area and wind load capacity? Based on the Contractor / Prospective Bidder's experience in delivering macro base stations, it is recommended that the windward area does not exceed 0.8 square meters.</t>
         </is>
       </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. The operational frequency authorization is governed by the National Telecommunications Commission (NTC) framework covering dedicated broadband wireless/private enterprise allocations within 1457.0 – 1518.0 MHz nationwide across the 5,000 candidate barangays. TelTech is finalizing formal commercial coordination with NTC; bidders shall design their RAN solutions for a standard 60 MHz TDD carrier (1457–1517 MHz) with 30 kHz Subcarrier Spacing (SCS).</t>
+          <t>Confirmed. For Class T1–T3 co-location sites, allowable antenna projected windward surface area, EPA (Effective Projected Area), and mounting centerline elevations are governed by each TowerCo's structural design limits and master lease agreements (MLA). Bidders shall submit equipment dimensions and weight specifications. For Class T4 Greenfield Monopoles, the tower structure must be designed to withstand NSCP 2015 wind speeds of up to 270 km/h (Category V typhoon resistance) accommodating 6 RRUs, 1 integrated active antenna (or 3 passive antennas), and up to 1.2 m² total microwave dish surface area.</t>
         </is>
       </c>
       <c r="H77" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10246,37 +10208,33 @@
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>Q073</t>
+          <t>Q074</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
         <is>
-          <t>Wireless and Delivery</t>
+          <t>Warranty</t>
         </is>
       </c>
       <c r="D78" s="5" t="inlineStr">
         <is>
-          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
-        </is>
-      </c>
-      <c r="E78" s="5" t="inlineStr">
-        <is>
-          <t>SECTION 1: RADIO ACCESS NETWORK (RAN) TECHNICAL SPECIFICATIONS</t>
-        </is>
-      </c>
+          <t>01_RFP_5G_FWA_Master_Tender_Document.pdf</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="n"/>
       <c r="F78" s="5" t="inlineStr">
         <is>
-          <t>Antennas are generally installed at relatively high positions on towers. Towers have requirements for the antenna's windward area and wind load capacity. Does TelTech have requirements for the antenna's windward area and wind load capacity? Based on the Contractor / Prospective Bidder's experience in delivering macro base stations, it is recommended that the windward area does not exceed 0.8 square meters.</t>
+          <t>Please confirm that the mandatory base Defect Liability Period (DLP / Hardware Warranty) for network equipment remains 24 months (2 years) from the date of PAC issuance per site/phase. Furthermore, please clarify whether the Extended Warranty and Spare Parts Management Service (SPMS) for Years 3–5 (as well as Years 6–10 for TCO calculation) should be quoted as separate, optional line items per Phase in the Appendix B Commercial BoQ.</t>
         </is>
       </c>
       <c r="G78" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. For Class T1–T3 co-location sites, allowable antenna projected windward surface area, EPA (Effective Projected Area), and mounting centerline elevations are governed by each TowerCo's structural design limits and master lease agreements (MLA). Bidders shall submit equipment dimensions and weight specifications. For Class T4 Greenfield Monopoles, the tower structure must be designed to withstand NSCP 2015 wind speeds of up to 270 km/h (Category V typhoon resistance) accommodating 6 RRUs, 1 integrated active antenna (or 3 passive antennas), and up to 1.2 m² total microwave dish surface area.</t>
+          <t>Confirmed. The mandatory base Defect Liability Period (DLP / Hardware Warranty) for all active network equipment (Lots 1, 2, 3, 6) is confirmed as twenty-four (24) months (2 years) commencing from the issuance of the Provisional Acceptance Certificate (PAC).</t>
         </is>
       </c>
       <c r="H78" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10286,12 +10244,12 @@
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>Q074</t>
+          <t>Q075</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Warranty</t>
+          <t>Training</t>
         </is>
       </c>
       <c r="D79" s="5" t="inlineStr">
@@ -10302,17 +10260,17 @@
       <c r="E79" s="5" t="n"/>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>Please confirm that the mandatory base Defect Liability Period (DLP / Hardware Warranty) for network equipment remains 24 months (2 years) from the date of PAC issuance per site/phase. Furthermore, please clarify whether the Extended Warranty and Spare Parts Management Service (SPMS) for Years 3–5 (as well as Years 6–10 for TCO calculation) should be quoted as separate, optional line items per Phase in the Appendix B Commercial BoQ.</t>
+          <t>Please clarify whether formal OEM technical training and certification programs (covering 5G SA Core, Band n50 RAN, BSS/OSS, and FMS) are required for TelTech’s engineering and O&amp;M personnel. If required, kindly provide the estimated number of trainees, preferred training location (e.g., local classroom in Manila/Clark vs. OEM headquarters), and confirm if this should be quoted as a dedicated line item in the Commercial BoQ.</t>
         </is>
       </c>
       <c r="G79" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. The mandatory base Defect Liability Period (DLP / Hardware Warranty) for all active network equipment (Lots 1, 2, 3, 6) is confirmed as twenty-four (24) months (2 years) commencing from the issuance of the Provisional Acceptance Certificate (PAC).</t>
+          <t>Confirmed. Formal OEM technical training and certification programs covering 5G SA Core administration, Band n50 RAN RF optimization, OSS/BSS operations, and field maintenance are mandatory deliverables under Lot 5 / Services, dimensioned for at least 20 TelTech engineering personnel.</t>
         </is>
       </c>
       <c r="H79" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10322,33 +10280,33 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Q075</t>
+          <t>Q076</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Training</t>
+          <t>Commercial Template</t>
         </is>
       </c>
       <c r="D80" s="5" t="inlineStr">
         <is>
-          <t>01_RFP_5G_FWA_Master_Tender_Document.pdf</t>
+          <t>Portal "3. Commercial BoQ &amp; Financing Lots 1-7"</t>
         </is>
       </c>
       <c r="E80" s="5" t="n"/>
       <c r="F80" s="5" t="inlineStr">
         <is>
-          <t>Please clarify whether formal OEM technical training and certification programs (covering 5G SA Core, Band n50 RAN, BSS/OSS, and FMS) are required for TelTech’s engineering and O&amp;M personnel. If required, kindly provide the estimated number of trainees, preferred training location (e.g., local classroom in Manila/Clark vs. OEM headquarters), and confirm if this should be quoted as a dedicated line item in the Commercial BoQ.</t>
+          <t>For the Years 6–10 Cumulative OPEX (Managed Services and Extended Maintenance) in the 10-Year TCO evaluation, please confirm if bidders are permitted to include an annual Consumer Price Index (CPI) inflation indexation and FX adjustment clause to account for long-term macroeconomic fluctuations.</t>
         </is>
       </c>
       <c r="G80" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Formal OEM technical training and certification programs covering 5G SA Core administration, Band n50 RAN RF optimization, OSS/BSS operations, and field maintenance are mandatory deliverables under Lot 5 / Services, dimensioned for at least 20 TelTech engineering personnel.</t>
+          <t>Confirmed. Bidders are permitted to quote Years 6–10 Managed Services and extended software maintenance as an optional annual escalation or fixed rate in the 10-Year Total Cost of Ownership (TCO) financial model.</t>
         </is>
       </c>
       <c r="H80" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10358,7 +10316,7 @@
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>Q076</t>
+          <t>Q077</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
@@ -10374,17 +10332,17 @@
       <c r="E81" s="5" t="n"/>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>For the Years 6–10 Cumulative OPEX (Managed Services and Extended Maintenance) in the 10-Year TCO evaluation, please confirm if bidders are permitted to include an annual Consumer Price Index (CPI) inflation indexation and FX adjustment clause to account for long-term macroeconomic fluctuations.</t>
+          <t>Are all unit prices in Commercial BOQ to be quoted in VAT Ex (Value Added Tax Exclusive)?</t>
         </is>
       </c>
       <c r="G81" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Bidders are permitted to quote Years 6–10 Managed Services and extended software maintenance as an optional annual escalation or fixed rate in the 10-Year Total Cost of Ownership (TCO) financial model.</t>
+          <t>Confirmed. All unit rates and total prices in the Commercial BoQ must be quoted exclusive of 12% Philippine Value Added Tax (VAT-Exclusive). VAT will be added as a separate line item on billing invoices in accordance with Bureau of Internal Revenue (BIR) regulations.</t>
         </is>
       </c>
       <c r="H81" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10394,61 +10352,25 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>Q077</t>
+          <t>Q078</t>
         </is>
       </c>
       <c r="C82" s="5" t="inlineStr">
         <is>
-          <t>Commercial Template</t>
+          <t>Power system and delivery</t>
         </is>
       </c>
       <c r="D82" s="5" t="inlineStr">
         <is>
-          <t>Portal "3. Commercial BoQ &amp; Financing Lots 1-7"</t>
-        </is>
-      </c>
-      <c r="E82" s="5" t="n"/>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="E82" s="5" t="inlineStr">
+        <is>
+          <t>SECTION 2: POWER SYSTEMS &amp; PASSIVE SITE INFRASTRUCTURE</t>
+        </is>
+      </c>
       <c r="F82" s="5" t="inlineStr">
-        <is>
-          <t>Are all unit prices in Commercial BOQ to be quoted in VAT Ex (Value Added Tax Exclusive)?</t>
-        </is>
-      </c>
-      <c r="G82" s="5" t="inlineStr">
-        <is>
-          <t>Confirmed. All unit rates and total prices in the Commercial BoQ must be quoted exclusive of 12% Philippine Value Added Tax (VAT-Exclusive). VAT will be added as a separate line item on billing invoices in accordance with Bureau of Internal Revenue (BIR) regulations.</t>
-        </is>
-      </c>
-      <c r="H82" s="12" t="inlineStr">
-        <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="4" t="n">
-        <v>79</v>
-      </c>
-      <c r="B83" s="4" t="inlineStr">
-        <is>
-          <t>Q078</t>
-        </is>
-      </c>
-      <c r="C83" s="5" t="inlineStr">
-        <is>
-          <t>Power system and delivery</t>
-        </is>
-      </c>
-      <c r="D83" s="5" t="inlineStr">
-        <is>
-          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
-        </is>
-      </c>
-      <c r="E83" s="5" t="inlineStr">
-        <is>
-          <t>SECTION 2: POWER SYSTEMS &amp; PASSIVE SITE INFRASTRUCTURE</t>
-        </is>
-      </c>
-      <c r="F83" s="5" t="inlineStr">
         <is>
           <t>1. Does it requires 2 Rectifier System per site or 2N Configuration? For ex: 1000 sites will be 2000 rectifier?
 2. Do they need monitoring software to cover all sites??
@@ -10456,14 +10378,54 @@
 4. If outdoor installation, does all the 5000 sites is same set up?</t>
         </is>
       </c>
+      <c r="G82" s="5" t="inlineStr">
+        <is>
+          <t>Confirmed. (1) Each site requires one (1) high-efficiency outdoor-rated rectifier system with N+1 modular rectifier redundancy (e.g. 3x 50A modules providing 100A N+1 output). For ground-based Greenfield sites, an outdoor cabinet-housed rectifier is utilized; for tower co-location sites with limited footprint, blade/pole-mounted outdoor rectifiers are preferred. (2) Remote power monitoring software/controller with SNMPv3 / Modbus-TCP telemetry reporting into the centralized OSS is mandatory.</t>
+        </is>
+      </c>
+      <c r="H82" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>Q079</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>OSS &amp; BSS Integration</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+        </is>
+      </c>
+      <c r="E83" s="5" t="inlineStr">
+        <is>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>In the FM app, is it acceptable that the navigation function redirects to an external app, such as Google Maps?</t>
+        </is>
+      </c>
       <c r="G83" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. (1) Each site requires one (1) high-efficiency outdoor-rated rectifier system with N+1 modular rectifier redundancy (e.g. 3x 50A modules providing 100A N+1 output). For ground-based Greenfield sites, an outdoor cabinet-housed rectifier is utilized; for tower co-location sites with limited footprint, blade/pole-mounted outdoor rectifiers are preferred. (2) Remote power monitoring software/controller with SNMPv3 / Modbus-TCP telemetry reporting into the centralized OSS is mandatory.</t>
+          <t>Confirmed. In the Field Force Management (FMS) mobile application, deep-linking or redirecting to external standard navigation applications (e.g., Google Maps, Waze) for route guidance to site/subscriber coordinates is fully acceptable.</t>
         </is>
       </c>
       <c r="H83" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10473,7 +10435,7 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>Q079</t>
+          <t>Q080</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr">
@@ -10493,17 +10455,17 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>In the FM app, is it acceptable that the navigation function redirects to an external app, such as Google Maps?</t>
+          <t>In the FM app, is the e-sign used only to collect users' handwritten signatures? If the electronic signature is used for strong authentication, a third-party SDK needs to be integrated. Currently, this is not supported.</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. In the Field Force Management (FMS) mobile application, deep-linking or redirecting to external standard navigation applications (e.g., Google Maps, Waze) for route guidance to site/subscriber coordinates is fully acceptable.</t>
+          <t>Confirmed. Capturing the subscriber's handwritten signature on the mobile touchscreen interface at completion of installation/service is acceptable for job acceptance. Third-party digital signature authority (CA/PKI) integration is not mandatory for standard residential installation sign-offs.</t>
         </is>
       </c>
       <c r="H84" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10513,7 +10475,7 @@
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>Q080</t>
+          <t>Q081</t>
         </is>
       </c>
       <c r="C85" s="5" t="inlineStr">
@@ -10533,17 +10495,17 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>In the FM app, is the e-sign used only to collect users' handwritten signatures? If the electronic signature is used for strong authentication, a third-party SDK needs to be integrated. Currently, this is not supported.</t>
+          <t>For RF signal verification, it is recommended to use professional software such as Cellular-Z to obtain more accurate and professional policy data.</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Capturing the subscriber's handwritten signature on the mobile touchscreen interface at completion of installation/service is acceptable for job acceptance. Third-party digital signature authority (CA/PKI) integration is not mandatory for standard residential installation sign-offs.</t>
+          <t>Confirmed. Any industry-standard, calibrated RF measurement application or handheld scanner (e.g., Cellular-Z, G-NetTrack Pro, Nemo Handy, or OEM-native diagnostic tool) is acceptable for post-installation RF verification, provided it logs accurate RSRP, RSRQ, SINR, and Cell ID parameters into the installation completion report.</t>
         </is>
       </c>
       <c r="H85" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10553,7 +10515,7 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Q081</t>
+          <t>Q082</t>
         </is>
       </c>
       <c r="C86" s="5" t="inlineStr">
@@ -10573,17 +10535,17 @@
       </c>
       <c r="F86" s="5" t="inlineStr">
         <is>
-          <t>For RF signal verification, it is recommended to use professional software such as Cellular-Z to obtain more accurate and professional policy data.</t>
+          <t>Does the installation order involve service provisioning?</t>
         </is>
       </c>
       <c r="G86" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Any industry-standard, calibrated RF measurement application or handheld scanner (e.g., Cellular-Z, G-NetTrack Pro, Nemo Handy, or OEM-native diagnostic tool) is acceptable for post-installation RF verification, provided it logs accurate RSRP, RSRQ, SINR, and Cell ID parameters into the installation completion report.</t>
+          <t>Confirmed. Installation work orders executed by field technicians must trigger automated service provisioning in the BSS/OSS upon successful on-site RF validation and customer digital sign-off, regardless of whether installation is performed by OEM managed service teams or outsourced subcontractors.</t>
         </is>
       </c>
       <c r="H86" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10593,12 +10555,12 @@
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>Q082</t>
+          <t>Q083</t>
         </is>
       </c>
       <c r="C87" s="5" t="inlineStr">
         <is>
-          <t>OSS &amp; BSS Integration</t>
+          <t>Wireless and Delivery</t>
         </is>
       </c>
       <c r="D87" s="5" t="inlineStr">
@@ -10608,22 +10570,22 @@
       </c>
       <c r="E87" s="5" t="inlineStr">
         <is>
-          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+          <t>SECTION 5: RF PLANNING, SITE SURVEY &amp; CLUSTER OPTIMIZATION</t>
         </is>
       </c>
       <c r="F87" s="5" t="inlineStr">
         <is>
-          <t>Does the installation order involve service provisioning?</t>
+          <t>The areas covered by the issued tender documents are mostly suburban or rural regions, which do not have the capability to use 5-meter HD maps. Should we switch to using 2D maps entirely for simulation planning?</t>
         </is>
       </c>
       <c r="G87" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Installation work orders executed by field technicians must trigger automated service provisioning in the BSS/OSS upon successful on-site RF validation and customer digital sign-off, regardless of whether installation is performed by OEM managed service teams or outsourced subcontractors.</t>
+          <t>Confirmed. For rural and remote Class T4 candidate barangays where 5-meter HD clutter maps are commercially unavailable, bidders are permitted to utilize standard 20m/25m digital elevation and land-use clutter datasets supplemented by satellite imagery and digital surface models (DSM) for macro-cellular nominal RF planning and cluster simulation.</t>
         </is>
       </c>
       <c r="H87" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10633,7 +10595,7 @@
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Q083</t>
+          <t>Q084</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr">
@@ -10648,22 +10610,22 @@
       </c>
       <c r="E88" s="5" t="inlineStr">
         <is>
-          <t>SECTION 5: RF PLANNING, SITE SURVEY &amp; CLUSTER OPTIMIZATION</t>
+          <t>SECTION 1: RADIO ACCESS NETWORK (RAN) TECHNICAL SPECIFICATIONS</t>
         </is>
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>The areas covered by the issued tender documents are mostly suburban or rural regions, which do not have the capability to use 5-meter HD maps. Should we switch to using 2D maps entirely for simulation planning?</t>
+          <t>According to the current site capability planning, the maximum average traffic of a single site does not exceed 1 Gbit/s. Therefore, the site does not need to support 2 x 10GE + 2 x 25GE interfaces. It is recommended that only the maximum capability be reserved, that is, 2 x 25GE interfaces.</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. For rural and remote Class T4 candidate barangays where 5-meter HD clutter maps are commercially unavailable, bidders are permitted to utilize standard 20m/25m digital elevation and land-use clutter datasets supplemented by satellite imagery and digital surface models (DSM) for macro-cellular nominal RF planning and cluster simulation.</t>
+          <t>Confirmed. An initial backhaul transport capacity of 1 Gbit/s per gNodeB site is acceptable for Day 1 traffic dimensioning. However, backhaul transmission interfaces (both optical transceivers and microwave links) must support hardware upgradeability to 10 Gbit/s via standard SFP+ interfaces to accommodate future multi-carrier expansion and subscriber growth.</t>
         </is>
       </c>
       <c r="H88" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10673,7 +10635,7 @@
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Q084</t>
+          <t>Q085</t>
         </is>
       </c>
       <c r="C89" s="5" t="inlineStr">
@@ -10683,27 +10645,27 @@
       </c>
       <c r="D89" s="5" t="inlineStr">
         <is>
-          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+          <t>07_RFP_5G_FWA_Candidate_Site_List_and_Rollout_Schedule.xlsx</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
         <is>
-          <t>SECTION 1: RADIO ACCESS NETWORK (RAN) TECHNICAL SPECIFICATIONS</t>
+          <t>Phase 1 (First 1,000 Sites)</t>
         </is>
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>According to the current site capability planning, the maximum average traffic of a single site does not exceed 1 Gbit/s. Therefore, the site does not need to support 2 x 10GE + 2 x 25GE interfaces. It is recommended that only the maximum capability be reserved, that is, 2 x 25GE interfaces.</t>
+          <t>Considering there are 897 co-sited base stations, is it advisable to use cabinet BBUs instead of blade BBUs?</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. An initial backhaul transport capacity of 1 Gbit/s per gNodeB site is acceptable for Day 1 traffic dimensioning. However, backhaul transmission interfaces (both optical transceivers and microwave links) must support hardware upgradeability to 10 Gbit/s via standard SFP+ interfaces to accommodate future multi-carrier expansion and subscriber growth.</t>
+          <t>Confirmed. Blade BBUs (outdoor zero-footprint pole/wall-mounted baseband units) are strongly preferred across all 897 co-location sites to eliminate ground footprint leasing penalties, reduce shelter space requirements, and facilitate rapid deployment. Compact outdoor cabinet BBUs are acceptable only where indoor/shelter space is pre-contracted or where blade mounting is structurally restricted by the TowerCo.</t>
         </is>
       </c>
       <c r="H89" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10713,37 +10675,37 @@
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>Q085</t>
+          <t>Q086</t>
         </is>
       </c>
       <c r="C90" s="5" t="inlineStr">
         <is>
-          <t>Wireless and Delivery</t>
+          <t>OSS &amp; BSS Integration</t>
         </is>
       </c>
       <c r="D90" s="5" t="inlineStr">
         <is>
-          <t>07_RFP_5G_FWA_Candidate_Site_List_and_Rollout_Schedule.xlsx</t>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 (First 1,000 Sites)</t>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
         </is>
       </c>
       <c r="F90" s="5" t="inlineStr">
         <is>
-          <t>Considering there are 897 co-sited base stations, is it advisable to use cabinet BBUs instead of blade BBUs?</t>
+          <t>Regarding the CPE recovery rate (&gt;= 70%), the Contractor / Prospective Bidder's 2-year warranty period allows for free replacement if any issues arise. Is such a service acceptable? The CPE recovery rate cannot be controlled.</t>
         </is>
       </c>
       <c r="G90" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. Blade BBUs (outdoor zero-footprint pole/wall-mounted baseband units) are strongly preferred across all 897 co-location sites to eliminate ground footprint leasing penalties, reduce shelter space requirements, and facilitate rapid deployment. Compact outdoor cabinet BBUs are acceptable only where indoor/shelter space is pre-contracted or where blade mounting is structurally restricted by the TowerCo.</t>
+          <t>Accepted and clarified. The &gt;= 70% CPE Recovery Rate defined in the RFP applies strictly to churned subscriber recovery and reverse logistics (retrieving TelTech-owned CPE hardware from canceled subscriber premises), not OEM warranty returns. For defective CPE units under the 24-month DLP, OEM free replacement applies for manufacturing defects. Hardware damage resulting from proven subscriber misuse, vandalism, or force majeure shall be handled via spare parts replacement at the contracted master rate card.</t>
         </is>
       </c>
       <c r="H90" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10753,37 +10715,39 @@
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>Q086</t>
+          <t>Q087</t>
         </is>
       </c>
       <c r="C91" s="5" t="inlineStr">
         <is>
-          <t>OSS &amp; BSS Integration</t>
+          <t>SLA&amp;KPIs</t>
         </is>
       </c>
       <c r="D91" s="5" t="inlineStr">
         <is>
-          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+          <t>04_Appendix_C_SLAs_KPIs_Liquidated_Damages.pdf</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
         <is>
-          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+          <t>3. RADIO ACCESS NETWORK (RAN) OPERATIONAL KPIS &amp; SERVICE CREDITS</t>
         </is>
       </c>
       <c r="F91" s="5" t="inlineStr">
         <is>
-          <t>Regarding the CPE recovery rate (&gt;= 70%), the Contractor / Prospective Bidder's 2-year warranty period allows for free replacement if any issues arise. Is such a service acceptable? The CPE recovery rate cannot be controlled.</t>
+          <t>Regarding the MTTR、NAV、SPMS SLA,
+Due to the lack of live network conditions and other inputs, it is impossible to assess the achievability of KPIs:
+SLA is recommended to be finalized based on the actual values observed during the 6 months following acceptance and commissioning.</t>
         </is>
       </c>
       <c r="G91" s="5" t="inlineStr">
         <is>
-          <t>Accepted and clarified. The &gt;= 70% CPE Recovery Rate defined in the RFP applies strictly to churned subscriber recovery and reverse logistics (retrieving TelTech-owned CPE hardware from canceled subscriber premises), not OEM warranty returns. For defective CPE units under the 24-month DLP, OEM free replacement applies for manufacturing defects. Hardware damage resulting from proven subscriber misuse, vandalism, or force majeure shall be handled via spare parts replacement at the contracted master rate card.</t>
+          <t>Confirmed. The SLA targets defined in Appendix C represent standard telecommunications industry benchmarks for enterprise 5G fixed wireless networks. For Phase 1, TelTech grants a 90-day post-PAC stabilization period for each rollout cluster, during which service credits / SLA penalties for network availability (NAV) and MTTR are waived while operational baselines and spares logistics are stabilized.</t>
         </is>
       </c>
       <c r="H91" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10793,39 +10757,37 @@
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Q087</t>
+          <t>Q088</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr">
         <is>
-          <t>SLA&amp;KPIs</t>
+          <t>SLI</t>
         </is>
       </c>
       <c r="D92" s="5" t="inlineStr">
         <is>
-          <t>04_Appendix_C_SLAs_KPIs_Liquidated_Damages.pdf</t>
+          <t>01_RFP_5G_FWA_Master_Tender_Document</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
         <is>
-          <t>3. RADIO ACCESS NETWORK (RAN) OPERATIONAL KPIS &amp; SERVICE CREDITS</t>
+          <t>LOT</t>
         </is>
       </c>
       <c r="F92" s="5" t="inlineStr">
         <is>
-          <t>Regarding the MTTR、NAV、SPMS SLA,
-Due to the lack of live network conditions and other inputs, it is impossible to assess the achievability of KPIs:
-SLA is recommended to be finalized based on the actual values observed during the 6 months following acceptance and commissioning.</t>
+          <t>What is installation? In which scenarios is installation required? Is the Contractor / Prospective Bidder responsible for the installation? How to calculate the New Installation Dispatch Lead Time?</t>
         </is>
       </c>
       <c r="G92" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. The SLA targets defined in Appendix C represent standard telecommunications industry benchmarks for enterprise 5G fixed wireless networks. For Phase 1, TelTech grants a 90-day post-PAC stabilization period for each rollout cluster, during which service credits / SLA penalties for network availability (NAV) and MTTR are waived while operational baselines and spares logistics are stabilized.</t>
+          <t>Installation refers to Customer Premises Equipment (CPE) installation and commissioning at subscriber premises, encompassing RF site survey, optimal wall/pole/roof mounting, outdoor Cat6 cabling up to 30m, PoE injector, Wi-Fi router setup, zero-touch provisioning via Field Force App, and speed test sign-off. When Lot 5 (Turnkey Managed Services) is awarded, the bidder is responsible for installation; otherwise, TelTech's accredited installation contractors execute the work.</t>
         </is>
       </c>
       <c r="H92" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10835,7 +10797,7 @@
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>Q088</t>
+          <t>Q089</t>
         </is>
       </c>
       <c r="C93" s="5" t="inlineStr">
@@ -10855,17 +10817,17 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>What is installation? In which scenarios is installation required? Is the Contractor / Prospective Bidder responsible for the installation? How to calculate the New Installation Dispatch Lead Time?</t>
+          <t>How is the First-Time-Right (FTR) Installation Rate calculated?</t>
         </is>
       </c>
       <c r="G93" s="5" t="inlineStr">
         <is>
-          <t>Installation refers to Customer Premises Equipment (CPE) installation and commissioning at subscriber premises, encompassing RF site survey, optimal wall/pole/roof mounting, outdoor Cat6 cabling up to 30m, PoE injector, Wi-Fi router setup, zero-touch provisioning via Field Force App, and speed test sign-off. When Lot 5 (Turnkey Managed Services) is awarded, the bidder is responsible for installation; otherwise, TelTech's accredited installation contractors execute the work.</t>
+          <t>The First-Time-Right (FTR) Installation Rate is calculated on a monthly rolling basis using the standard formula: FTR Rate = [(Total Completed Installations - Repeat Truck Rolls within 14 Days) / Total Completed Installations] x 100%. Any physical revisit required within 14 calendar days due to hardware failure, cabling defect, antenna misalignment, or provisioning failure counts against FTR.</t>
         </is>
       </c>
       <c r="H93" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10875,7 +10837,7 @@
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>Q089</t>
+          <t>Q090</t>
         </is>
       </c>
       <c r="C94" s="5" t="inlineStr">
@@ -10895,17 +10857,17 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>How is the First-Time-Right (FTR) Installation Rate calculated?</t>
+          <t>Please provide the procedures for CPE distribution, recovery, and maintenance.</t>
         </is>
       </c>
       <c r="G94" s="5" t="inlineStr">
         <is>
-          <t>The First-Time-Right (FTR) Installation Rate is calculated on a monthly rolling basis using the standard formula: FTR Rate = [(Total Completed Installations - Repeat Truck Rolls within 14 Days) / Total Completed Installations] x 100%. Any physical revisit required within 14 calendar days due to hardware failure, cabling defect, antenna misalignment, or provisioning failure counts against FTR.</t>
+          <t>TelTech's standard CPE lifecycle procedure operates as follows: (1) Distribution/Provisioning: Bulk CPE shipments arrive at TelTech's central staging warehouse, undergo barcode/IMEI ingestion into BSS/OSS asset tracking, and are dispatched to regional forward staging hubs. Installers scan serial numbers on-site and initiate automated zero-touch provisioning (TR-069 / USP via ACS). (2) Maintenance/RMA: Faulty units identified during subscriber trouble tickets are swapped by field technicians with buffer units from regional staging stock. Defective units are returned for RMA batching under the 24-month DLP warranty. (3) Recovery/Reverse Logistics: Upon subscriber service termination, BSS triggers a CPE Retrieval Work Order in the Field Force App. Recovered units undergo factory reset, testing, refurbishment, repackaging, and re-entry into active inventory.</t>
         </is>
       </c>
       <c r="H94" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10915,37 +10877,37 @@
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>Q090</t>
+          <t>Q091</t>
         </is>
       </c>
       <c r="C95" s="5" t="inlineStr">
         <is>
-          <t>SLI</t>
+          <t>SLA&amp;KPIs</t>
         </is>
       </c>
       <c r="D95" s="5" t="inlineStr">
         <is>
-          <t>01_RFP_5G_FWA_Master_Tender_Document</t>
+          <t>04_Appendix_C_SLAs_KPIs_Liquidated_Damages.pdf</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
         <is>
-          <t>LOT</t>
+          <t>3. RADIO ACCESS NETWORK (RAN) OPERATIONAL KPIS &amp; SERVICE CREDITS</t>
         </is>
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>Please provide the procedures for CPE distribution, recovery, and maintenance.</t>
+          <t>Does NBD in SPMS mean sending to the Contractor / Prospective Bidder's regional spare parts warehouse?</t>
         </is>
       </c>
       <c r="G95" s="5" t="inlineStr">
         <is>
-          <t>TelTech's standard CPE lifecycle procedure operates as follows: (1) Distribution/Provisioning: Bulk CPE shipments arrive at TelTech's central staging warehouse, undergo barcode/IMEI ingestion into BSS/OSS asset tracking, and are dispatched to regional forward staging hubs. Installers scan serial numbers on-site and initiate automated zero-touch provisioning (TR-069 / USP via ACS). (2) Maintenance/RMA: Faulty units identified during subscriber trouble tickets are swapped by field technicians with buffer units from regional staging stock. Defective units are returned for RMA batching under the 24-month DLP warranty. (3) Recovery/Reverse Logistics: Upon subscriber service termination, BSS triggers a CPE Retrieval Work Order in the Field Force App. Recovered units undergo factory reset, testing, refurbishment, repackaging, and re-entry into active inventory.</t>
+          <t>NBD (Next Business Day) replacement under the Spare Parts Management Service (SPMS) requires the replacement spare part to be delivered to the designated regional forward logistics hub / TelTech regional maintenance center within the next business day (Monday through Saturday, cut-off time 15:00) following RMA dispatch notification.</t>
         </is>
       </c>
       <c r="H95" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10955,37 +10917,37 @@
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Q091</t>
+          <t>Q092</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr">
         <is>
-          <t>SLA&amp;KPIs</t>
+          <t>OSS &amp; BSS Integration</t>
         </is>
       </c>
       <c r="D96" s="5" t="inlineStr">
         <is>
-          <t>04_Appendix_C_SLAs_KPIs_Liquidated_Damages.pdf</t>
+          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
         <is>
-          <t>3. RADIO ACCESS NETWORK (RAN) OPERATIONAL KPIS &amp; SERVICE CREDITS</t>
+          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
         </is>
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>Does NBD in SPMS mean sending to the Contractor / Prospective Bidder's regional spare parts warehouse?</t>
+          <t>Can the standalone OSS/BSS software scope be decoupled from  the following indicators: New Installation Dispatch Lead Time, First-Time-Right (FTR) Installation Rate, and Churned CPE Hardware Recovery Rate.</t>
         </is>
       </c>
       <c r="G96" s="5" t="inlineStr">
         <is>
-          <t>NBD (Next Business Day) replacement under the Spare Parts Management Service (SPMS) requires the replacement spare part to be delivered to the designated regional forward logistics hub / TelTech regional maintenance center within the next business day (Monday through Saturday, cut-off time 15:00) following RMA dispatch notification.</t>
+          <t>Accepted and clarified. For standalone OSS/BSS software delivery (Lot 4), SLA commitments apply to software availability, transaction processing latency, and API throughput (e.g. system uptime &gt;= 99.95%, work order dispatch generation &lt; 5 seconds). Operational field performance indicators such as New Installation Dispatch Lead Time, First-Time-Right (FTR) Installation Rate, and Churned CPE Recovery Rate apply strictly to the Managed Services &amp; Field Operations scope (Lot 5 / Appendix E) when awarded to the managed service provider.</t>
         </is>
       </c>
       <c r="H96" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -10995,37 +10957,38 @@
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>Q092</t>
+          <t>Q093</t>
         </is>
       </c>
       <c r="C97" s="5" t="inlineStr">
         <is>
-          <t>OSS &amp; BSS Integration</t>
+          <t>Site, civil work, and managed services</t>
         </is>
       </c>
       <c r="D97" s="5" t="inlineStr">
         <is>
-          <t>02_Appendix_A_Technical_Specifications_Compliance_Matrix.xlsx</t>
+          <t>APPENDIX E: SERVICES STATEMENT OF WORK &amp; MASTER RATE CARD</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
         <is>
-          <t>SECTION 4: CONVERGED DIGITAL OSS/BSS &amp; FIELD FORCE AUTOMATION</t>
+          <t>4. MASTER SERVICES PRICING SCHEDULE &amp; COMMERCIAL RATE CARD</t>
         </is>
       </c>
       <c r="F97" s="5" t="inlineStr">
         <is>
-          <t>Can the standalone OSS/BSS software scope be decoupled from  the following indicators: New Installation Dispatch Lead Time, First-Time-Right (FTR) Installation Rate, and Churned CPE Hardware Recovery Rate.</t>
+          <t>1. Please suggest on which scenario we need to do tower retrofitting works, since towerco tower is belong to towerco to do retrofitting.
+2. Tower retrofitting need to have retrofitting design first, and this scope are based on each site situation, case by case, Please suggest how to quote this item.</t>
         </is>
       </c>
       <c r="G97" s="5" t="inlineStr">
         <is>
-          <t>Accepted and clarified. For standalone OSS/BSS software delivery (Lot 4), SLA commitments apply to software availability, transaction processing latency, and API throughput (e.g. system uptime &gt;= 99.95%, work order dispatch generation &lt; 5 seconds). Operational field performance indicators such as New Installation Dispatch Lead Time, First-Time-Right (FTR) Installation Rate, and Churned CPE Recovery Rate apply strictly to the Managed Services &amp; Field Operations scope (Lot 5 / Appendix E) when awarded to the managed service provider.</t>
+          <t>Confirmed. For Class T1–T3 co-location sites, tower structural strengthening is primary responsibility of the respective TowerCo under master co-location arrangements. However, to mitigate potential TowerCo lead time delays, bidders shall provide unit rate pricing in the Appendix E Master Rate Card for structural surveys, structural integrity assessments, engineering design, and structural reinforcement fabrication/installation in the event TelTech elects to self-execute retrofitting.</t>
         </is>
       </c>
       <c r="H97" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -11035,38 +10998,39 @@
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Q093</t>
+          <t>Q094</t>
         </is>
       </c>
       <c r="C98" s="5" t="inlineStr">
         <is>
-          <t>Site, civil work, and managed services</t>
+          <t>SLA&amp;KPIs</t>
         </is>
       </c>
       <c r="D98" s="5" t="inlineStr">
         <is>
-          <t>APPENDIX E: SERVICES STATEMENT OF WORK &amp; MASTER RATE CARD</t>
+          <t>05_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
         <is>
-          <t>4. MASTER SERVICES PRICING SCHEDULE &amp; COMMERCIAL RATE CARD</t>
+          <t>3.1 Core Radio KPIs
+(Calculated 24/7/366 Nationwide)</t>
         </is>
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>1. Please suggest on which scenario we need to do tower retrofitting works, since towerco tower is belong to towerco to do retrofitting.
-2. Tower retrofitting need to have retrofitting design first, and this scope are based on each site situation, case by case, Please suggest how to quote this item.</t>
+          <t>Suggest CSSR target 97%, minimum threshold 96; based on huawei global FWA network experience , RRC setup success rate 99% , and qos 98.5%；
+The CSSR further improvement is constrainted from terminal compatibility issues, the extent of network coverage, and transmission loss in indoor CPE.</t>
         </is>
       </c>
       <c r="G98" s="5" t="inlineStr">
         <is>
-          <t>Confirmed. For Class T1–T3 co-location sites, tower structural strengthening is primary responsibility of the respective TowerCo under master co-location arrangements. However, to mitigate potential TowerCo lead time delays, bidders shall provide unit rate pricing in the Appendix E Master Rate Card for structural surveys, structural integrity assessments, engineering design, and structural reinforcement fabrication/installation in the event TelTech elects to self-execute retrofitting.</t>
+          <t>Accepted. TelTech officially updates the nationwide Call/Session Setup Success Rate (CSSR) operational KPI as follows: Target Standard: 97.0% (revised from 99.0%); Minimum Threshold: 96.0% (revised from 97.5%). This adjustment accounts for real-world FWA CPE propagation environments while maintaining premium carrier-grade service reliability.</t>
         </is>
       </c>
       <c r="H98" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -11076,7 +11040,7 @@
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>Q094</t>
+          <t>Q095</t>
         </is>
       </c>
       <c r="C99" s="5" t="inlineStr">
@@ -11097,18 +11061,18 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>Suggest CSSR target 97%, minimum threshold 96; based on huawei global FWA network experience , RRC setup success rate 99% , and qos 98.5%；
-The CSSR further improvement is constrainted from terminal compatibility issues, the extent of network coverage, and transmission loss in indoor CPE.</t>
+          <t>Suggest target 1.5%， maximum 2%；
+The same reason that KPI CDR further improvement is constrainted from terminal compatibility issues, the extent of network coverage, and transmission loss in indoor CPE.</t>
         </is>
       </c>
       <c r="G99" s="5" t="inlineStr">
         <is>
-          <t>Accepted. TelTech officially updates the nationwide Call/Session Setup Success Rate (CSSR) operational KPI as follows: Target Standard: 97.0% (revised from 99.0%); Minimum Threshold: 96.0% (revised from 97.5%). This adjustment accounts for real-world FWA CPE propagation environments while maintaining premium carrier-grade service reliability.</t>
+          <t>Accepted. TelTech officially updates the nationwide Call Drop Rate (CDR) operational KPI as follows: Target Standard: &lt;= 1.5% (revised from &lt;= 0.5%); Maximum Threshold: &lt;= 2.0% (revised from &lt;= 1.0%). Service Credits apply only if monthly nationwide aggregate CDR exceeds 2.0%.</t>
         </is>
       </c>
       <c r="H99" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -11118,7 +11082,7 @@
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Q095</t>
+          <t>Q096</t>
         </is>
       </c>
       <c r="C100" s="5" t="inlineStr">
@@ -11139,18 +11103,17 @@
       </c>
       <c r="F100" s="5" t="inlineStr">
         <is>
-          <t>Suggest target 1.5%， maximum 2%；
-The same reason that KPI CDR further improvement is constrainted from terminal compatibility issues, the extent of network coverage, and transmission loss in indoor CPE.</t>
+          <t>suggest to remove both KPIs , this is more factored by user behavior and user distribution ;also throughput already reflected in SSV KPI</t>
         </is>
       </c>
       <c r="G100" s="5" t="inlineStr">
         <is>
-          <t>Accepted. TelTech officially updates the nationwide Call Drop Rate (CDR) operational KPI as follows: Target Standard: &lt;= 1.5% (revised from &lt;= 0.5%); Maximum Threshold: &lt;= 2.0% (revised from &lt;= 1.0%). Service Credits apply only if monthly nationwide aggregate CDR exceeds 2.0%.</t>
+          <t>Accepted in part. TelTech confirms that contractual financial liquidated damages / service credits shall not be assessed against daily instantaneous user throughput OSS counters. However, gNodeB scheduler throughput metrics (5-percentile and 50-percentile user throughput) shall remain active in OSS performance management for network traffic monitoring and capacity trigger planning.</t>
         </is>
       </c>
       <c r="H100" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -11160,7 +11123,7 @@
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>Q096</t>
+          <t>Q097</t>
         </is>
       </c>
       <c r="C101" s="5" t="inlineStr">
@@ -11181,17 +11144,17 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>suggest to remove both KPIs , this is more factored by user behavior and user distribution ;also throughput already reflected in SSV KPI</t>
+          <t>There is no OSS KPI latency statistics; only drive tests are available, which have been reflected in SSV.</t>
         </is>
       </c>
       <c r="G101" s="5" t="inlineStr">
         <is>
-          <t>Accepted in part. TelTech confirms that contractual financial liquidated damages / service credits shall not be assessed against daily instantaneous user throughput OSS counters. However, gNodeB scheduler throughput metrics (5-percentile and 50-percentile user throughput) shall remain active in OSS performance management for network traffic monitoring and capacity trigger planning.</t>
+          <t>Accepted. TelTech confirms that the round-trip latency KPI (target &lt;= 20 ms) shall be formally validated during Single Site Verification (SSV) and periodic cluster drive testing using standardized ping / TWAMP (Two-Way Active Measurement Protocol) test procedures between the test CPE and gNodeB / UPF test endpoints.</t>
         </is>
       </c>
       <c r="H101" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -11201,7 +11164,7 @@
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>Q097</t>
+          <t>Q098</t>
         </is>
       </c>
       <c r="C102" s="5" t="inlineStr">
@@ -11222,17 +11185,17 @@
       </c>
       <c r="F102" s="5" t="inlineStr">
         <is>
-          <t>There is no OSS KPI latency statistics; only drive tests are available, which have been reflected in SSV.</t>
+          <t>suggest target 0.1%，0.2% max; and PDCP layer;</t>
         </is>
       </c>
       <c r="G102" s="5" t="inlineStr">
         <is>
-          <t>Accepted. TelTech confirms that the round-trip latency KPI (target &lt;= 20 ms) shall be formally validated during Single Site Verification (SSV) and periodic cluster drive testing using standardized ping / TWAMP (Two-Way Active Measurement Protocol) test procedures between the test CPE and gNodeB / UPF test endpoints.</t>
+          <t>Accepted. Packet loss rate shall be formally evaluated at the PDCP (Packet Data Convergence Protocol) layer per 3GPP TS 38.314 standards, with updated KPI thresholds: Target Standard: &lt;= 0.10%; Maximum Threshold: &lt;= 0.20%.</t>
         </is>
       </c>
       <c r="H102" s="12" t="inlineStr">
         <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>
@@ -11242,66 +11205,25 @@
       </c>
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>Q098</t>
+          <t>Q099</t>
         </is>
       </c>
       <c r="C103" s="5" t="inlineStr">
         <is>
-          <t>SLA&amp;KPIs</t>
+          <t>Wireless and Delivery</t>
         </is>
       </c>
       <c r="D103" s="5" t="inlineStr">
         <is>
-          <t>05_Appendix_C_SLAs_KPIs_Liquidated_Damages</t>
+          <t>05_Appendix_D_Site_Survey_RF_Planning_Civil_Power_Guidelines.pdf</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
         <is>
-          <t>3.1 Core Radio KPIs
-(Calculated 24/7/366 Nationwide)</t>
+          <t>5.. SINGLE SITE VERIFICATION (SSV) &amp; CLUSTER ACCEPTANCE CRITERIA</t>
         </is>
       </c>
       <c r="F103" s="5" t="inlineStr">
-        <is>
-          <t>suggest target 0.1%，0.2% max; and PDCP layer;</t>
-        </is>
-      </c>
-      <c r="G103" s="5" t="inlineStr">
-        <is>
-          <t>Accepted. Packet loss rate shall be formally evaluated at the PDCP (Packet Data Convergence Protocol) layer per 3GPP TS 38.314 standards, with updated KPI thresholds: Target Standard: &lt;= 0.10%; Maximum Threshold: &lt;= 0.20%.</t>
-        </is>
-      </c>
-      <c r="H103" s="12" t="inlineStr">
-        <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="B104" s="4" t="inlineStr">
-        <is>
-          <t>Q099</t>
-        </is>
-      </c>
-      <c r="C104" s="5" t="inlineStr">
-        <is>
-          <t>Wireless and Delivery</t>
-        </is>
-      </c>
-      <c r="D104" s="5" t="inlineStr">
-        <is>
-          <t>05_Appendix_D_Site_Survey_RF_Planning_Civil_Power_Guidelines.pdf</t>
-        </is>
-      </c>
-      <c r="E104" s="5" t="inlineStr">
-        <is>
-          <t>5.. SINGLE SITE VERIFICATION (SSV) &amp; CLUSTER ACCEPTANCE CRITERIA</t>
-        </is>
-      </c>
-      <c r="F104" s="5" t="inlineStr">
         <is>
           <t>from last time clarification , converage feedback :
 SSV SPEED TARGETS PER DISTANCE ZONE:
@@ -11315,56 +11237,56 @@
 [-95~-105)dBm: DL 35Mbps/UL 1.5Mbps</t>
         </is>
       </c>
-      <c r="G104" s="5" t="inlineStr">
+      <c r="G103" s="5" t="inlineStr">
         <is>
           <t>Accepted with clarification. TelTech approves the adoption of RSRP-correlated benchmark thresholds for static Single Site Verification (SSV) under a standard 8:2 (DDDDDDDSUU) or 7:3 TDD frame structure in a 60 MHz Band n50 channel: (1) Near Zone (RSRP &gt;= -80 dBm): DL &gt;= 200 Mbps / UL &gt;= 25 Mbps; (2) Mid Zone (-95 dBm &lt;= RSRP &lt; -80 dBm): DL &gt;= 100 Mbps / UL &gt;= 10 Mbps; (3) Cell Edge Zone (-105 dBm &lt;= RSRP &lt; -95 dBm): DL &gt;= 35 Mbps / UL &gt;= 5 Mbps (UL minimum floor of 5 Mbps is maintained to ensure reliable TCP ACK and two-way interactive video traffic). Stationary SSV measurements shall be recorded using standard outdoor/indoor CPE units matching Lot 7 technical specifications.</t>
         </is>
       </c>
-      <c r="H104" s="12" t="inlineStr">
-        <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="4" t="n">
-        <v>101</v>
-      </c>
-      <c r="B105" s="4" t="inlineStr">
+      <c r="H103" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="4" t="n">
+        <v>100</v>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
         <is>
           <t>Q100</t>
         </is>
       </c>
-      <c r="C105" s="5" t="inlineStr">
+      <c r="C104" s="5" t="inlineStr">
         <is>
           <t>Transmission</t>
         </is>
       </c>
-      <c r="D105" s="5" t="inlineStr">
+      <c r="D104" s="5" t="inlineStr">
         <is>
           <t>01_RFP_5G_FWA_Master_Tender_Document</t>
         </is>
       </c>
-      <c r="E105" s="5" t="inlineStr">
+      <c r="E104" s="5" t="inlineStr">
         <is>
           <t>2.3 Transmission &amp; Backhaul Topology</t>
         </is>
       </c>
-      <c r="F105" s="5" t="inlineStr">
+      <c r="F104" s="5" t="inlineStr">
         <is>
           <t>1, The SFP of Transmission devices for Interconnections with BBU will be provided by the Contractor / Prospective Bidder or TelTech/TelTech?
 2, The SFP of BBU will be 25GE/10GE Adaptive Optical Module, the SFP of transmission device will be adaptive also, or specific ones and what types they will be(need confirm the transmission port capability also)
 3, The related configurations on Transmission backhaul for BBU integration will be under TelTech or the Contractor / Prospective Bidder?</t>
         </is>
       </c>
-      <c r="G105" s="5" t="inlineStr">
+      <c r="G104" s="5" t="inlineStr">
         <is>
           <t>Confirmed. 1. SFP Supply Boundary: The RAN bidder is responsible for supplying optical transceivers (SFPs) for all BBU/gNodeB ports. TelTech/TelTech will provide the compatible optical transceivers for the customer-facing ports on the demarcation transmission device (IP-RAN router / cell site gateway / GPON ONT). 2. Optics Specification: BBU optical modules shall be dual-rate 10GE/25GE eCPRI/CPRI/Ethernet adaptive transceivers (supporting standard 1310nm Single-Mode Fiber, LC duplex connectors, up to 10 km reach). Demarcation switch ports provided by TelTech support auto-negotiation at 10GE and 25GE. 3. Configuration Responsibilities: The RAN bidder is responsible for end-to-end BBU interface configuration (VLAN tagging, IP addressing, QoS markings per DSCP matrix, and sync synchronization IEEE 1588v2 PTP / SyncE). TelTech/TelTech transmission engineers will configure the transport network (VLAN tunneling, MPLS-VPN / SRv6 L2/L3 transport) up to the BBU handoff port.</t>
         </is>
       </c>
-      <c r="H105" s="12" t="inlineStr">
-        <is>
-          <t>Binding Ruling (Bid Bulletin No. 2)</t>
+      <c r="H104" s="12" t="inlineStr">
+        <is>
+          <t>Binding Ruling (Bid Bulletin No. 2.1 - Oct 30, 2026)</t>
         </is>
       </c>
     </row>

</xml_diff>